<commit_message>
sync: full update from as_upstream (15-10)
</commit_message>
<xml_diff>
--- a/db/inflections/inflection_templates.xlsx
+++ b/db/inflections/inflection_templates.xlsx
@@ -7095,12 +7095,10 @@
     <t xml:space="preserve">kubbamhe</t>
   </si>
   <si>
-    <t xml:space="preserve">karotu
-kubbatu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">karontu
-kubbantu</t>
+    <t xml:space="preserve">kubbatu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kubbantu</t>
   </si>
   <si>
     <t xml:space="preserve">kubbataṃ</t>
@@ -7126,8 +7124,7 @@
 kubbaye</t>
   </si>
   <si>
-    <t xml:space="preserve">kareyyuṃ
-kubbeyyuṃ
+    <t xml:space="preserve">kubbeyyuṃ
 kayiruṃ</t>
   </si>
   <si>
@@ -7202,7 +7199,9 @@
     <t xml:space="preserve">karaṃ</t>
   </si>
   <si>
-    <t xml:space="preserve">karimhe</t>
+    <t xml:space="preserve">karimhe
+karamhasa
+karamhase</t>
   </si>
   <si>
     <t xml:space="preserve">jantu</t>
@@ -66151,7 +66150,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="41.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="21" t="s">
         <v>482</v>
       </c>

</xml_diff>

<commit_message>
sync: full update from as_upstream (06-12)
</commit_message>
<xml_diff>
--- a/db/inflections/inflection_templates.xlsx
+++ b/db/inflections/inflection_templates.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9962" uniqueCount="2678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9966" uniqueCount="2679">
   <si>
     <t xml:space="preserve">inflection name</t>
   </si>
@@ -6842,6 +6842,9 @@
 santamhā
 santasmā
 santā</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ete</t>
   </si>
   <si>
     <t xml:space="preserve">ubhayamhi
@@ -63440,47 +63443,55 @@
       <c r="CW164" s="71" t="s">
         <v>447</v>
       </c>
-      <c r="CX164" s="70"/>
-      <c r="CY164" s="71"/>
-      <c r="CZ164" s="70"/>
-      <c r="DA164" s="71"/>
+      <c r="CX164" s="70" t="s">
+        <v>1933</v>
+      </c>
+      <c r="CY164" s="71" t="s">
+        <v>449</v>
+      </c>
+      <c r="CZ164" s="70" t="s">
+        <v>860</v>
+      </c>
+      <c r="DA164" s="71" t="s">
+        <v>451</v>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="21" t="s">
         <v>596</v>
       </c>
       <c r="B165" s="21" t="s">
-        <v>1933</v>
+        <v>1934</v>
       </c>
       <c r="C165" s="48" t="s">
         <v>598</v>
       </c>
       <c r="D165" s="21" t="s">
-        <v>1934</v>
+        <v>1935</v>
       </c>
       <c r="E165" s="48" t="s">
         <v>600</v>
       </c>
       <c r="F165" s="37" t="s">
-        <v>1935</v>
+        <v>1936</v>
       </c>
       <c r="G165" s="49" t="s">
         <v>602</v>
       </c>
       <c r="H165" s="37" t="s">
-        <v>1936</v>
+        <v>1937</v>
       </c>
       <c r="I165" s="49" t="s">
         <v>604</v>
       </c>
       <c r="J165" s="21" t="s">
-        <v>1933</v>
+        <v>1934</v>
       </c>
       <c r="K165" s="48" t="s">
         <v>605</v>
       </c>
       <c r="L165" s="21" t="s">
-        <v>1934</v>
+        <v>1935</v>
       </c>
       <c r="M165" s="48" t="s">
         <v>606</v>
@@ -63509,7 +63520,7 @@
         <v>596</v>
       </c>
       <c r="BF165" s="41" t="s">
-        <v>1937</v>
+        <v>1938</v>
       </c>
       <c r="BG165" s="56" t="s">
         <v>598</v>
@@ -63551,7 +63562,7 @@
         <v>636</v>
       </c>
       <c r="B166" s="21" t="s">
-        <v>1938</v>
+        <v>1939</v>
       </c>
       <c r="C166" s="48" t="s">
         <v>636</v>
@@ -63758,13 +63769,13 @@
         <v>570</v>
       </c>
       <c r="CX168" s="46" t="s">
-        <v>1939</v>
+        <v>1940</v>
       </c>
       <c r="CY168" s="19" t="s">
         <v>572</v>
       </c>
       <c r="CZ168" s="46" t="s">
-        <v>1940</v>
+        <v>1941</v>
       </c>
       <c r="DA168" s="19" t="s">
         <v>574</v>
@@ -63857,7 +63868,7 @@
         <v>592</v>
       </c>
       <c r="CZ169" s="46" t="s">
-        <v>1941</v>
+        <v>1942</v>
       </c>
       <c r="DA169" s="19" t="s">
         <v>594</v>
@@ -63927,13 +63938,13 @@
         <v>417</v>
       </c>
       <c r="BF170" s="41" t="s">
-        <v>1942</v>
+        <v>1943</v>
       </c>
       <c r="BG170" s="56" t="s">
         <v>419</v>
       </c>
       <c r="BH170" s="41" t="s">
-        <v>1943</v>
+        <v>1944</v>
       </c>
       <c r="BI170" s="56" t="s">
         <v>421</v>
@@ -63948,7 +63959,7 @@
         <v>618</v>
       </c>
       <c r="CT170" s="70" t="s">
-        <v>1944</v>
+        <v>1945</v>
       </c>
       <c r="CU170" s="71" t="s">
         <v>620</v>
@@ -64036,13 +64047,13 @@
         <v>455</v>
       </c>
       <c r="BF171" s="41" t="s">
-        <v>1945</v>
+        <v>1946</v>
       </c>
       <c r="BG171" s="56" t="s">
         <v>456</v>
       </c>
       <c r="BH171" s="41" t="s">
-        <v>1943</v>
+        <v>1944</v>
       </c>
       <c r="BI171" s="56" t="s">
         <v>458</v>
@@ -64057,13 +64068,13 @@
         <v>642</v>
       </c>
       <c r="CT171" s="70" t="s">
-        <v>1946</v>
+        <v>1947</v>
       </c>
       <c r="CU171" s="71" t="s">
         <v>644</v>
       </c>
       <c r="CV171" s="70" t="s">
-        <v>1947</v>
+        <v>1948</v>
       </c>
       <c r="CW171" s="71" t="s">
         <v>646</v>
@@ -64145,13 +64156,13 @@
         <v>482</v>
       </c>
       <c r="BF172" s="41" t="s">
-        <v>1948</v>
+        <v>1949</v>
       </c>
       <c r="BG172" s="56" t="s">
         <v>484</v>
       </c>
       <c r="BH172" s="41" t="s">
-        <v>1949</v>
+        <v>1950</v>
       </c>
       <c r="BI172" s="56" t="s">
         <v>486</v>
@@ -64166,13 +64177,13 @@
         <v>652</v>
       </c>
       <c r="CT172" s="70" t="s">
-        <v>1950</v>
+        <v>1951</v>
       </c>
       <c r="CU172" s="71" t="s">
         <v>654</v>
       </c>
       <c r="CV172" s="70" t="s">
-        <v>1951</v>
+        <v>1952</v>
       </c>
       <c r="CW172" s="71" t="s">
         <v>656</v>
@@ -64254,13 +64265,13 @@
         <v>519</v>
       </c>
       <c r="BF173" s="41" t="s">
-        <v>1952</v>
+        <v>1953</v>
       </c>
       <c r="BG173" s="56" t="s">
         <v>521</v>
       </c>
       <c r="BH173" s="41" t="s">
-        <v>1953</v>
+        <v>1954</v>
       </c>
       <c r="BI173" s="56" t="s">
         <v>523</v>
@@ -64275,25 +64286,25 @@
         <v>664</v>
       </c>
       <c r="CT173" s="46" t="s">
-        <v>1954</v>
+        <v>1955</v>
       </c>
       <c r="CU173" s="19" t="s">
         <v>666</v>
       </c>
       <c r="CV173" s="46" t="s">
-        <v>1955</v>
+        <v>1956</v>
       </c>
       <c r="CW173" s="19" t="s">
         <v>668</v>
       </c>
       <c r="CX173" s="46" t="s">
-        <v>1956</v>
+        <v>1957</v>
       </c>
       <c r="CY173" s="19" t="s">
         <v>670</v>
       </c>
       <c r="CZ173" s="46" t="s">
-        <v>1957</v>
+        <v>1958</v>
       </c>
       <c r="DA173" s="19" t="s">
         <v>672</v>
@@ -64363,13 +64374,13 @@
         <v>549</v>
       </c>
       <c r="BF174" s="41" t="s">
-        <v>1958</v>
+        <v>1959</v>
       </c>
       <c r="BG174" s="56" t="s">
         <v>551</v>
       </c>
       <c r="BH174" s="41" t="s">
-        <v>1949</v>
+        <v>1950</v>
       </c>
       <c r="BI174" s="56" t="s">
         <v>552</v>
@@ -64384,25 +64395,25 @@
         <v>691</v>
       </c>
       <c r="CT174" s="46" t="s">
-        <v>1959</v>
+        <v>1960</v>
       </c>
       <c r="CU174" s="19" t="s">
         <v>693</v>
       </c>
       <c r="CV174" s="46" t="s">
-        <v>1960</v>
+        <v>1961</v>
       </c>
       <c r="CW174" s="19" t="s">
         <v>695</v>
       </c>
       <c r="CX174" s="46" t="s">
-        <v>1961</v>
+        <v>1962</v>
       </c>
       <c r="CY174" s="19" t="s">
         <v>697</v>
       </c>
       <c r="CZ174" s="46" t="s">
-        <v>1962</v>
+        <v>1963</v>
       </c>
       <c r="DA174" s="19" t="s">
         <v>699</v>
@@ -64472,13 +64483,13 @@
         <v>576</v>
       </c>
       <c r="BF175" s="41" t="s">
-        <v>1952</v>
+        <v>1953</v>
       </c>
       <c r="BG175" s="56" t="s">
         <v>578</v>
       </c>
       <c r="BH175" s="41" t="s">
-        <v>1953</v>
+        <v>1954</v>
       </c>
       <c r="BI175" s="56" t="s">
         <v>579</v>
@@ -64493,25 +64504,25 @@
         <v>724</v>
       </c>
       <c r="CT175" s="46" t="s">
-        <v>1963</v>
+        <v>1964</v>
       </c>
       <c r="CU175" s="19" t="s">
         <v>726</v>
       </c>
       <c r="CV175" s="46" t="s">
-        <v>1964</v>
+        <v>1965</v>
       </c>
       <c r="CW175" s="19" t="s">
         <v>728</v>
       </c>
       <c r="CX175" s="46" t="s">
-        <v>1965</v>
+        <v>1966</v>
       </c>
       <c r="CY175" s="19" t="s">
         <v>730</v>
       </c>
       <c r="CZ175" s="46" t="s">
-        <v>1966</v>
+        <v>1967</v>
       </c>
       <c r="DA175" s="19" t="s">
         <v>732</v>
@@ -64581,13 +64592,13 @@
         <v>596</v>
       </c>
       <c r="BF176" s="41" t="s">
-        <v>1967</v>
+        <v>1968</v>
       </c>
       <c r="BG176" s="56" t="s">
         <v>598</v>
       </c>
       <c r="BH176" s="41" t="s">
-        <v>1968</v>
+        <v>1969</v>
       </c>
       <c r="BI176" s="56" t="s">
         <v>600</v>
@@ -64672,13 +64683,13 @@
         <v>627</v>
       </c>
       <c r="BF177" s="41" t="s">
-        <v>1942</v>
+        <v>1943</v>
       </c>
       <c r="BG177" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH177" s="41" t="s">
-        <v>1943</v>
+        <v>1944</v>
       </c>
       <c r="BI177" s="56" t="s">
         <v>630</v>
@@ -64734,7 +64745,7 @@
         <v>636</v>
       </c>
       <c r="BF178" s="41" t="s">
-        <v>1969</v>
+        <v>1970</v>
       </c>
       <c r="BG178" s="56" t="s">
         <v>636</v>
@@ -64799,13 +64810,13 @@
         <v>673</v>
       </c>
       <c r="CT179" s="70" t="s">
-        <v>1970</v>
+        <v>1971</v>
       </c>
       <c r="CU179" s="71" t="s">
         <v>675</v>
       </c>
       <c r="CV179" s="70" t="s">
-        <v>1971</v>
+        <v>1972</v>
       </c>
       <c r="CW179" s="71" t="s">
         <v>677</v>
@@ -64884,7 +64895,7 @@
         <v>701</v>
       </c>
       <c r="CV180" s="70" t="s">
-        <v>1972</v>
+        <v>1973</v>
       </c>
       <c r="CW180" s="71" t="s">
         <v>703</v>
@@ -64975,7 +64986,7 @@
         <v>733</v>
       </c>
       <c r="CT181" s="70" t="s">
-        <v>1973</v>
+        <v>1974</v>
       </c>
       <c r="CU181" s="71" t="s">
         <v>735</v>
@@ -65136,7 +65147,7 @@
         <v>482</v>
       </c>
       <c r="BF183" s="41" t="s">
-        <v>1974</v>
+        <v>1975</v>
       </c>
       <c r="BG183" s="56" t="s">
         <v>484</v>
@@ -65218,7 +65229,7 @@
         <v>519</v>
       </c>
       <c r="BF184" s="41" t="s">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="BG184" s="56" t="s">
         <v>521</v>
@@ -65319,7 +65330,7 @@
         <v>549</v>
       </c>
       <c r="BF185" s="41" t="s">
-        <v>1976</v>
+        <v>1977</v>
       </c>
       <c r="BG185" s="56" t="s">
         <v>551</v>
@@ -65345,13 +65356,13 @@
         <v>618</v>
       </c>
       <c r="CT185" s="62" t="s">
-        <v>1977</v>
+        <v>1978</v>
       </c>
       <c r="CU185" s="63" t="s">
         <v>620</v>
       </c>
       <c r="CV185" s="62" t="s">
-        <v>1978</v>
+        <v>1979</v>
       </c>
       <c r="CW185" s="63" t="s">
         <v>622</v>
@@ -65431,7 +65442,7 @@
         <v>576</v>
       </c>
       <c r="BF186" s="41" t="s">
-        <v>1975</v>
+        <v>1976</v>
       </c>
       <c r="BG186" s="56" t="s">
         <v>578</v>
@@ -65457,7 +65468,7 @@
         <v>642</v>
       </c>
       <c r="CT186" s="62" t="s">
-        <v>1979</v>
+        <v>1980</v>
       </c>
       <c r="CU186" s="63" t="s">
         <v>644</v>
@@ -65541,7 +65552,7 @@
         <v>596</v>
       </c>
       <c r="BF187" s="41" t="s">
-        <v>1980</v>
+        <v>1981</v>
       </c>
       <c r="BG187" s="56" t="s">
         <v>598</v>
@@ -65567,13 +65578,13 @@
         <v>652</v>
       </c>
       <c r="CT187" s="62" t="s">
-        <v>1981</v>
+        <v>1982</v>
       </c>
       <c r="CU187" s="63" t="s">
         <v>654</v>
       </c>
       <c r="CV187" s="62" t="s">
-        <v>1982</v>
+        <v>1983</v>
       </c>
       <c r="CW187" s="63" t="s">
         <v>656</v>
@@ -65651,13 +65662,13 @@
         <v>627</v>
       </c>
       <c r="BF188" s="41" t="s">
-        <v>1983</v>
+        <v>1984</v>
       </c>
       <c r="BG188" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH188" s="41" t="s">
-        <v>1984</v>
+        <v>1985</v>
       </c>
       <c r="BI188" s="56" t="s">
         <v>630</v>
@@ -65727,7 +65738,7 @@
         <v>636</v>
       </c>
       <c r="BF189" s="41" t="s">
-        <v>1985</v>
+        <v>1986</v>
       </c>
       <c r="BG189" s="56" t="s">
         <v>636</v>
@@ -65890,25 +65901,25 @@
         <v>443</v>
       </c>
       <c r="CT191" s="70" t="s">
-        <v>1986</v>
+        <v>1987</v>
       </c>
       <c r="CU191" s="71" t="s">
         <v>445</v>
       </c>
       <c r="CV191" s="70" t="s">
-        <v>1987</v>
+        <v>1988</v>
       </c>
       <c r="CW191" s="71" t="s">
         <v>447</v>
       </c>
       <c r="CX191" s="70" t="s">
-        <v>1988</v>
+        <v>1989</v>
       </c>
       <c r="CY191" s="71" t="s">
         <v>449</v>
       </c>
       <c r="CZ191" s="70" t="s">
-        <v>1989</v>
+        <v>1990</v>
       </c>
       <c r="DA191" s="71" t="s">
         <v>451</v>
@@ -65978,7 +65989,7 @@
         <v>417</v>
       </c>
       <c r="BF192" s="41" t="s">
-        <v>1990</v>
+        <v>1991</v>
       </c>
       <c r="BG192" s="56" t="s">
         <v>419</v>
@@ -66002,25 +66013,25 @@
         <v>470</v>
       </c>
       <c r="CT192" s="70" t="s">
-        <v>1991</v>
+        <v>1992</v>
       </c>
       <c r="CU192" s="71" t="s">
         <v>472</v>
       </c>
       <c r="CV192" s="70" t="s">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="CW192" s="71" t="s">
         <v>474</v>
       </c>
       <c r="CX192" s="70" t="s">
-        <v>1993</v>
+        <v>1994</v>
       </c>
       <c r="CY192" s="71" t="s">
         <v>476</v>
       </c>
       <c r="CZ192" s="70" t="s">
-        <v>1994</v>
+        <v>1995</v>
       </c>
       <c r="DA192" s="71" t="s">
         <v>478</v>
@@ -66090,7 +66101,7 @@
         <v>455</v>
       </c>
       <c r="BF193" s="41" t="s">
-        <v>1995</v>
+        <v>1996</v>
       </c>
       <c r="BG193" s="56" t="s">
         <v>456</v>
@@ -66114,25 +66125,25 @@
         <v>507</v>
       </c>
       <c r="CT193" s="70" t="s">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="CU193" s="71" t="s">
         <v>509</v>
       </c>
       <c r="CV193" s="70" t="s">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="CW193" s="71" t="s">
         <v>511</v>
       </c>
       <c r="CX193" s="70" t="s">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="CY193" s="71" t="s">
         <v>512</v>
       </c>
       <c r="CZ193" s="70" t="s">
-        <v>1999</v>
+        <v>2000</v>
       </c>
       <c r="DA193" s="71" t="s">
         <v>514</v>
@@ -66224,25 +66235,25 @@
         <v>538</v>
       </c>
       <c r="CT194" s="46" t="s">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="CU194" s="19" t="s">
         <v>540</v>
       </c>
       <c r="CV194" s="46" t="s">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="CW194" s="19" t="s">
         <v>542</v>
       </c>
       <c r="CX194" s="46" t="s">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="CY194" s="19" t="s">
         <v>544</v>
       </c>
       <c r="CZ194" s="46" t="s">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="DA194" s="19" t="s">
         <v>546</v>
@@ -66334,25 +66345,25 @@
         <v>567</v>
       </c>
       <c r="CT195" s="46" t="s">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="CU195" s="19" t="s">
         <v>569</v>
       </c>
       <c r="CV195" s="46" t="s">
-        <v>1992</v>
+        <v>1993</v>
       </c>
       <c r="CW195" s="19" t="s">
         <v>570</v>
       </c>
       <c r="CX195" s="46" t="s">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="CY195" s="19" t="s">
         <v>572</v>
       </c>
       <c r="CZ195" s="46" t="s">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="DA195" s="19" t="s">
         <v>574</v>
@@ -66444,25 +66455,25 @@
         <v>589</v>
       </c>
       <c r="CT196" s="46" t="s">
-        <v>1996</v>
+        <v>1997</v>
       </c>
       <c r="CU196" s="19" t="s">
         <v>590</v>
       </c>
       <c r="CV196" s="46" t="s">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="CW196" s="19" t="s">
         <v>591</v>
       </c>
       <c r="CX196" s="46" t="s">
-        <v>1998</v>
+        <v>1999</v>
       </c>
       <c r="CY196" s="19" t="s">
         <v>592</v>
       </c>
       <c r="CZ196" s="46" t="s">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="DA196" s="19" t="s">
         <v>594</v>
@@ -66554,25 +66565,25 @@
         <v>618</v>
       </c>
       <c r="CT197" s="70" t="s">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="CU197" s="71" t="s">
         <v>620</v>
       </c>
       <c r="CV197" s="70" t="s">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="CW197" s="71" t="s">
         <v>622</v>
       </c>
       <c r="CX197" s="70" t="s">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="CY197" s="71" t="s">
         <v>624</v>
       </c>
       <c r="CZ197" s="70" t="s">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="DA197" s="71" t="s">
         <v>626</v>
@@ -66664,25 +66675,25 @@
         <v>642</v>
       </c>
       <c r="CT198" s="70" t="s">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="CU198" s="71" t="s">
         <v>644</v>
       </c>
       <c r="CV198" s="70" t="s">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="CW198" s="71" t="s">
         <v>646</v>
       </c>
       <c r="CX198" s="70" t="s">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="CY198" s="71" t="s">
         <v>648</v>
       </c>
       <c r="CZ198" s="70" t="s">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="DA198" s="71" t="s">
         <v>650</v>
@@ -66774,25 +66785,25 @@
         <v>652</v>
       </c>
       <c r="CT199" s="70" t="s">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="CU199" s="71" t="s">
         <v>654</v>
       </c>
       <c r="CV199" s="70" t="s">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="CW199" s="71" t="s">
         <v>656</v>
       </c>
       <c r="CX199" s="70" t="s">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="CY199" s="71" t="s">
         <v>658</v>
       </c>
       <c r="CZ199" s="70" t="s">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="DA199" s="71" t="s">
         <v>660</v>
@@ -66973,25 +66984,25 @@
         <v>673</v>
       </c>
       <c r="CT202" s="70" t="s">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="CU202" s="71" t="s">
         <v>675</v>
       </c>
       <c r="CV202" s="70" t="s">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="CW202" s="71" t="s">
         <v>677</v>
       </c>
       <c r="CX202" s="70" t="s">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="CY202" s="71" t="s">
         <v>946</v>
       </c>
       <c r="CZ202" s="70" t="s">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="DA202" s="71" t="s">
         <v>948</v>
@@ -67054,25 +67065,25 @@
         <v>700</v>
       </c>
       <c r="CT203" s="70" t="s">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="CU203" s="71" t="s">
         <v>701</v>
       </c>
       <c r="CV203" s="70" t="s">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="CW203" s="71" t="s">
         <v>703</v>
       </c>
       <c r="CX203" s="70" t="s">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="CY203" s="71" t="s">
         <v>960</v>
       </c>
       <c r="CZ203" s="70" t="s">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="DA203" s="71" t="s">
         <v>962</v>
@@ -67135,25 +67146,25 @@
         <v>733</v>
       </c>
       <c r="CT204" s="70" t="s">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="CU204" s="71" t="s">
         <v>735</v>
       </c>
       <c r="CV204" s="70" t="s">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="CW204" s="71" t="s">
         <v>737</v>
       </c>
       <c r="CX204" s="70" t="s">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="CY204" s="71" t="s">
         <v>975</v>
       </c>
       <c r="CZ204" s="70" t="s">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="DA204" s="71" t="s">
         <v>977</v>
@@ -67316,7 +67327,7 @@
         <v>549</v>
       </c>
       <c r="BF207" s="41" t="s">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="BG207" s="56" t="s">
         <v>551</v>
@@ -67728,13 +67739,13 @@
         <v>417</v>
       </c>
       <c r="BF214" s="41" t="s">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="BG214" s="56" t="s">
         <v>419</v>
       </c>
       <c r="BH214" s="41" t="s">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="BI214" s="56" t="s">
         <v>421</v>
@@ -67782,13 +67793,13 @@
         <v>455</v>
       </c>
       <c r="BF215" s="41" t="s">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="BG215" s="56" t="s">
         <v>456</v>
       </c>
       <c r="BH215" s="41" t="s">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="BI215" s="56" t="s">
         <v>458</v>
@@ -67836,13 +67847,13 @@
         <v>482</v>
       </c>
       <c r="BF216" s="41" t="s">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="BG216" s="56" t="s">
         <v>484</v>
       </c>
       <c r="BH216" s="41" t="s">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="BI216" s="56" t="s">
         <v>486</v>
@@ -67890,13 +67901,13 @@
         <v>519</v>
       </c>
       <c r="BF217" s="41" t="s">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="BG217" s="56" t="s">
         <v>521</v>
       </c>
       <c r="BH217" s="41" t="s">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="BI217" s="56" t="s">
         <v>523</v>
@@ -67944,13 +67955,13 @@
         <v>549</v>
       </c>
       <c r="BF218" s="41" t="s">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="BG218" s="56" t="s">
         <v>551</v>
       </c>
       <c r="BH218" s="41" t="s">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="BI218" s="56" t="s">
         <v>552</v>
@@ -67998,13 +68009,13 @@
         <v>576</v>
       </c>
       <c r="BF219" s="41" t="s">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="BG219" s="56" t="s">
         <v>578</v>
       </c>
       <c r="BH219" s="41" t="s">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="BI219" s="56" t="s">
         <v>579</v>
@@ -68047,13 +68058,13 @@
         <v>596</v>
       </c>
       <c r="BF220" s="41" t="s">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="BG220" s="56" t="s">
         <v>598</v>
       </c>
       <c r="BH220" s="41" t="s">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="BI220" s="56" t="s">
         <v>600</v>
@@ -68096,13 +68107,13 @@
         <v>627</v>
       </c>
       <c r="BF221" s="41" t="s">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="BG221" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH221" s="41" t="s">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="BI221" s="56" t="s">
         <v>630</v>
@@ -68145,7 +68156,7 @@
         <v>636</v>
       </c>
       <c r="BF222" s="41" t="s">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="BG222" s="56" t="s">
         <v>636</v>
@@ -68272,13 +68283,13 @@
         <v>417</v>
       </c>
       <c r="BF225" s="41" t="s">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="BG225" s="56" t="s">
         <v>419</v>
       </c>
       <c r="BH225" s="41" t="s">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="BI225" s="56" t="s">
         <v>421</v>
@@ -68321,13 +68332,13 @@
         <v>455</v>
       </c>
       <c r="BF226" s="41" t="s">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="BG226" s="56" t="s">
         <v>456</v>
       </c>
       <c r="BH226" s="41" t="s">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="BI226" s="56" t="s">
         <v>458</v>
@@ -68370,13 +68381,13 @@
         <v>482</v>
       </c>
       <c r="BF227" s="41" t="s">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="BG227" s="56" t="s">
         <v>484</v>
       </c>
       <c r="BH227" s="41" t="s">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="BI227" s="56" t="s">
         <v>486</v>
@@ -68419,13 +68430,13 @@
         <v>519</v>
       </c>
       <c r="BF228" s="41" t="s">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="BG228" s="56" t="s">
         <v>521</v>
       </c>
       <c r="BH228" s="41" t="s">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="BI228" s="56" t="s">
         <v>523</v>
@@ -68468,13 +68479,13 @@
         <v>549</v>
       </c>
       <c r="BF229" s="41" t="s">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="BG229" s="56" t="s">
         <v>551</v>
       </c>
       <c r="BH229" s="41" t="s">
-        <v>2049</v>
+        <v>2050</v>
       </c>
       <c r="BI229" s="56" t="s">
         <v>552</v>
@@ -68517,13 +68528,13 @@
         <v>576</v>
       </c>
       <c r="BF230" s="41" t="s">
-        <v>2050</v>
+        <v>2051</v>
       </c>
       <c r="BG230" s="56" t="s">
         <v>578</v>
       </c>
       <c r="BH230" s="41" t="s">
-        <v>2051</v>
+        <v>2052</v>
       </c>
       <c r="BI230" s="56" t="s">
         <v>579</v>
@@ -68566,13 +68577,13 @@
         <v>596</v>
       </c>
       <c r="BF231" s="41" t="s">
-        <v>2052</v>
+        <v>2053</v>
       </c>
       <c r="BG231" s="56" t="s">
         <v>598</v>
       </c>
       <c r="BH231" s="41" t="s">
-        <v>2053</v>
+        <v>2054</v>
       </c>
       <c r="BI231" s="56" t="s">
         <v>600</v>
@@ -68615,13 +68626,13 @@
         <v>627</v>
       </c>
       <c r="BF232" s="41" t="s">
-        <v>2054</v>
+        <v>2055</v>
       </c>
       <c r="BG232" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH232" s="41" t="s">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="BI232" s="56" t="s">
         <v>630</v>
@@ -68664,7 +68675,7 @@
         <v>636</v>
       </c>
       <c r="BF233" s="41" t="s">
-        <v>2055</v>
+        <v>2056</v>
       </c>
       <c r="BG233" s="56" t="s">
         <v>636</v>
@@ -68791,13 +68802,13 @@
         <v>417</v>
       </c>
       <c r="BF236" s="41" t="s">
-        <v>2056</v>
+        <v>2057</v>
       </c>
       <c r="BG236" s="56" t="s">
         <v>419</v>
       </c>
       <c r="BH236" s="41" t="s">
-        <v>2057</v>
+        <v>2058</v>
       </c>
       <c r="BI236" s="56" t="s">
         <v>421</v>
@@ -68840,13 +68851,13 @@
         <v>455</v>
       </c>
       <c r="BF237" s="41" t="s">
-        <v>2058</v>
+        <v>2059</v>
       </c>
       <c r="BG237" s="56" t="s">
         <v>456</v>
       </c>
       <c r="BH237" s="41" t="s">
-        <v>2059</v>
+        <v>2060</v>
       </c>
       <c r="BI237" s="56" t="s">
         <v>458</v>
@@ -68889,13 +68900,13 @@
         <v>482</v>
       </c>
       <c r="BF238" s="41" t="s">
-        <v>2060</v>
+        <v>2061</v>
       </c>
       <c r="BG238" s="56" t="s">
         <v>484</v>
       </c>
       <c r="BH238" s="41" t="s">
-        <v>2061</v>
+        <v>2062</v>
       </c>
       <c r="BI238" s="56" t="s">
         <v>486</v>
@@ -68938,13 +68949,13 @@
         <v>519</v>
       </c>
       <c r="BF239" s="41" t="s">
-        <v>2062</v>
+        <v>2063</v>
       </c>
       <c r="BG239" s="56" t="s">
         <v>521</v>
       </c>
       <c r="BH239" s="41" t="s">
-        <v>2063</v>
+        <v>2064</v>
       </c>
       <c r="BI239" s="56" t="s">
         <v>523</v>
@@ -68987,13 +68998,13 @@
         <v>549</v>
       </c>
       <c r="BF240" s="41" t="s">
-        <v>2064</v>
+        <v>2065</v>
       </c>
       <c r="BG240" s="56" t="s">
         <v>551</v>
       </c>
       <c r="BH240" s="41" t="s">
-        <v>2061</v>
+        <v>2062</v>
       </c>
       <c r="BI240" s="56" t="s">
         <v>552</v>
@@ -69036,13 +69047,13 @@
         <v>576</v>
       </c>
       <c r="BF241" s="41" t="s">
-        <v>2062</v>
+        <v>2063</v>
       </c>
       <c r="BG241" s="56" t="s">
         <v>578</v>
       </c>
       <c r="BH241" s="41" t="s">
-        <v>2063</v>
+        <v>2064</v>
       </c>
       <c r="BI241" s="56" t="s">
         <v>579</v>
@@ -69085,13 +69096,13 @@
         <v>596</v>
       </c>
       <c r="BF242" s="41" t="s">
-        <v>2065</v>
+        <v>2066</v>
       </c>
       <c r="BG242" s="56" t="s">
         <v>598</v>
       </c>
       <c r="BH242" s="41" t="s">
-        <v>2066</v>
+        <v>2067</v>
       </c>
       <c r="BI242" s="56" t="s">
         <v>600</v>
@@ -69134,13 +69145,13 @@
         <v>627</v>
       </c>
       <c r="BF243" s="41" t="s">
-        <v>2067</v>
+        <v>2068</v>
       </c>
       <c r="BG243" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH243" s="41" t="s">
-        <v>2068</v>
+        <v>2069</v>
       </c>
       <c r="BI243" s="56" t="s">
         <v>630</v>
@@ -69183,7 +69194,7 @@
         <v>636</v>
       </c>
       <c r="BF244" s="41" t="s">
-        <v>2069</v>
+        <v>2070</v>
       </c>
       <c r="BG244" s="56" t="s">
         <v>636</v>
@@ -69653,7 +69664,7 @@
         <v>627</v>
       </c>
       <c r="BF254" s="41" t="s">
-        <v>2070</v>
+        <v>2071</v>
       </c>
       <c r="BG254" s="56" t="s">
         <v>629</v>
@@ -69876,7 +69887,7 @@
         <v>455</v>
       </c>
       <c r="BF259" s="41" t="s">
-        <v>2071</v>
+        <v>2072</v>
       </c>
       <c r="BG259" s="56" t="s">
         <v>456</v>
@@ -69968,7 +69979,7 @@
         <v>519</v>
       </c>
       <c r="BF261" s="41" t="s">
-        <v>2072</v>
+        <v>2073</v>
       </c>
       <c r="BG261" s="56" t="s">
         <v>521</v>
@@ -70047,7 +70058,7 @@
         <v>576</v>
       </c>
       <c r="BF263" s="41" t="s">
-        <v>2072</v>
+        <v>2073</v>
       </c>
       <c r="BG263" s="56" t="s">
         <v>578</v>
@@ -70084,7 +70095,7 @@
         <v>596</v>
       </c>
       <c r="BF264" s="41" t="s">
-        <v>2073</v>
+        <v>2074</v>
       </c>
       <c r="BG264" s="56" t="s">
         <v>598</v>
@@ -70255,13 +70266,13 @@
         <v>417</v>
       </c>
       <c r="BF269" s="41" t="s">
-        <v>2074</v>
+        <v>2075</v>
       </c>
       <c r="BG269" s="56" t="s">
         <v>419</v>
       </c>
       <c r="BH269" s="41" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="BI269" s="56" t="s">
         <v>421</v>
@@ -70294,13 +70305,13 @@
         <v>455</v>
       </c>
       <c r="BF270" s="41" t="s">
-        <v>2076</v>
+        <v>2077</v>
       </c>
       <c r="BG270" s="56" t="s">
         <v>456</v>
       </c>
       <c r="BH270" s="41" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="BI270" s="56" t="s">
         <v>458</v>
@@ -70333,13 +70344,13 @@
         <v>482</v>
       </c>
       <c r="BF271" s="41" t="s">
-        <v>2077</v>
+        <v>2078</v>
       </c>
       <c r="BG271" s="56" t="s">
         <v>484</v>
       </c>
       <c r="BH271" s="41" t="s">
-        <v>2078</v>
+        <v>2079</v>
       </c>
       <c r="BI271" s="56" t="s">
         <v>486</v>
@@ -70372,13 +70383,13 @@
         <v>519</v>
       </c>
       <c r="BF272" s="41" t="s">
-        <v>2079</v>
+        <v>2080</v>
       </c>
       <c r="BG272" s="56" t="s">
         <v>521</v>
       </c>
       <c r="BH272" s="41" t="s">
-        <v>2080</v>
+        <v>2081</v>
       </c>
       <c r="BI272" s="56" t="s">
         <v>523</v>
@@ -70411,13 +70422,13 @@
         <v>549</v>
       </c>
       <c r="BF273" s="41" t="s">
-        <v>2081</v>
+        <v>2082</v>
       </c>
       <c r="BG273" s="56" t="s">
         <v>551</v>
       </c>
       <c r="BH273" s="41" t="s">
-        <v>2078</v>
+        <v>2079</v>
       </c>
       <c r="BI273" s="56" t="s">
         <v>552</v>
@@ -70450,13 +70461,13 @@
         <v>576</v>
       </c>
       <c r="BF274" s="41" t="s">
-        <v>2082</v>
+        <v>2083</v>
       </c>
       <c r="BG274" s="56" t="s">
         <v>578</v>
       </c>
       <c r="BH274" s="41" t="s">
-        <v>2080</v>
+        <v>2081</v>
       </c>
       <c r="BI274" s="56" t="s">
         <v>579</v>
@@ -70489,13 +70500,13 @@
         <v>596</v>
       </c>
       <c r="BF275" s="41" t="s">
-        <v>2083</v>
+        <v>2084</v>
       </c>
       <c r="BG275" s="56" t="s">
         <v>598</v>
       </c>
       <c r="BH275" s="41" t="s">
-        <v>2084</v>
+        <v>2085</v>
       </c>
       <c r="BI275" s="56" t="s">
         <v>600</v>
@@ -70528,13 +70539,13 @@
         <v>627</v>
       </c>
       <c r="BF276" s="41" t="s">
-        <v>2085</v>
+        <v>2086</v>
       </c>
       <c r="BG276" s="56" t="s">
         <v>629</v>
       </c>
       <c r="BH276" s="41" t="s">
-        <v>2075</v>
+        <v>2076</v>
       </c>
       <c r="BI276" s="56" t="s">
         <v>630</v>
@@ -70567,7 +70578,7 @@
         <v>636</v>
       </c>
       <c r="BF277" s="41" t="s">
-        <v>2086</v>
+        <v>2087</v>
       </c>
       <c r="BG277" s="56" t="s">
         <v>636</v>
@@ -70760,7 +70771,7 @@
         <v>519</v>
       </c>
       <c r="BF283" s="41" t="s">
-        <v>2087</v>
+        <v>2088</v>
       </c>
       <c r="BG283" s="56" t="s">
         <v>521</v>
@@ -70806,7 +70817,7 @@
         <v>576</v>
       </c>
       <c r="BF285" s="41" t="s">
-        <v>2087</v>
+        <v>2088</v>
       </c>
       <c r="BG285" s="56" t="s">
         <v>578</v>
@@ -71463,46 +71474,46 @@
   <sheetData>
     <row r="1" s="22" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="22" t="s">
-        <v>2088</v>
+        <v>2089</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>2089</v>
+        <v>2090</v>
       </c>
       <c r="C1" s="81" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D1" s="81" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>2092</v>
+        <v>2093</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>2093</v>
+        <v>2094</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>2094</v>
+        <v>2095</v>
       </c>
       <c r="H1" s="81" t="s">
-        <v>2095</v>
+        <v>2096</v>
       </c>
       <c r="I1" s="22" t="s">
-        <v>2096</v>
+        <v>2097</v>
       </c>
       <c r="J1" s="81" t="s">
-        <v>2097</v>
+        <v>2098</v>
       </c>
       <c r="K1" s="81" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="L1" s="81" t="s">
-        <v>2099</v>
+        <v>2100</v>
       </c>
       <c r="M1" s="81" t="s">
-        <v>2100</v>
+        <v>2101</v>
       </c>
       <c r="N1" s="81" t="s">
-        <v>2101</v>
+        <v>2102</v>
       </c>
       <c r="AMI1" s="20"/>
       <c r="AMJ1" s="20"/>
@@ -71512,40 +71523,40 @@
         <v>417</v>
       </c>
       <c r="B2" s="82" t="s">
-        <v>2102</v>
+        <v>2103</v>
       </c>
       <c r="C2" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E2" s="83" t="s">
-        <v>2103</v>
+        <v>2104</v>
       </c>
       <c r="F2" s="83" t="s">
-        <v>2104</v>
+        <v>2105</v>
       </c>
       <c r="G2" s="83" t="s">
-        <v>2105</v>
+        <v>2106</v>
       </c>
       <c r="H2" s="83" t="s">
-        <v>2106</v>
+        <v>2107</v>
       </c>
       <c r="I2" s="82" t="s">
-        <v>2107</v>
+        <v>2108</v>
       </c>
       <c r="J2" s="82" t="s">
-        <v>2108</v>
+        <v>2109</v>
       </c>
       <c r="K2" s="83" t="s">
-        <v>2109</v>
+        <v>2110</v>
       </c>
       <c r="L2" s="83" t="s">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="M2" s="83" t="s">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="N2" s="83" t="s">
-        <v>2112</v>
+        <v>2113</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71553,40 +71564,40 @@
         <v>455</v>
       </c>
       <c r="B3" s="82" t="s">
-        <v>2113</v>
+        <v>2114</v>
       </c>
       <c r="C3" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E3" s="83" t="s">
-        <v>2114</v>
+        <v>2115</v>
       </c>
       <c r="F3" s="83" t="s">
-        <v>2115</v>
+        <v>2116</v>
       </c>
       <c r="G3" s="83" t="s">
-        <v>2116</v>
+        <v>2117</v>
       </c>
       <c r="H3" s="83" t="s">
-        <v>2117</v>
+        <v>2118</v>
       </c>
       <c r="I3" s="82" t="s">
-        <v>2118</v>
+        <v>2119</v>
       </c>
       <c r="J3" s="82" t="s">
-        <v>2119</v>
+        <v>2120</v>
       </c>
       <c r="K3" s="83" t="s">
-        <v>2120</v>
+        <v>2121</v>
       </c>
       <c r="L3" s="83" t="s">
-        <v>2121</v>
+        <v>2122</v>
       </c>
       <c r="M3" s="83" t="s">
-        <v>2122</v>
+        <v>2123</v>
       </c>
       <c r="N3" s="83" t="s">
-        <v>2123</v>
+        <v>2124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71594,40 +71605,40 @@
         <v>482</v>
       </c>
       <c r="B4" s="82" t="s">
-        <v>2124</v>
+        <v>2125</v>
       </c>
       <c r="C4" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E4" s="83" t="s">
-        <v>2125</v>
+        <v>2126</v>
       </c>
       <c r="F4" s="83" t="s">
-        <v>2126</v>
+        <v>2127</v>
       </c>
       <c r="G4" s="83" t="s">
-        <v>2127</v>
+        <v>2128</v>
       </c>
       <c r="H4" s="83" t="s">
-        <v>2128</v>
+        <v>2129</v>
       </c>
       <c r="I4" s="82" t="s">
-        <v>2129</v>
+        <v>2130</v>
       </c>
       <c r="J4" s="82" t="s">
-        <v>2130</v>
+        <v>2131</v>
       </c>
       <c r="K4" s="83" t="s">
-        <v>2131</v>
+        <v>2132</v>
       </c>
       <c r="L4" s="83" t="s">
-        <v>2132</v>
+        <v>2133</v>
       </c>
       <c r="M4" s="83" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="N4" s="83" t="s">
-        <v>2134</v>
+        <v>2135</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71635,40 +71646,40 @@
         <v>519</v>
       </c>
       <c r="B5" s="82" t="s">
-        <v>2135</v>
+        <v>2136</v>
       </c>
       <c r="C5" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E5" s="83" t="s">
-        <v>2136</v>
+        <v>2137</v>
       </c>
       <c r="F5" s="83" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="G5" s="83" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="H5" s="83" t="s">
-        <v>2139</v>
+        <v>2140</v>
       </c>
       <c r="I5" s="82" t="s">
-        <v>2140</v>
+        <v>2141</v>
       </c>
       <c r="J5" s="82" t="s">
-        <v>2141</v>
+        <v>2142</v>
       </c>
       <c r="K5" s="83" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="L5" s="83" t="s">
-        <v>2143</v>
+        <v>2144</v>
       </c>
       <c r="M5" s="83" t="s">
-        <v>2144</v>
+        <v>2145</v>
       </c>
       <c r="N5" s="83" t="s">
-        <v>2145</v>
+        <v>2146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71676,40 +71687,40 @@
         <v>549</v>
       </c>
       <c r="B6" s="82" t="s">
-        <v>2146</v>
+        <v>2147</v>
       </c>
       <c r="C6" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E6" s="83" t="s">
-        <v>2147</v>
+        <v>2148</v>
       </c>
       <c r="F6" s="83" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="G6" s="83" t="s">
-        <v>2149</v>
+        <v>2150</v>
       </c>
       <c r="H6" s="83" t="s">
-        <v>2150</v>
+        <v>2151</v>
       </c>
       <c r="I6" s="82" t="s">
-        <v>2151</v>
+        <v>2152</v>
       </c>
       <c r="J6" s="82" t="s">
-        <v>2152</v>
+        <v>2153</v>
       </c>
       <c r="K6" s="83" t="s">
-        <v>2153</v>
+        <v>2154</v>
       </c>
       <c r="L6" s="83" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="M6" s="83" t="s">
-        <v>2155</v>
+        <v>2156</v>
       </c>
       <c r="N6" s="83" t="s">
-        <v>2156</v>
+        <v>2157</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71717,40 +71728,40 @@
         <v>576</v>
       </c>
       <c r="B7" s="82" t="s">
-        <v>2157</v>
+        <v>2158</v>
       </c>
       <c r="C7" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E7" s="83" t="s">
-        <v>2158</v>
+        <v>2159</v>
       </c>
       <c r="F7" s="83" t="s">
-        <v>2159</v>
+        <v>2160</v>
       </c>
       <c r="G7" s="83" t="s">
-        <v>2160</v>
+        <v>2161</v>
       </c>
       <c r="H7" s="83" t="s">
-        <v>2161</v>
+        <v>2162</v>
       </c>
       <c r="I7" s="82" t="s">
-        <v>2162</v>
+        <v>2163</v>
       </c>
       <c r="J7" s="82" t="s">
-        <v>2163</v>
+        <v>2164</v>
       </c>
       <c r="K7" s="83" t="s">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="L7" s="83" t="s">
-        <v>2165</v>
+        <v>2166</v>
       </c>
       <c r="M7" s="83" t="s">
-        <v>2166</v>
+        <v>2167</v>
       </c>
       <c r="N7" s="83" t="s">
-        <v>2167</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71758,40 +71769,40 @@
         <v>596</v>
       </c>
       <c r="B8" s="82" t="s">
-        <v>2168</v>
+        <v>2169</v>
       </c>
       <c r="C8" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E8" s="83" t="s">
-        <v>2169</v>
+        <v>2170</v>
       </c>
       <c r="F8" s="83" t="s">
-        <v>2170</v>
+        <v>2171</v>
       </c>
       <c r="G8" s="83" t="s">
-        <v>2171</v>
+        <v>2172</v>
       </c>
       <c r="H8" s="83" t="s">
-        <v>2172</v>
+        <v>2173</v>
       </c>
       <c r="I8" s="82" t="s">
-        <v>2173</v>
+        <v>2174</v>
       </c>
       <c r="J8" s="82" t="s">
-        <v>2174</v>
+        <v>2175</v>
       </c>
       <c r="K8" s="83" t="s">
-        <v>2175</v>
+        <v>2176</v>
       </c>
       <c r="L8" s="83" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="M8" s="83" t="s">
-        <v>2177</v>
+        <v>2178</v>
       </c>
       <c r="N8" s="83" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71799,40 +71810,40 @@
         <v>627</v>
       </c>
       <c r="B9" s="82" t="s">
-        <v>2179</v>
+        <v>2180</v>
       </c>
       <c r="C9" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E9" s="83" t="s">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="F9" s="83" t="s">
-        <v>2181</v>
+        <v>2182</v>
       </c>
       <c r="G9" s="83" t="s">
-        <v>2182</v>
+        <v>2183</v>
       </c>
       <c r="H9" s="83" t="s">
-        <v>2183</v>
+        <v>2184</v>
       </c>
       <c r="I9" s="82" t="s">
-        <v>2184</v>
+        <v>2185</v>
       </c>
       <c r="J9" s="82" t="s">
-        <v>2185</v>
+        <v>2186</v>
       </c>
       <c r="K9" s="83" t="s">
-        <v>2186</v>
+        <v>2187</v>
       </c>
       <c r="L9" s="83" t="s">
-        <v>2187</v>
+        <v>2188</v>
       </c>
       <c r="M9" s="83" t="s">
-        <v>2188</v>
+        <v>2189</v>
       </c>
       <c r="N9" s="83" t="s">
-        <v>2189</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -71840,202 +71851,202 @@
         <v>636</v>
       </c>
       <c r="B10" s="82" t="s">
-        <v>2190</v>
+        <v>2191</v>
       </c>
       <c r="E10" s="83" t="s">
-        <v>2191</v>
+        <v>2192</v>
       </c>
       <c r="F10" s="83" t="s">
-        <v>2191</v>
+        <v>2192</v>
       </c>
       <c r="G10" s="83" t="s">
-        <v>2192</v>
+        <v>2193</v>
       </c>
       <c r="H10" s="83" t="s">
-        <v>2193</v>
+        <v>2194</v>
       </c>
       <c r="I10" s="82" t="s">
-        <v>2194</v>
+        <v>2195</v>
       </c>
       <c r="J10" s="82" t="s">
-        <v>2195</v>
+        <v>2196</v>
       </c>
       <c r="K10" s="83" t="s">
-        <v>2196</v>
+        <v>2197</v>
       </c>
       <c r="L10" s="83" t="s">
-        <v>2196</v>
+        <v>2197</v>
       </c>
       <c r="M10" s="83" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
       <c r="N10" s="83" t="s">
-        <v>2198</v>
+        <v>2199</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="82" t="s">
-        <v>2199</v>
+        <v>2200</v>
       </c>
       <c r="B12" s="82" t="s">
-        <v>2200</v>
+        <v>2201</v>
       </c>
       <c r="C12" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E12" s="83" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="F12" s="83" t="s">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="G12" s="83" t="s">
-        <v>2203</v>
+        <v>2204</v>
       </c>
       <c r="H12" s="83" t="s">
-        <v>2204</v>
+        <v>2205</v>
       </c>
       <c r="I12" s="82" t="s">
-        <v>2205</v>
+        <v>2206</v>
       </c>
       <c r="J12" s="82" t="s">
-        <v>2206</v>
+        <v>2207</v>
       </c>
       <c r="K12" s="83" t="s">
-        <v>2207</v>
+        <v>2208</v>
       </c>
       <c r="L12" s="83" t="s">
-        <v>2208</v>
+        <v>2209</v>
       </c>
       <c r="M12" s="83" t="s">
-        <v>2209</v>
+        <v>2210</v>
       </c>
       <c r="N12" s="83" t="s">
-        <v>2210</v>
+        <v>2211</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="82" t="s">
-        <v>2211</v>
+        <v>2212</v>
       </c>
       <c r="B13" s="82" t="s">
-        <v>2212</v>
+        <v>2213</v>
       </c>
       <c r="C13" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E13" s="83" t="s">
-        <v>2213</v>
+        <v>2214</v>
       </c>
       <c r="F13" s="83" t="s">
-        <v>2214</v>
+        <v>2215</v>
       </c>
       <c r="G13" s="83" t="s">
-        <v>2215</v>
+        <v>2216</v>
       </c>
       <c r="H13" s="83" t="s">
-        <v>2216</v>
+        <v>2217</v>
       </c>
       <c r="I13" s="82" t="s">
-        <v>2217</v>
+        <v>2218</v>
       </c>
       <c r="J13" s="82" t="s">
-        <v>2218</v>
+        <v>2219</v>
       </c>
       <c r="K13" s="83" t="s">
-        <v>2219</v>
+        <v>2220</v>
       </c>
       <c r="L13" s="83" t="s">
-        <v>2220</v>
+        <v>2221</v>
       </c>
       <c r="M13" s="83" t="s">
-        <v>2221</v>
+        <v>2222</v>
       </c>
       <c r="N13" s="83" t="s">
-        <v>2222</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="82" t="s">
-        <v>2223</v>
+        <v>2224</v>
       </c>
       <c r="B14" s="82" t="s">
-        <v>2224</v>
+        <v>2225</v>
       </c>
       <c r="C14" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E14" s="83" t="s">
-        <v>2225</v>
+        <v>2226</v>
       </c>
       <c r="F14" s="83" t="s">
-        <v>2226</v>
+        <v>2227</v>
       </c>
       <c r="G14" s="83" t="s">
-        <v>2227</v>
+        <v>2228</v>
       </c>
       <c r="H14" s="83" t="s">
-        <v>2228</v>
+        <v>2229</v>
       </c>
       <c r="I14" s="82" t="s">
-        <v>2229</v>
+        <v>2230</v>
       </c>
       <c r="J14" s="82" t="s">
-        <v>2230</v>
+        <v>2231</v>
       </c>
       <c r="K14" s="83" t="s">
-        <v>2231</v>
+        <v>2232</v>
       </c>
       <c r="L14" s="83" t="s">
-        <v>2232</v>
+        <v>2233</v>
       </c>
       <c r="M14" s="83" t="s">
-        <v>2233</v>
+        <v>2234</v>
       </c>
       <c r="N14" s="83" t="s">
-        <v>2234</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="82" t="s">
-        <v>2235</v>
+        <v>2236</v>
       </c>
       <c r="B15" s="82" t="s">
-        <v>2236</v>
+        <v>2237</v>
       </c>
       <c r="C15" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E15" s="83" t="s">
-        <v>2237</v>
+        <v>2238</v>
       </c>
       <c r="F15" s="83" t="s">
-        <v>2237</v>
+        <v>2238</v>
       </c>
       <c r="G15" s="83" t="s">
-        <v>2238</v>
+        <v>2239</v>
       </c>
       <c r="H15" s="83" t="s">
-        <v>2239</v>
+        <v>2240</v>
       </c>
       <c r="I15" s="82" t="s">
-        <v>2240</v>
+        <v>2241</v>
       </c>
       <c r="J15" s="82" t="s">
-        <v>2241</v>
+        <v>2242</v>
       </c>
       <c r="K15" s="83" t="s">
-        <v>2242</v>
+        <v>2243</v>
       </c>
       <c r="L15" s="83" t="s">
-        <v>2242</v>
+        <v>2243</v>
       </c>
       <c r="M15" s="83" t="s">
-        <v>2243</v>
+        <v>2244</v>
       </c>
       <c r="N15" s="83" t="s">
-        <v>2244</v>
+        <v>2245</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -72044,40 +72055,40 @@
         <v>413</v>
       </c>
       <c r="B17" s="82" t="s">
-        <v>2245</v>
+        <v>2246</v>
       </c>
       <c r="C17" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E17" s="83" t="s">
-        <v>2246</v>
+        <v>2247</v>
       </c>
       <c r="F17" s="83" t="s">
-        <v>2247</v>
+        <v>2248</v>
       </c>
       <c r="G17" s="83" t="s">
-        <v>2248</v>
+        <v>2249</v>
       </c>
       <c r="H17" s="83" t="s">
-        <v>2249</v>
+        <v>2250</v>
       </c>
       <c r="I17" s="82" t="s">
-        <v>2250</v>
+        <v>2251</v>
       </c>
       <c r="J17" s="82" t="s">
-        <v>2251</v>
+        <v>2252</v>
       </c>
       <c r="K17" s="83" t="s">
-        <v>2252</v>
+        <v>2253</v>
       </c>
       <c r="L17" s="83" t="s">
-        <v>2253</v>
+        <v>2254</v>
       </c>
       <c r="M17" s="83" t="s">
-        <v>2254</v>
+        <v>2255</v>
       </c>
       <c r="N17" s="83" t="s">
-        <v>2255</v>
+        <v>2256</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -72085,40 +72096,40 @@
         <v>414</v>
       </c>
       <c r="B18" s="82" t="s">
-        <v>2256</v>
+        <v>2257</v>
       </c>
       <c r="C18" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E18" s="83" t="s">
-        <v>2257</v>
+        <v>2258</v>
       </c>
       <c r="F18" s="83" t="s">
-        <v>2258</v>
+        <v>2259</v>
       </c>
       <c r="G18" s="83" t="s">
-        <v>2259</v>
+        <v>2260</v>
       </c>
       <c r="H18" s="83" t="s">
-        <v>2260</v>
+        <v>2261</v>
       </c>
       <c r="I18" s="82" t="s">
-        <v>2261</v>
+        <v>2262</v>
       </c>
       <c r="J18" s="82" t="s">
-        <v>2262</v>
+        <v>2263</v>
       </c>
       <c r="K18" s="83" t="s">
-        <v>2263</v>
+        <v>2264</v>
       </c>
       <c r="L18" s="83" t="s">
-        <v>2264</v>
+        <v>2265</v>
       </c>
       <c r="M18" s="83" t="s">
-        <v>2265</v>
+        <v>2266</v>
       </c>
       <c r="N18" s="83" t="s">
-        <v>2266</v>
+        <v>2267</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -72129,597 +72140,597 @@
         <v>1300</v>
       </c>
       <c r="C19" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E19" s="83" t="s">
-        <v>2267</v>
+        <v>2268</v>
       </c>
       <c r="F19" s="83" t="s">
-        <v>2268</v>
+        <v>2269</v>
       </c>
       <c r="G19" s="83" t="s">
-        <v>2269</v>
+        <v>2270</v>
       </c>
       <c r="H19" s="83" t="s">
-        <v>2270</v>
+        <v>2271</v>
       </c>
       <c r="I19" s="82" t="s">
-        <v>2271</v>
+        <v>2272</v>
       </c>
       <c r="J19" s="82" t="s">
-        <v>2272</v>
+        <v>2273</v>
       </c>
       <c r="K19" s="83" t="s">
-        <v>2273</v>
+        <v>2274</v>
       </c>
       <c r="L19" s="83" t="s">
-        <v>2274</v>
+        <v>2275</v>
       </c>
       <c r="M19" s="83" t="s">
-        <v>2275</v>
+        <v>2276</v>
       </c>
       <c r="N19" s="83" t="s">
-        <v>2276</v>
+        <v>2277</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="82" t="s">
-        <v>2277</v>
+        <v>2278</v>
       </c>
       <c r="B21" s="82" t="s">
-        <v>2278</v>
+        <v>2279</v>
       </c>
       <c r="C21" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E21" s="83" t="s">
-        <v>2279</v>
+        <v>2280</v>
       </c>
       <c r="F21" s="83" t="s">
-        <v>2280</v>
+        <v>2281</v>
       </c>
       <c r="G21" s="83" t="s">
-        <v>2281</v>
+        <v>2282</v>
       </c>
       <c r="H21" s="83" t="s">
-        <v>2282</v>
+        <v>2283</v>
       </c>
       <c r="I21" s="82" t="s">
-        <v>2283</v>
+        <v>2284</v>
       </c>
       <c r="J21" s="82" t="s">
-        <v>2284</v>
+        <v>2285</v>
       </c>
       <c r="K21" s="83" t="s">
-        <v>2285</v>
+        <v>2286</v>
       </c>
       <c r="L21" s="83" t="s">
-        <v>2286</v>
+        <v>2287</v>
       </c>
       <c r="M21" s="83" t="s">
-        <v>2287</v>
+        <v>2288</v>
       </c>
       <c r="N21" s="83" t="s">
-        <v>2288</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="82" t="s">
-        <v>2289</v>
+        <v>2290</v>
       </c>
       <c r="B22" s="82" t="s">
-        <v>2290</v>
+        <v>2291</v>
       </c>
       <c r="C22" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E22" s="83" t="s">
-        <v>2291</v>
+        <v>2292</v>
       </c>
       <c r="F22" s="83" t="s">
-        <v>2292</v>
+        <v>2293</v>
       </c>
       <c r="G22" s="83" t="s">
-        <v>2293</v>
+        <v>2294</v>
       </c>
       <c r="H22" s="83" t="s">
-        <v>2294</v>
+        <v>2295</v>
       </c>
       <c r="I22" s="82" t="s">
-        <v>2295</v>
+        <v>2296</v>
       </c>
       <c r="J22" s="82" t="s">
-        <v>2296</v>
+        <v>2297</v>
       </c>
       <c r="K22" s="83" t="s">
-        <v>2297</v>
+        <v>2298</v>
       </c>
       <c r="L22" s="83" t="s">
-        <v>2298</v>
+        <v>2299</v>
       </c>
       <c r="M22" s="83" t="s">
-        <v>2299</v>
+        <v>2300</v>
       </c>
       <c r="N22" s="83" t="s">
-        <v>2300</v>
+        <v>2301</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="82" t="s">
-        <v>2301</v>
+        <v>2302</v>
       </c>
       <c r="B24" s="82" t="s">
-        <v>2302</v>
+        <v>2303</v>
       </c>
       <c r="C24" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D24" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E24" s="83" t="s">
-        <v>2303</v>
+        <v>2304</v>
       </c>
       <c r="F24" s="83" t="s">
-        <v>2304</v>
+        <v>2305</v>
       </c>
       <c r="G24" s="83" t="s">
-        <v>2305</v>
+        <v>2306</v>
       </c>
       <c r="H24" s="83" t="s">
-        <v>2306</v>
+        <v>2307</v>
       </c>
       <c r="I24" s="82" t="s">
-        <v>2307</v>
+        <v>2308</v>
       </c>
       <c r="J24" s="82" t="s">
-        <v>2308</v>
+        <v>2309</v>
       </c>
       <c r="K24" s="83" t="s">
-        <v>2309</v>
+        <v>2310</v>
       </c>
       <c r="L24" s="83" t="s">
-        <v>2310</v>
+        <v>2311</v>
       </c>
       <c r="M24" s="83" t="s">
-        <v>2311</v>
+        <v>2312</v>
       </c>
       <c r="N24" s="83" t="s">
-        <v>2312</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="82" t="s">
-        <v>2313</v>
+        <v>2314</v>
       </c>
       <c r="B25" s="82" t="s">
-        <v>2314</v>
+        <v>2315</v>
       </c>
       <c r="C25" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D25" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E25" s="83" t="s">
-        <v>2315</v>
+        <v>2316</v>
       </c>
       <c r="F25" s="83" t="s">
-        <v>2316</v>
+        <v>2317</v>
       </c>
       <c r="G25" s="83" t="s">
-        <v>2317</v>
+        <v>2318</v>
       </c>
       <c r="H25" s="83" t="s">
-        <v>2318</v>
+        <v>2319</v>
       </c>
       <c r="I25" s="82" t="s">
-        <v>2319</v>
+        <v>2320</v>
       </c>
       <c r="J25" s="82" t="s">
-        <v>2320</v>
+        <v>2321</v>
       </c>
       <c r="K25" s="83" t="s">
-        <v>2321</v>
+        <v>2322</v>
       </c>
       <c r="L25" s="83" t="s">
-        <v>2322</v>
+        <v>2323</v>
       </c>
       <c r="M25" s="83" t="s">
-        <v>2323</v>
+        <v>2324</v>
       </c>
       <c r="N25" s="83" t="s">
-        <v>2324</v>
+        <v>2325</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="82" t="s">
-        <v>2325</v>
+        <v>2326</v>
       </c>
       <c r="B26" s="82" t="s">
-        <v>2326</v>
+        <v>2327</v>
       </c>
       <c r="C26" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D26" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E26" s="83" t="s">
-        <v>2327</v>
+        <v>2328</v>
       </c>
       <c r="F26" s="83" t="s">
-        <v>2328</v>
+        <v>2329</v>
       </c>
       <c r="G26" s="83" t="s">
-        <v>2329</v>
+        <v>2330</v>
       </c>
       <c r="H26" s="83" t="s">
-        <v>2330</v>
+        <v>2331</v>
       </c>
       <c r="I26" s="82" t="s">
-        <v>2331</v>
+        <v>2332</v>
       </c>
       <c r="J26" s="82" t="s">
-        <v>2332</v>
+        <v>2333</v>
       </c>
       <c r="K26" s="83" t="s">
-        <v>2333</v>
+        <v>2334</v>
       </c>
       <c r="L26" s="83" t="s">
-        <v>2334</v>
+        <v>2335</v>
       </c>
       <c r="M26" s="83" t="s">
-        <v>2335</v>
+        <v>2336</v>
       </c>
       <c r="N26" s="83" t="s">
-        <v>2336</v>
+        <v>2337</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="82" t="s">
-        <v>2337</v>
+        <v>2338</v>
       </c>
       <c r="B27" s="82" t="s">
-        <v>2338</v>
+        <v>2339</v>
       </c>
       <c r="C27" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D27" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E27" s="83" t="s">
-        <v>2339</v>
+        <v>2340</v>
       </c>
       <c r="F27" s="83" t="s">
-        <v>2340</v>
+        <v>2341</v>
       </c>
       <c r="G27" s="83" t="s">
-        <v>2341</v>
+        <v>2342</v>
       </c>
       <c r="H27" s="83" t="s">
-        <v>2342</v>
+        <v>2343</v>
       </c>
       <c r="I27" s="82" t="s">
-        <v>2343</v>
+        <v>2344</v>
       </c>
       <c r="J27" s="82" t="s">
-        <v>2344</v>
+        <v>2345</v>
       </c>
       <c r="K27" s="83" t="s">
-        <v>2345</v>
+        <v>2346</v>
       </c>
       <c r="L27" s="83" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="M27" s="83" t="s">
-        <v>2346</v>
+        <v>2347</v>
       </c>
       <c r="N27" s="83" t="s">
-        <v>2347</v>
+        <v>2348</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="82" t="s">
-        <v>2348</v>
+        <v>2349</v>
       </c>
       <c r="B28" s="82" t="s">
-        <v>2349</v>
+        <v>2350</v>
       </c>
       <c r="C28" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D28" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E28" s="83" t="s">
-        <v>2350</v>
+        <v>2351</v>
       </c>
       <c r="F28" s="83" t="s">
-        <v>2351</v>
+        <v>2352</v>
       </c>
       <c r="G28" s="83" t="s">
-        <v>2352</v>
+        <v>2353</v>
       </c>
       <c r="H28" s="83" t="s">
-        <v>2353</v>
+        <v>2354</v>
       </c>
       <c r="I28" s="82" t="s">
-        <v>2354</v>
+        <v>2355</v>
       </c>
       <c r="J28" s="82" t="s">
-        <v>2355</v>
+        <v>2356</v>
       </c>
       <c r="K28" s="83" t="s">
-        <v>2356</v>
+        <v>2357</v>
       </c>
       <c r="L28" s="83" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="M28" s="83" t="s">
-        <v>2357</v>
+        <v>2358</v>
       </c>
       <c r="N28" s="83" t="s">
-        <v>2358</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="82" t="s">
-        <v>2359</v>
+        <v>2360</v>
       </c>
       <c r="B29" s="82" t="s">
-        <v>2360</v>
+        <v>2361</v>
       </c>
       <c r="C29" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D29" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E29" s="83" t="s">
-        <v>2361</v>
+        <v>2362</v>
       </c>
       <c r="F29" s="83" t="s">
-        <v>2362</v>
+        <v>2363</v>
       </c>
       <c r="G29" s="83" t="s">
-        <v>2363</v>
+        <v>2364</v>
       </c>
       <c r="H29" s="83" t="s">
-        <v>2364</v>
+        <v>2365</v>
       </c>
       <c r="I29" s="82" t="s">
-        <v>2365</v>
+        <v>2366</v>
       </c>
       <c r="J29" s="82" t="s">
-        <v>2366</v>
+        <v>2367</v>
       </c>
       <c r="K29" s="83" t="s">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="L29" s="83" t="s">
-        <v>2368</v>
+        <v>2369</v>
       </c>
       <c r="M29" s="83" t="s">
-        <v>2369</v>
+        <v>2370</v>
       </c>
       <c r="N29" s="83" t="s">
-        <v>2370</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="82" t="s">
-        <v>2371</v>
+        <v>2372</v>
       </c>
       <c r="B30" s="82" t="s">
-        <v>2372</v>
+        <v>2373</v>
       </c>
       <c r="C30" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D30" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E30" s="83" t="s">
-        <v>2373</v>
+        <v>2374</v>
       </c>
       <c r="F30" s="83" t="s">
-        <v>2374</v>
+        <v>2375</v>
       </c>
       <c r="G30" s="83" t="s">
-        <v>2375</v>
+        <v>2376</v>
       </c>
       <c r="H30" s="83" t="s">
-        <v>2376</v>
+        <v>2377</v>
       </c>
       <c r="I30" s="82" t="s">
-        <v>2377</v>
+        <v>2378</v>
       </c>
       <c r="J30" s="82" t="s">
-        <v>2378</v>
+        <v>2379</v>
       </c>
       <c r="K30" s="83" t="s">
-        <v>2379</v>
+        <v>2380</v>
       </c>
       <c r="L30" s="83" t="s">
-        <v>2380</v>
+        <v>2381</v>
       </c>
       <c r="M30" s="83" t="s">
-        <v>2381</v>
+        <v>2382</v>
       </c>
       <c r="N30" s="83" t="s">
-        <v>2382</v>
+        <v>2383</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="82" t="s">
-        <v>2383</v>
+        <v>2384</v>
       </c>
       <c r="B31" s="82" t="s">
-        <v>2384</v>
+        <v>2385</v>
       </c>
       <c r="C31" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="D31" s="82" t="s">
-        <v>2091</v>
+        <v>2092</v>
       </c>
       <c r="E31" s="83" t="s">
-        <v>2385</v>
+        <v>2386</v>
       </c>
       <c r="F31" s="83" t="s">
-        <v>2386</v>
+        <v>2387</v>
       </c>
       <c r="G31" s="83" t="s">
-        <v>2387</v>
+        <v>2388</v>
       </c>
       <c r="H31" s="83" t="s">
-        <v>2388</v>
+        <v>2389</v>
       </c>
       <c r="I31" s="82" t="s">
-        <v>2389</v>
+        <v>2390</v>
       </c>
       <c r="J31" s="82" t="s">
-        <v>2390</v>
+        <v>2391</v>
       </c>
       <c r="K31" s="83" t="s">
-        <v>2391</v>
+        <v>2392</v>
       </c>
       <c r="L31" s="83" t="s">
-        <v>2392</v>
+        <v>2393</v>
       </c>
       <c r="M31" s="83" t="s">
-        <v>2393</v>
+        <v>2394</v>
       </c>
       <c r="N31" s="83" t="s">
-        <v>2394</v>
+        <v>2395</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="82" t="s">
-        <v>2395</v>
+        <v>2396</v>
       </c>
       <c r="B33" s="82" t="s">
-        <v>2396</v>
+        <v>2397</v>
       </c>
       <c r="C33" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E33" s="83" t="s">
-        <v>2397</v>
+        <v>2398</v>
       </c>
       <c r="F33" s="83" t="s">
-        <v>2398</v>
+        <v>2399</v>
       </c>
       <c r="G33" s="83" t="s">
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="H33" s="83" t="s">
-        <v>2400</v>
+        <v>2401</v>
       </c>
       <c r="I33" s="20" t="n">
         <v>1</v>
       </c>
       <c r="J33" s="82" t="s">
-        <v>2401</v>
+        <v>2402</v>
       </c>
       <c r="K33" s="83" t="s">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="L33" s="83" t="s">
-        <v>2403</v>
+        <v>2404</v>
       </c>
       <c r="M33" s="83" t="s">
-        <v>2404</v>
+        <v>2405</v>
       </c>
       <c r="N33" s="83" t="s">
-        <v>2405</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="82" t="s">
-        <v>2406</v>
+        <v>2407</v>
       </c>
       <c r="B34" s="82" t="s">
-        <v>2407</v>
+        <v>2408</v>
       </c>
       <c r="C34" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E34" s="83" t="s">
-        <v>2408</v>
+        <v>2409</v>
       </c>
       <c r="F34" s="83" t="s">
-        <v>2409</v>
+        <v>2410</v>
       </c>
       <c r="G34" s="83" t="s">
-        <v>2410</v>
+        <v>2411</v>
       </c>
       <c r="H34" s="83" t="s">
-        <v>2411</v>
+        <v>2412</v>
       </c>
       <c r="I34" s="20" t="n">
         <v>2</v>
       </c>
       <c r="J34" s="82" t="s">
-        <v>2412</v>
+        <v>2413</v>
       </c>
       <c r="K34" s="83" t="s">
-        <v>2413</v>
+        <v>2414</v>
       </c>
       <c r="L34" s="83" t="s">
-        <v>2414</v>
+        <v>2415</v>
       </c>
       <c r="M34" s="83" t="s">
-        <v>2415</v>
+        <v>2416</v>
       </c>
       <c r="N34" s="83" t="s">
-        <v>2416</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="82" t="s">
-        <v>2417</v>
+        <v>2418</v>
       </c>
       <c r="B35" s="82" t="s">
-        <v>2418</v>
+        <v>2419</v>
       </c>
       <c r="C35" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E35" s="83" t="s">
-        <v>2419</v>
+        <v>2420</v>
       </c>
       <c r="F35" s="83" t="s">
-        <v>2420</v>
+        <v>2421</v>
       </c>
       <c r="G35" s="83" t="s">
-        <v>2421</v>
+        <v>2422</v>
       </c>
       <c r="H35" s="83" t="s">
-        <v>2422</v>
+        <v>2423</v>
       </c>
       <c r="I35" s="20" t="n">
         <v>3</v>
       </c>
       <c r="J35" s="82" t="s">
-        <v>2423</v>
+        <v>2424</v>
       </c>
       <c r="K35" s="83" t="s">
-        <v>2424</v>
+        <v>2425</v>
       </c>
       <c r="L35" s="83" t="s">
-        <v>2425</v>
+        <v>2426</v>
       </c>
       <c r="M35" s="83" t="s">
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="N35" s="83" t="s">
-        <v>2427</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -72728,542 +72739,542 @@
         <v>32</v>
       </c>
       <c r="B37" s="82" t="s">
-        <v>2428</v>
+        <v>2429</v>
       </c>
       <c r="C37" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="G37" s="83" t="s">
-        <v>2429</v>
+        <v>2430</v>
       </c>
       <c r="H37" s="83" t="s">
-        <v>2429</v>
+        <v>2430</v>
       </c>
       <c r="I37" s="82" t="s">
-        <v>2430</v>
+        <v>2431</v>
       </c>
       <c r="J37" s="82" t="s">
-        <v>2431</v>
+        <v>2432</v>
       </c>
       <c r="M37" s="83" t="s">
-        <v>2432</v>
+        <v>2433</v>
       </c>
       <c r="N37" s="83" t="s">
-        <v>2433</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="B38" s="82" t="s">
-        <v>2434</v>
+        <v>2435</v>
       </c>
       <c r="C38" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E38" s="83" t="s">
-        <v>2435</v>
+        <v>2436</v>
       </c>
       <c r="F38" s="83" t="s">
-        <v>2435</v>
+        <v>2436</v>
       </c>
       <c r="G38" s="83" t="s">
-        <v>2436</v>
+        <v>2437</v>
       </c>
       <c r="H38" s="83" t="s">
-        <v>2437</v>
+        <v>2438</v>
       </c>
       <c r="I38" s="82" t="s">
-        <v>2438</v>
+        <v>2439</v>
       </c>
       <c r="J38" s="82" t="s">
-        <v>2439</v>
+        <v>2440</v>
       </c>
       <c r="K38" s="83" t="s">
-        <v>2440</v>
+        <v>2441</v>
       </c>
       <c r="L38" s="83" t="s">
-        <v>2440</v>
+        <v>2441</v>
       </c>
       <c r="M38" s="83" t="s">
-        <v>2441</v>
+        <v>2442</v>
       </c>
       <c r="N38" s="83" t="s">
-        <v>2442</v>
+        <v>2443</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="82" t="s">
-        <v>2443</v>
+        <v>2444</v>
       </c>
       <c r="B39" s="82" t="s">
-        <v>2444</v>
+        <v>2445</v>
       </c>
       <c r="C39" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E39" s="83" t="s">
-        <v>2445</v>
+        <v>2446</v>
       </c>
       <c r="F39" s="83" t="s">
-        <v>2445</v>
+        <v>2446</v>
       </c>
       <c r="G39" s="83" t="s">
-        <v>2446</v>
+        <v>2447</v>
       </c>
       <c r="H39" s="83" t="s">
-        <v>2447</v>
+        <v>2448</v>
       </c>
       <c r="I39" s="82" t="s">
-        <v>2448</v>
+        <v>2449</v>
       </c>
       <c r="J39" s="82" t="s">
-        <v>2449</v>
+        <v>2450</v>
       </c>
       <c r="K39" s="83" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="L39" s="83" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="M39" s="83" t="s">
-        <v>2451</v>
+        <v>2452</v>
       </c>
       <c r="N39" s="83" t="s">
-        <v>2452</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C40" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="82" t="s">
-        <v>2453</v>
+        <v>2454</v>
       </c>
       <c r="B41" s="82" t="s">
-        <v>2454</v>
+        <v>2455</v>
       </c>
       <c r="C41" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E41" s="83" t="s">
-        <v>2455</v>
+        <v>2456</v>
       </c>
       <c r="F41" s="83" t="s">
-        <v>2455</v>
+        <v>2456</v>
       </c>
       <c r="G41" s="83" t="s">
-        <v>2456</v>
+        <v>2457</v>
       </c>
       <c r="H41" s="83" t="s">
-        <v>2457</v>
+        <v>2458</v>
       </c>
       <c r="I41" s="82" t="s">
-        <v>2458</v>
+        <v>2459</v>
       </c>
       <c r="J41" s="82" t="s">
-        <v>2459</v>
+        <v>2460</v>
       </c>
       <c r="K41" s="83" t="s">
-        <v>2460</v>
+        <v>2461</v>
       </c>
       <c r="M41" s="83" t="s">
-        <v>2461</v>
+        <v>2462</v>
       </c>
       <c r="N41" s="83" t="s">
-        <v>2462</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="82" t="s">
-        <v>2463</v>
+        <v>2464</v>
       </c>
       <c r="B42" s="82" t="s">
-        <v>2464</v>
+        <v>2465</v>
       </c>
       <c r="C42" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E42" s="83" t="s">
-        <v>2465</v>
+        <v>2466</v>
       </c>
       <c r="F42" s="83" t="s">
-        <v>2465</v>
+        <v>2466</v>
       </c>
       <c r="G42" s="83" t="s">
-        <v>2466</v>
+        <v>2467</v>
       </c>
       <c r="H42" s="83" t="s">
-        <v>2467</v>
+        <v>2468</v>
       </c>
       <c r="I42" s="82" t="s">
-        <v>2468</v>
+        <v>2469</v>
       </c>
       <c r="J42" s="82" t="s">
-        <v>2469</v>
+        <v>2470</v>
       </c>
       <c r="K42" s="83" t="s">
-        <v>2470</v>
+        <v>2471</v>
       </c>
       <c r="L42" s="83" t="s">
-        <v>2471</v>
+        <v>2472</v>
       </c>
       <c r="M42" s="83" t="s">
-        <v>2472</v>
+        <v>2473</v>
       </c>
       <c r="N42" s="83" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="82" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
       <c r="B43" s="82" t="s">
-        <v>2475</v>
+        <v>2476</v>
       </c>
       <c r="C43" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E43" s="83" t="s">
-        <v>2476</v>
+        <v>2477</v>
       </c>
       <c r="F43" s="83" t="s">
-        <v>2477</v>
+        <v>2478</v>
       </c>
       <c r="G43" s="83" t="s">
-        <v>2478</v>
+        <v>2479</v>
       </c>
       <c r="H43" s="83" t="s">
-        <v>2479</v>
+        <v>2480</v>
       </c>
       <c r="I43" s="82" t="s">
-        <v>2480</v>
+        <v>2481</v>
       </c>
       <c r="J43" s="82" t="s">
-        <v>2481</v>
+        <v>2482</v>
       </c>
       <c r="M43" s="83" t="s">
-        <v>2482</v>
+        <v>2483</v>
       </c>
       <c r="N43" s="83" t="s">
-        <v>2483</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="82" t="s">
-        <v>2484</v>
+        <v>2485</v>
       </c>
       <c r="B44" s="82" t="s">
-        <v>2484</v>
+        <v>2485</v>
       </c>
       <c r="C44" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E44" s="83" t="s">
-        <v>2485</v>
+        <v>2486</v>
       </c>
       <c r="G44" s="83" t="s">
-        <v>2486</v>
+        <v>2487</v>
       </c>
       <c r="H44" s="83" t="s">
-        <v>2486</v>
+        <v>2487</v>
       </c>
       <c r="I44" s="82" t="s">
-        <v>2487</v>
+        <v>2488</v>
       </c>
       <c r="J44" s="82" t="s">
-        <v>2488</v>
+        <v>2489</v>
       </c>
       <c r="K44" s="83" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
       <c r="L44" s="83" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
       <c r="M44" s="83" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
       <c r="N44" s="83" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="82" t="s">
-        <v>2492</v>
+        <v>2493</v>
       </c>
       <c r="B45" s="82" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
       <c r="C45" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E45" s="83" t="s">
-        <v>2494</v>
+        <v>2495</v>
       </c>
       <c r="F45" s="83" t="s">
-        <v>2495</v>
+        <v>2496</v>
       </c>
       <c r="G45" s="83" t="s">
-        <v>2496</v>
+        <v>2497</v>
       </c>
       <c r="H45" s="83" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
       <c r="I45" s="82" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="J45" s="82" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="K45" s="83" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="L45" s="83" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="M45" s="83" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
       <c r="N45" s="83" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="82" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
       <c r="B46" s="82" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
       <c r="C46" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E46" s="83" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="F46" s="83" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="G46" s="83" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="H46" s="83" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
       <c r="I46" s="82" t="s">
-        <v>2507</v>
+        <v>2508</v>
       </c>
       <c r="J46" s="82" t="s">
-        <v>2508</v>
+        <v>2509</v>
       </c>
       <c r="K46" s="83" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="L46" s="83" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="M46" s="83" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
       <c r="N46" s="83" t="s">
-        <v>2511</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="82" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
       <c r="B47" s="82" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
       <c r="C47" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E47" s="83" t="s">
-        <v>2513</v>
+        <v>2514</v>
       </c>
       <c r="F47" s="83" t="s">
-        <v>2514</v>
+        <v>2515</v>
       </c>
       <c r="G47" s="83" t="s">
-        <v>2192</v>
+        <v>2193</v>
       </c>
       <c r="H47" s="83" t="s">
-        <v>2515</v>
+        <v>2516</v>
       </c>
       <c r="I47" s="82" t="s">
-        <v>2516</v>
+        <v>2517</v>
       </c>
       <c r="J47" s="82" t="s">
-        <v>2517</v>
+        <v>2518</v>
       </c>
       <c r="K47" s="83" t="s">
-        <v>2518</v>
+        <v>2519</v>
       </c>
       <c r="L47" s="83" t="s">
-        <v>2518</v>
+        <v>2519</v>
       </c>
       <c r="M47" s="83" t="s">
-        <v>2197</v>
+        <v>2198</v>
       </c>
       <c r="N47" s="83" t="s">
-        <v>2519</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="82" t="s">
-        <v>2520</v>
+        <v>2521</v>
       </c>
       <c r="B48" s="82" t="s">
-        <v>2521</v>
+        <v>2522</v>
       </c>
       <c r="C48" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E48" s="83" t="s">
-        <v>2522</v>
+        <v>2523</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>2522</v>
+        <v>2523</v>
       </c>
       <c r="G48" s="83" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
       <c r="H48" s="83" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
       <c r="I48" s="82" t="s">
-        <v>2524</v>
+        <v>2525</v>
       </c>
       <c r="J48" s="82" t="s">
-        <v>2525</v>
+        <v>2526</v>
       </c>
       <c r="K48" s="83" t="s">
-        <v>2526</v>
+        <v>2527</v>
       </c>
       <c r="L48" s="83" t="s">
-        <v>2526</v>
+        <v>2527</v>
       </c>
       <c r="M48" s="83" t="s">
-        <v>2527</v>
+        <v>2528</v>
       </c>
       <c r="N48" s="83" t="s">
-        <v>2527</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="82" t="s">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="B49" s="82" t="s">
-        <v>2529</v>
+        <v>2530</v>
       </c>
       <c r="C49" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E49" s="83" t="s">
-        <v>2530</v>
+        <v>2531</v>
       </c>
       <c r="F49" s="83" t="s">
-        <v>2530</v>
+        <v>2531</v>
       </c>
       <c r="G49" s="83" t="s">
-        <v>2456</v>
+        <v>2457</v>
       </c>
       <c r="H49" s="83" t="s">
-        <v>2457</v>
+        <v>2458</v>
       </c>
       <c r="I49" s="82" t="s">
-        <v>2531</v>
+        <v>2532</v>
       </c>
       <c r="J49" s="82" t="s">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="K49" s="83" t="s">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="L49" s="83" t="s">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="M49" s="83" t="s">
-        <v>2534</v>
+        <v>2535</v>
       </c>
       <c r="N49" s="83" t="s">
-        <v>2535</v>
+        <v>2536</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="82" t="s">
-        <v>2536</v>
+        <v>2537</v>
       </c>
       <c r="B50" s="82" t="s">
-        <v>2536</v>
+        <v>2537</v>
       </c>
       <c r="C50" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="G50" s="83" t="s">
-        <v>2537</v>
+        <v>2538</v>
       </c>
       <c r="H50" s="83" t="s">
-        <v>2537</v>
+        <v>2538</v>
       </c>
       <c r="I50" s="82" t="s">
-        <v>2538</v>
+        <v>2539</v>
       </c>
       <c r="J50" s="82" t="s">
-        <v>2538</v>
+        <v>2539</v>
       </c>
       <c r="M50" s="83" t="s">
-        <v>2539</v>
+        <v>2540</v>
       </c>
       <c r="N50" s="83" t="s">
-        <v>2540</v>
+        <v>2541</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="82" t="s">
-        <v>2541</v>
+        <v>2542</v>
       </c>
       <c r="B51" s="82" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="C51" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E51" s="83" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="F51" s="83" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="G51" s="83" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="H51" s="83" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="I51" s="82" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
       <c r="J51" s="82" t="s">
-        <v>2546</v>
+        <v>2547</v>
       </c>
       <c r="K51" s="83" t="s">
-        <v>2547</v>
+        <v>2548</v>
       </c>
       <c r="L51" s="83" t="s">
-        <v>2548</v>
+        <v>2549</v>
       </c>
       <c r="M51" s="83" t="s">
-        <v>2549</v>
+        <v>2550</v>
       </c>
       <c r="N51" s="83" t="s">
-        <v>2550</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -73274,498 +73285,498 @@
         <v>2</v>
       </c>
       <c r="C52" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E52" s="83" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
       <c r="F52" s="83" t="s">
-        <v>2552</v>
+        <v>2553</v>
       </c>
       <c r="G52" s="83" t="s">
-        <v>2553</v>
+        <v>2554</v>
       </c>
       <c r="H52" s="83" t="s">
-        <v>2553</v>
+        <v>2554</v>
       </c>
       <c r="I52" s="82" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
       <c r="J52" s="82" t="s">
-        <v>2554</v>
+        <v>2555</v>
       </c>
       <c r="K52" s="83" t="s">
-        <v>2555</v>
+        <v>2556</v>
       </c>
       <c r="L52" s="83" t="s">
-        <v>2555</v>
+        <v>2556</v>
       </c>
       <c r="M52" s="83" t="s">
-        <v>2556</v>
+        <v>2557</v>
       </c>
       <c r="N52" s="83" t="s">
-        <v>2557</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="82" t="s">
-        <v>2558</v>
+        <v>2559</v>
       </c>
       <c r="B53" s="82" t="s">
-        <v>2559</v>
+        <v>2560</v>
       </c>
       <c r="C53" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="G53" s="83" t="s">
-        <v>2560</v>
+        <v>2561</v>
       </c>
       <c r="H53" s="83" t="s">
-        <v>2561</v>
+        <v>2562</v>
       </c>
       <c r="I53" s="82" t="s">
-        <v>2562</v>
+        <v>2563</v>
       </c>
       <c r="J53" s="82" t="s">
-        <v>2563</v>
+        <v>2564</v>
       </c>
       <c r="K53" s="83" t="s">
-        <v>2564</v>
+        <v>2565</v>
       </c>
       <c r="L53" s="83" t="s">
-        <v>2564</v>
+        <v>2565</v>
       </c>
       <c r="M53" s="83" t="s">
-        <v>2565</v>
+        <v>2566</v>
       </c>
       <c r="N53" s="83" t="s">
-        <v>2566</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="82" t="s">
-        <v>2567</v>
+        <v>2568</v>
       </c>
       <c r="B54" s="82" t="s">
-        <v>2567</v>
+        <v>2568</v>
       </c>
       <c r="C54" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E54" s="83" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="F54" s="83" t="s">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="G54" s="83" t="s">
-        <v>2568</v>
+        <v>2569</v>
       </c>
       <c r="H54" s="83" t="s">
-        <v>2568</v>
+        <v>2569</v>
       </c>
       <c r="I54" s="82" t="s">
-        <v>2569</v>
+        <v>2570</v>
       </c>
       <c r="J54" s="82" t="s">
-        <v>2569</v>
+        <v>2570</v>
       </c>
       <c r="K54" s="83" t="s">
-        <v>2570</v>
+        <v>2571</v>
       </c>
       <c r="L54" s="83" t="s">
-        <v>2570</v>
+        <v>2571</v>
       </c>
       <c r="M54" s="83" t="s">
-        <v>2571</v>
+        <v>2572</v>
       </c>
       <c r="N54" s="83" t="s">
-        <v>2572</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="82" t="s">
-        <v>2573</v>
+        <v>2574</v>
       </c>
       <c r="B55" s="82" t="s">
-        <v>2574</v>
+        <v>2575</v>
       </c>
       <c r="C55" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E55" s="83" t="s">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="F55" s="83" t="s">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="G55" s="83" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="H55" s="83" t="s">
-        <v>2577</v>
+        <v>2578</v>
       </c>
       <c r="I55" s="82" t="s">
-        <v>2578</v>
+        <v>2579</v>
       </c>
       <c r="J55" s="82" t="s">
-        <v>2579</v>
+        <v>2580</v>
       </c>
       <c r="K55" s="83" t="s">
-        <v>2580</v>
+        <v>2581</v>
       </c>
       <c r="L55" s="83" t="s">
-        <v>2580</v>
+        <v>2581</v>
       </c>
       <c r="M55" s="83" t="s">
-        <v>2581</v>
+        <v>2582</v>
       </c>
       <c r="N55" s="83" t="s">
-        <v>2581</v>
+        <v>2582</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="82" t="s">
-        <v>2582</v>
+        <v>2583</v>
       </c>
       <c r="B56" s="82" t="s">
-        <v>2582</v>
+        <v>2583</v>
       </c>
       <c r="C56" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E56" s="83" t="s">
-        <v>2583</v>
+        <v>2584</v>
       </c>
       <c r="F56" s="83" t="s">
-        <v>2583</v>
+        <v>2584</v>
       </c>
       <c r="G56" s="83" t="s">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="H56" s="83" t="s">
-        <v>2585</v>
+        <v>2586</v>
       </c>
       <c r="I56" s="82" t="s">
-        <v>2586</v>
+        <v>2587</v>
       </c>
       <c r="J56" s="82" t="s">
-        <v>2587</v>
+        <v>2588</v>
       </c>
       <c r="K56" s="83" t="s">
-        <v>2588</v>
+        <v>2589</v>
       </c>
       <c r="L56" s="83" t="s">
-        <v>2588</v>
+        <v>2589</v>
       </c>
       <c r="M56" s="83" t="s">
-        <v>2589</v>
+        <v>2590</v>
       </c>
       <c r="N56" s="83" t="s">
-        <v>2590</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="82" t="s">
-        <v>2591</v>
+        <v>2592</v>
       </c>
       <c r="B57" s="82" t="s">
-        <v>2592</v>
+        <v>2593</v>
       </c>
       <c r="C57" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E57" s="83" t="s">
-        <v>2593</v>
+        <v>2594</v>
       </c>
       <c r="F57" s="83" t="s">
-        <v>2593</v>
+        <v>2594</v>
       </c>
       <c r="G57" s="83" t="s">
-        <v>2594</v>
+        <v>2595</v>
       </c>
       <c r="H57" s="83" t="s">
-        <v>2595</v>
+        <v>2596</v>
       </c>
       <c r="I57" s="82" t="s">
-        <v>2596</v>
+        <v>2597</v>
       </c>
       <c r="J57" s="82" t="s">
-        <v>2597</v>
+        <v>2598</v>
       </c>
       <c r="K57" s="83" t="s">
-        <v>2598</v>
+        <v>2599</v>
       </c>
       <c r="L57" s="83" t="s">
-        <v>2598</v>
+        <v>2599</v>
       </c>
       <c r="M57" s="83" t="s">
-        <v>2599</v>
+        <v>2600</v>
       </c>
       <c r="N57" s="83" t="s">
-        <v>2600</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="82" t="s">
-        <v>2601</v>
+        <v>2602</v>
       </c>
       <c r="B58" s="82" t="s">
-        <v>2602</v>
+        <v>2603</v>
       </c>
       <c r="C58" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E58" s="83" t="s">
-        <v>2603</v>
+        <v>2604</v>
       </c>
       <c r="F58" s="83" t="s">
-        <v>2604</v>
+        <v>2605</v>
       </c>
       <c r="G58" s="83" t="s">
-        <v>2605</v>
+        <v>2606</v>
       </c>
       <c r="H58" s="83" t="s">
-        <v>2606</v>
+        <v>2607</v>
       </c>
       <c r="I58" s="82" t="s">
-        <v>2607</v>
+        <v>2608</v>
       </c>
       <c r="J58" s="82" t="s">
-        <v>2608</v>
+        <v>2609</v>
       </c>
       <c r="K58" s="83" t="s">
-        <v>2609</v>
+        <v>2610</v>
       </c>
       <c r="L58" s="83" t="s">
-        <v>2609</v>
+        <v>2610</v>
       </c>
       <c r="M58" s="83" t="s">
-        <v>2610</v>
+        <v>2611</v>
       </c>
       <c r="N58" s="83" t="s">
-        <v>2610</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="82" t="s">
-        <v>2611</v>
+        <v>2612</v>
       </c>
       <c r="B59" s="82" t="s">
-        <v>2612</v>
+        <v>2613</v>
       </c>
       <c r="C59" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="G59" s="83" t="s">
-        <v>2613</v>
+        <v>2614</v>
       </c>
       <c r="H59" s="83" t="s">
-        <v>2614</v>
+        <v>2615</v>
       </c>
       <c r="I59" s="82" t="s">
-        <v>2615</v>
+        <v>2616</v>
       </c>
       <c r="J59" s="82" t="s">
-        <v>2616</v>
+        <v>2617</v>
       </c>
       <c r="K59" s="83" t="s">
-        <v>2617</v>
+        <v>2618</v>
       </c>
       <c r="L59" s="83" t="s">
-        <v>2617</v>
+        <v>2618</v>
       </c>
       <c r="M59" s="83" t="s">
-        <v>2618</v>
+        <v>2619</v>
       </c>
       <c r="N59" s="83" t="s">
-        <v>2618</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="82" t="s">
-        <v>2619</v>
+        <v>2620</v>
       </c>
       <c r="B60" s="82" t="s">
-        <v>2619</v>
+        <v>2620</v>
       </c>
       <c r="C60" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E60" s="83" t="s">
-        <v>2620</v>
+        <v>2621</v>
       </c>
       <c r="F60" s="83" t="s">
-        <v>2620</v>
+        <v>2621</v>
       </c>
       <c r="G60" s="83" t="s">
-        <v>2621</v>
+        <v>2622</v>
       </c>
       <c r="H60" s="83" t="s">
-        <v>2622</v>
+        <v>2623</v>
       </c>
       <c r="I60" s="82" t="s">
-        <v>2623</v>
+        <v>2624</v>
       </c>
       <c r="J60" s="82" t="s">
-        <v>2623</v>
+        <v>2624</v>
       </c>
       <c r="K60" s="83" t="s">
-        <v>2624</v>
+        <v>2625</v>
       </c>
       <c r="L60" s="83" t="s">
-        <v>2624</v>
+        <v>2625</v>
       </c>
       <c r="M60" s="83" t="s">
-        <v>2625</v>
+        <v>2626</v>
       </c>
       <c r="N60" s="83" t="s">
-        <v>2626</v>
+        <v>2627</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="82" t="s">
-        <v>2627</v>
+        <v>2628</v>
       </c>
       <c r="B61" s="82" t="s">
-        <v>2627</v>
+        <v>2628</v>
       </c>
       <c r="C61" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E61" s="83" t="s">
-        <v>2628</v>
+        <v>2629</v>
       </c>
       <c r="F61" s="83" t="s">
-        <v>2628</v>
+        <v>2629</v>
       </c>
       <c r="G61" s="83" t="s">
-        <v>2629</v>
+        <v>2630</v>
       </c>
       <c r="H61" s="83" t="s">
-        <v>2629</v>
+        <v>2630</v>
       </c>
       <c r="I61" s="82" t="s">
-        <v>2630</v>
+        <v>2631</v>
       </c>
       <c r="J61" s="82" t="s">
-        <v>2630</v>
+        <v>2631</v>
       </c>
       <c r="K61" s="83" t="s">
-        <v>2631</v>
+        <v>2632</v>
       </c>
       <c r="L61" s="83" t="s">
-        <v>2631</v>
+        <v>2632</v>
       </c>
       <c r="M61" s="83" t="s">
-        <v>2632</v>
+        <v>2633</v>
       </c>
       <c r="N61" s="83" t="s">
-        <v>2632</v>
+        <v>2633</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="82" t="s">
-        <v>2633</v>
+        <v>2634</v>
       </c>
       <c r="B62" s="82" t="s">
-        <v>2633</v>
+        <v>2634</v>
       </c>
       <c r="C62" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E62" s="83" t="s">
-        <v>2634</v>
+        <v>2635</v>
       </c>
       <c r="F62" s="83" t="s">
-        <v>2634</v>
+        <v>2635</v>
       </c>
       <c r="G62" s="83" t="s">
-        <v>2635</v>
+        <v>2636</v>
       </c>
       <c r="H62" s="83" t="s">
-        <v>2635</v>
+        <v>2636</v>
       </c>
       <c r="I62" s="82" t="s">
-        <v>2636</v>
+        <v>2637</v>
       </c>
       <c r="J62" s="82" t="s">
-        <v>2637</v>
+        <v>2638</v>
       </c>
       <c r="K62" s="83" t="s">
-        <v>2638</v>
+        <v>2639</v>
       </c>
       <c r="L62" s="83" t="s">
-        <v>2638</v>
+        <v>2639</v>
       </c>
       <c r="M62" s="83" t="s">
-        <v>2639</v>
+        <v>2640</v>
       </c>
       <c r="N62" s="83" t="s">
-        <v>2640</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="82" t="s">
-        <v>2641</v>
+        <v>2642</v>
       </c>
       <c r="B63" s="82" t="s">
-        <v>2642</v>
+        <v>2643</v>
       </c>
       <c r="C63" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
       <c r="E63" s="83" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="F63" s="83" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="G63" s="83" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="H63" s="83" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
       <c r="I63" s="82" t="s">
-        <v>2643</v>
+        <v>2644</v>
       </c>
       <c r="J63" s="82" t="s">
-        <v>2644</v>
+        <v>2645</v>
       </c>
       <c r="K63" s="83" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="L63" s="83" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
       <c r="M63" s="83" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
       <c r="N63" s="83" t="s">
-        <v>2511</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="82" t="s">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="B64" s="82" t="s">
-        <v>2645</v>
+        <v>2646</v>
       </c>
       <c r="C64" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="82" t="s">
-        <v>2646</v>
+        <v>2647</v>
       </c>
       <c r="B66" s="82" t="s">
-        <v>2647</v>
+        <v>2648</v>
       </c>
       <c r="C66" s="82" t="s">
-        <v>2090</v>
+        <v>2091</v>
       </c>
     </row>
   </sheetData>
@@ -73793,174 +73804,174 @@
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2"/>
       <c r="B1" s="84" t="s">
-        <v>2648</v>
+        <v>2649</v>
       </c>
       <c r="C1" s="84" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="84" t="s">
-        <v>2098</v>
+        <v>2099</v>
       </c>
       <c r="B2" s="84" t="s">
+        <v>2651</v>
+      </c>
+      <c r="C2" s="84" t="s">
         <v>2650</v>
-      </c>
-      <c r="C2" s="84" t="s">
-        <v>2649</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="84" t="s">
-        <v>2651</v>
+        <v>2652</v>
       </c>
       <c r="B3" s="84" t="s">
-        <v>2652</v>
+        <v>2653</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="84" t="s">
-        <v>2096</v>
+        <v>2097</v>
       </c>
       <c r="B4" s="84" t="s">
-        <v>2653</v>
+        <v>2654</v>
       </c>
       <c r="C4" s="84" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="84" t="s">
-        <v>2094</v>
+        <v>2095</v>
       </c>
       <c r="B5" s="84" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="C5" s="84" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="84" t="s">
-        <v>2655</v>
+        <v>2656</v>
       </c>
       <c r="B6" s="84" t="s">
-        <v>2656</v>
+        <v>2657</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="84" t="s">
-        <v>2657</v>
+        <v>2658</v>
       </c>
       <c r="B7" s="84" t="s">
-        <v>2658</v>
+        <v>2659</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="84" t="s">
-        <v>2659</v>
+        <v>2660</v>
       </c>
       <c r="B8" s="84" t="s">
-        <v>2660</v>
+        <v>2661</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="84" t="s">
-        <v>2661</v>
+        <v>2662</v>
       </c>
       <c r="B9" s="84" t="s">
-        <v>2662</v>
+        <v>2663</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="84" t="s">
-        <v>2663</v>
+        <v>2664</v>
       </c>
       <c r="B10" s="84" t="s">
-        <v>2664</v>
+        <v>2665</v>
       </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="84" t="s">
-        <v>2665</v>
+        <v>2666</v>
       </c>
       <c r="B11" s="84" t="s">
-        <v>2666</v>
+        <v>2667</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="84" t="s">
-        <v>2667</v>
+        <v>2668</v>
       </c>
       <c r="B12" s="84" t="s">
-        <v>2648</v>
+        <v>2649</v>
       </c>
       <c r="C12" s="84" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="84" t="s">
-        <v>2668</v>
+        <v>2669</v>
       </c>
       <c r="B13" s="84" t="s">
-        <v>2669</v>
+        <v>2670</v>
       </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="84" t="s">
-        <v>2670</v>
+        <v>2671</v>
       </c>
       <c r="B14" s="84" t="s">
-        <v>2671</v>
+        <v>2672</v>
       </c>
       <c r="C14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="84" t="s">
-        <v>2092</v>
+        <v>2093</v>
       </c>
       <c r="B15" s="84" t="s">
-        <v>2672</v>
+        <v>2673</v>
       </c>
       <c r="C15" s="84" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="84" t="s">
-        <v>2100</v>
+        <v>2101</v>
       </c>
       <c r="B16" s="84" t="s">
-        <v>2673</v>
+        <v>2674</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>2649</v>
+        <v>2650</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="84" t="s">
-        <v>2674</v>
+        <v>2675</v>
       </c>
       <c r="B17" s="84" t="s">
-        <v>2675</v>
+        <v>2676</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="84" t="s">
-        <v>2676</v>
+        <v>2677</v>
       </c>
       <c r="B18" s="84" t="s">
-        <v>2677</v>
+        <v>2678</v>
       </c>
       <c r="C18" s="2"/>
     </row>

</xml_diff>

<commit_message>
sync: selective update from as_upstream (10-02)
</commit_message>
<xml_diff>
--- a/db/inflections/inflection_templates.xlsx
+++ b/db/inflections/inflection_templates.xlsx
@@ -3310,7 +3310,28 @@
     <t xml:space="preserve">catunnaṃ</t>
   </si>
   <si>
-    <t xml:space="preserve">catassannaṃ</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Crimson Pro"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">catassannaṃ
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Crimson Pro"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">catunnaṃ</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">assa
@@ -9182,7 +9203,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -9271,6 +9292,13 @@
       <name val="Crimson Pro"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Crimson Pro"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -9783,11 +9811,11 @@
       <alignment horizontal="justify" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9795,11 +9823,11 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9823,7 +9851,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>

<commit_message>
#sync: upstream pull 518672a6..be49bffe, 363 files, 2026-07-09
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/db/inflections/inflection_templates.xlsx
+++ b/db/inflections/inflection_templates.xlsx
@@ -5186,31 +5186,11 @@
 antamhā</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Crimson Pro"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">viyā
+    <t xml:space="preserve">viyā
 vyā
 byā
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Crimson Pro"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">vito
+vito
 vīto</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">āmhe
@@ -5306,30 +5286,10 @@
 antamhi</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Crimson Pro"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">viyā
+    <t xml:space="preserve">viyā
 vyā
 byā
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Crimson Pro"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">viyaṃ</t>
-    </r>
+viyaṃ</t>
   </si>
   <si>
     <t xml:space="preserve">vīsu</t>
@@ -9291,7 +9251,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -9393,13 +9353,7 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Crimson Pro"/>
-      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -9613,7 +9567,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="86">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9918,10 +9872,6 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -9954,7 +9904,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -53668,7 +53618,7 @@
       <c r="CV91" s="2"/>
       <c r="CW91" s="2"/>
     </row>
-    <row r="92" customFormat="false" ht="41.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="41.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="21" t="s">
         <v>420</v>
       </c>
@@ -53963,7 +53913,7 @@
       </c>
       <c r="DA93" s="47"/>
     </row>
-    <row r="94" customFormat="false" ht="41.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="41.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="21" t="s">
         <v>485</v>
       </c>
@@ -54193,7 +54143,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="41.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="41.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="21" t="s">
         <v>522</v>
       </c>
@@ -54575,7 +54525,7 @@
       <c r="BQ96" s="27" t="s">
         <v>552</v>
       </c>
-      <c r="BR96" s="76" t="s">
+      <c r="BR96" s="27" t="s">
         <v>1483</v>
       </c>
       <c r="BS96" s="42" t="s">
@@ -55003,7 +54953,7 @@
       <c r="BQ98" s="27" t="s">
         <v>599</v>
       </c>
-      <c r="BR98" s="76" t="s">
+      <c r="BR98" s="27" t="s">
         <v>1507</v>
       </c>
       <c r="BS98" s="42" t="s">
@@ -55630,17 +55580,17 @@
         <v>409</v>
       </c>
       <c r="BI102" s="41"/>
-      <c r="BQ102" s="77" t="s">
+      <c r="BQ102" s="76" t="s">
         <v>251</v>
       </c>
-      <c r="BR102" s="77" t="s">
+      <c r="BR102" s="76" t="s">
         <v>410</v>
       </c>
-      <c r="BS102" s="78"/>
-      <c r="BT102" s="77" t="s">
+      <c r="BS102" s="77"/>
+      <c r="BT102" s="76" t="s">
         <v>411</v>
       </c>
-      <c r="BU102" s="78"/>
+      <c r="BU102" s="77"/>
       <c r="CC102" s="22"/>
       <c r="CD102" s="22"/>
       <c r="CF102" s="22"/>
@@ -55782,19 +55732,19 @@
       <c r="BI103" s="56" t="s">
         <v>424</v>
       </c>
-      <c r="BQ103" s="77" t="s">
+      <c r="BQ103" s="76" t="s">
         <v>420</v>
       </c>
-      <c r="BR103" s="77" t="s">
+      <c r="BR103" s="76" t="s">
         <v>1541</v>
       </c>
-      <c r="BS103" s="79" t="s">
+      <c r="BS103" s="78" t="s">
         <v>426</v>
       </c>
-      <c r="BT103" s="77" t="s">
+      <c r="BT103" s="76" t="s">
         <v>1542</v>
       </c>
-      <c r="BU103" s="79" t="s">
+      <c r="BU103" s="78" t="s">
         <v>428</v>
       </c>
       <c r="CC103" s="22"/>
@@ -55922,19 +55872,19 @@
       <c r="BI104" s="56" t="s">
         <v>461</v>
       </c>
-      <c r="BQ104" s="77" t="s">
+      <c r="BQ104" s="76" t="s">
         <v>458</v>
       </c>
-      <c r="BR104" s="77" t="s">
+      <c r="BR104" s="76" t="s">
         <v>1545</v>
       </c>
-      <c r="BS104" s="79" t="s">
+      <c r="BS104" s="78" t="s">
         <v>462</v>
       </c>
-      <c r="BT104" s="77" t="s">
+      <c r="BT104" s="76" t="s">
         <v>1542</v>
       </c>
-      <c r="BU104" s="79" t="s">
+      <c r="BU104" s="78" t="s">
         <v>463</v>
       </c>
       <c r="CC104" s="22"/>
@@ -56053,19 +56003,19 @@
       <c r="BI105" s="56" t="s">
         <v>489</v>
       </c>
-      <c r="BQ105" s="77" t="s">
+      <c r="BQ105" s="76" t="s">
         <v>485</v>
       </c>
-      <c r="BR105" s="77" t="s">
+      <c r="BR105" s="76" t="s">
         <v>1548</v>
       </c>
-      <c r="BS105" s="79" t="s">
+      <c r="BS105" s="78" t="s">
         <v>491</v>
       </c>
-      <c r="BT105" s="77" t="s">
+      <c r="BT105" s="76" t="s">
         <v>1549</v>
       </c>
-      <c r="BU105" s="79" t="s">
+      <c r="BU105" s="78" t="s">
         <v>493</v>
       </c>
       <c r="CC105" s="22"/>
@@ -56217,19 +56167,19 @@
       <c r="BI106" s="56" t="s">
         <v>526</v>
       </c>
-      <c r="BQ106" s="77" t="s">
+      <c r="BQ106" s="76" t="s">
         <v>522</v>
       </c>
-      <c r="BR106" s="77" t="s">
+      <c r="BR106" s="76" t="s">
         <v>1548</v>
       </c>
-      <c r="BS106" s="79" t="s">
+      <c r="BS106" s="78" t="s">
         <v>527</v>
       </c>
-      <c r="BT106" s="77" t="s">
+      <c r="BT106" s="76" t="s">
         <v>1552</v>
       </c>
-      <c r="BU106" s="79" t="s">
+      <c r="BU106" s="78" t="s">
         <v>529</v>
       </c>
       <c r="CC106" s="22"/>
@@ -56397,19 +56347,19 @@
       <c r="BI107" s="56" t="s">
         <v>555</v>
       </c>
-      <c r="BQ107" s="77" t="s">
+      <c r="BQ107" s="76" t="s">
         <v>552</v>
       </c>
-      <c r="BR107" s="77" t="s">
+      <c r="BR107" s="76" t="s">
         <v>1548</v>
       </c>
-      <c r="BS107" s="79" t="s">
+      <c r="BS107" s="78" t="s">
         <v>556</v>
       </c>
-      <c r="BT107" s="77" t="s">
+      <c r="BT107" s="76" t="s">
         <v>1549</v>
       </c>
-      <c r="BU107" s="79" t="s">
+      <c r="BU107" s="78" t="s">
         <v>557</v>
       </c>
       <c r="CC107" s="22"/>
@@ -56577,19 +56527,19 @@
       <c r="BI108" s="56" t="s">
         <v>582</v>
       </c>
-      <c r="BQ108" s="77" t="s">
+      <c r="BQ108" s="76" t="s">
         <v>579</v>
       </c>
-      <c r="BR108" s="77" t="s">
+      <c r="BR108" s="76" t="s">
         <v>1548</v>
       </c>
-      <c r="BS108" s="79" t="s">
+      <c r="BS108" s="78" t="s">
         <v>583</v>
       </c>
-      <c r="BT108" s="77" t="s">
+      <c r="BT108" s="76" t="s">
         <v>1552</v>
       </c>
-      <c r="BU108" s="79" t="s">
+      <c r="BU108" s="78" t="s">
         <v>584</v>
       </c>
       <c r="CC108" s="22"/>
@@ -56757,19 +56707,19 @@
       <c r="BI109" s="56" t="s">
         <v>603</v>
       </c>
-      <c r="BQ109" s="77" t="s">
+      <c r="BQ109" s="76" t="s">
         <v>599</v>
       </c>
-      <c r="BR109" s="77" t="s">
+      <c r="BR109" s="76" t="s">
         <v>1583</v>
       </c>
-      <c r="BS109" s="79" t="s">
+      <c r="BS109" s="78" t="s">
         <v>605</v>
       </c>
-      <c r="BT109" s="77" t="s">
+      <c r="BT109" s="76" t="s">
         <v>1584</v>
       </c>
-      <c r="BU109" s="79" t="s">
+      <c r="BU109" s="78" t="s">
         <v>607</v>
       </c>
       <c r="CC109" s="22"/>
@@ -56919,19 +56869,19 @@
       <c r="BI110" s="56" t="s">
         <v>633</v>
       </c>
-      <c r="BQ110" s="77" t="s">
+      <c r="BQ110" s="76" t="s">
         <v>630</v>
       </c>
-      <c r="BR110" s="77" t="s">
+      <c r="BR110" s="76" t="s">
         <v>1541</v>
       </c>
-      <c r="BS110" s="79" t="s">
+      <c r="BS110" s="78" t="s">
         <v>634</v>
       </c>
-      <c r="BT110" s="77" t="s">
+      <c r="BT110" s="76" t="s">
         <v>1588</v>
       </c>
-      <c r="BU110" s="79" t="s">
+      <c r="BU110" s="78" t="s">
         <v>635</v>
       </c>
       <c r="CC110" s="22"/>
@@ -57033,17 +56983,17 @@
       </c>
       <c r="BH111" s="41"/>
       <c r="BI111" s="56"/>
-      <c r="BQ111" s="77" t="s">
+      <c r="BQ111" s="76" t="s">
         <v>639</v>
       </c>
-      <c r="BR111" s="77" t="s">
+      <c r="BR111" s="76" t="s">
         <v>1541</v>
       </c>
       <c r="BS111" s="57" t="s">
         <v>639</v>
       </c>
-      <c r="BT111" s="77"/>
-      <c r="BU111" s="78"/>
+      <c r="BT111" s="76"/>
+      <c r="BU111" s="77"/>
       <c r="CC111" s="22"/>
       <c r="CD111" s="22"/>
       <c r="CF111" s="22"/>
@@ -57264,17 +57214,17 @@
         <v>409</v>
       </c>
       <c r="BI113" s="41"/>
-      <c r="BQ113" s="77" t="s">
+      <c r="BQ113" s="76" t="s">
         <v>253</v>
       </c>
-      <c r="BR113" s="77" t="s">
+      <c r="BR113" s="76" t="s">
         <v>410</v>
       </c>
-      <c r="BS113" s="78"/>
-      <c r="BT113" s="77" t="s">
+      <c r="BS113" s="77"/>
+      <c r="BT113" s="76" t="s">
         <v>411</v>
       </c>
-      <c r="BU113" s="78"/>
+      <c r="BU113" s="77"/>
       <c r="CC113" s="22"/>
       <c r="CD113" s="22"/>
       <c r="CF113" s="22"/>
@@ -57440,25 +57390,25 @@
       <c r="BI114" s="56" t="s">
         <v>424</v>
       </c>
-      <c r="BQ114" s="77" t="s">
+      <c r="BQ114" s="76" t="s">
         <v>420</v>
       </c>
-      <c r="BR114" s="77" t="s">
+      <c r="BR114" s="76" t="s">
         <v>1615</v>
       </c>
-      <c r="BS114" s="79" t="s">
+      <c r="BS114" s="78" t="s">
         <v>426</v>
       </c>
-      <c r="BT114" s="77" t="s">
+      <c r="BT114" s="76" t="s">
         <v>1616</v>
       </c>
-      <c r="BU114" s="79" t="s">
+      <c r="BU114" s="78" t="s">
         <v>428</v>
       </c>
       <c r="CC114" s="22"/>
       <c r="CD114" s="22"/>
       <c r="CF114" s="22"/>
-      <c r="CI114" s="80" t="s">
+      <c r="CI114" s="79" t="s">
         <v>736</v>
       </c>
       <c r="CJ114" s="59" t="s">
@@ -57620,19 +57570,19 @@
       <c r="BI115" s="56" t="s">
         <v>461</v>
       </c>
-      <c r="BQ115" s="77" t="s">
+      <c r="BQ115" s="76" t="s">
         <v>458</v>
       </c>
-      <c r="BR115" s="77" t="s">
+      <c r="BR115" s="76" t="s">
         <v>1627</v>
       </c>
-      <c r="BS115" s="79" t="s">
+      <c r="BS115" s="78" t="s">
         <v>462</v>
       </c>
-      <c r="BT115" s="77" t="s">
+      <c r="BT115" s="76" t="s">
         <v>1616</v>
       </c>
-      <c r="BU115" s="79" t="s">
+      <c r="BU115" s="78" t="s">
         <v>463</v>
       </c>
       <c r="CC115" s="22"/>
@@ -57782,19 +57732,19 @@
       <c r="BI116" s="56" t="s">
         <v>489</v>
       </c>
-      <c r="BQ116" s="77" t="s">
+      <c r="BQ116" s="76" t="s">
         <v>485</v>
       </c>
-      <c r="BR116" s="77" t="s">
+      <c r="BR116" s="76" t="s">
         <v>1641</v>
       </c>
-      <c r="BS116" s="79" t="s">
+      <c r="BS116" s="78" t="s">
         <v>491</v>
       </c>
-      <c r="BT116" s="77" t="s">
+      <c r="BT116" s="76" t="s">
         <v>1642</v>
       </c>
-      <c r="BU116" s="79" t="s">
+      <c r="BU116" s="78" t="s">
         <v>493</v>
       </c>
       <c r="CC116" s="22"/>
@@ -57940,25 +57890,25 @@
       <c r="BI117" s="56" t="s">
         <v>526</v>
       </c>
-      <c r="BQ117" s="77" t="s">
+      <c r="BQ117" s="76" t="s">
         <v>522</v>
       </c>
-      <c r="BR117" s="77" t="s">
+      <c r="BR117" s="76" t="s">
         <v>1641</v>
       </c>
-      <c r="BS117" s="79" t="s">
+      <c r="BS117" s="78" t="s">
         <v>527</v>
       </c>
-      <c r="BT117" s="77" t="s">
+      <c r="BT117" s="76" t="s">
         <v>1654</v>
       </c>
-      <c r="BU117" s="79" t="s">
+      <c r="BU117" s="78" t="s">
         <v>529</v>
       </c>
       <c r="CC117" s="22"/>
       <c r="CD117" s="22"/>
       <c r="CF117" s="22"/>
-      <c r="CI117" s="81" t="s">
+      <c r="CI117" s="80" t="s">
         <v>321</v>
       </c>
       <c r="CJ117" s="29" t="s">
@@ -58112,25 +58062,25 @@
       <c r="BI118" s="56" t="s">
         <v>555</v>
       </c>
-      <c r="BQ118" s="77" t="s">
+      <c r="BQ118" s="76" t="s">
         <v>552</v>
       </c>
-      <c r="BR118" s="77" t="s">
+      <c r="BR118" s="76" t="s">
         <v>1641</v>
       </c>
-      <c r="BS118" s="79" t="s">
+      <c r="BS118" s="78" t="s">
         <v>556</v>
       </c>
-      <c r="BT118" s="77" t="s">
+      <c r="BT118" s="76" t="s">
         <v>1642</v>
       </c>
-      <c r="BU118" s="79" t="s">
+      <c r="BU118" s="78" t="s">
         <v>557</v>
       </c>
       <c r="CC118" s="22"/>
       <c r="CD118" s="22"/>
       <c r="CF118" s="22"/>
-      <c r="CI118" s="80" t="s">
+      <c r="CI118" s="79" t="s">
         <v>1661</v>
       </c>
       <c r="CJ118" s="59" t="s">
@@ -58274,25 +58224,25 @@
       <c r="BI119" s="56" t="s">
         <v>582</v>
       </c>
-      <c r="BQ119" s="77" t="s">
+      <c r="BQ119" s="76" t="s">
         <v>579</v>
       </c>
-      <c r="BR119" s="77" t="s">
+      <c r="BR119" s="76" t="s">
         <v>1641</v>
       </c>
-      <c r="BS119" s="79" t="s">
+      <c r="BS119" s="78" t="s">
         <v>583</v>
       </c>
-      <c r="BT119" s="77" t="s">
+      <c r="BT119" s="76" t="s">
         <v>1654</v>
       </c>
-      <c r="BU119" s="79" t="s">
+      <c r="BU119" s="78" t="s">
         <v>584</v>
       </c>
       <c r="CC119" s="22"/>
       <c r="CD119" s="22"/>
       <c r="CF119" s="22"/>
-      <c r="CI119" s="80" t="s">
+      <c r="CI119" s="79" t="s">
         <v>1669</v>
       </c>
       <c r="CJ119" s="59" t="s">
@@ -58427,19 +58377,19 @@
       <c r="BI120" s="56" t="s">
         <v>603</v>
       </c>
-      <c r="BQ120" s="77" t="s">
+      <c r="BQ120" s="76" t="s">
         <v>599</v>
       </c>
-      <c r="BR120" s="77" t="s">
+      <c r="BR120" s="76" t="s">
         <v>1683</v>
       </c>
-      <c r="BS120" s="79" t="s">
+      <c r="BS120" s="78" t="s">
         <v>605</v>
       </c>
-      <c r="BT120" s="77" t="s">
+      <c r="BT120" s="76" t="s">
         <v>1684</v>
       </c>
-      <c r="BU120" s="79" t="s">
+      <c r="BU120" s="78" t="s">
         <v>607</v>
       </c>
       <c r="CC120" s="22"/>
@@ -58579,19 +58529,19 @@
       <c r="BI121" s="56" t="s">
         <v>633</v>
       </c>
-      <c r="BQ121" s="77" t="s">
+      <c r="BQ121" s="76" t="s">
         <v>630</v>
       </c>
-      <c r="BR121" s="77" t="s">
+      <c r="BR121" s="76" t="s">
         <v>1697</v>
       </c>
-      <c r="BS121" s="79" t="s">
+      <c r="BS121" s="78" t="s">
         <v>634</v>
       </c>
-      <c r="BT121" s="77" t="s">
+      <c r="BT121" s="76" t="s">
         <v>1616</v>
       </c>
-      <c r="BU121" s="79" t="s">
+      <c r="BU121" s="78" t="s">
         <v>635</v>
       </c>
       <c r="CC121" s="22"/>
@@ -58685,17 +58635,17 @@
       </c>
       <c r="BH122" s="41"/>
       <c r="BI122" s="56"/>
-      <c r="BQ122" s="77" t="s">
+      <c r="BQ122" s="76" t="s">
         <v>639</v>
       </c>
-      <c r="BR122" s="77" t="s">
+      <c r="BR122" s="76" t="s">
         <v>1697</v>
       </c>
       <c r="BS122" s="57" t="s">
         <v>639</v>
       </c>
-      <c r="BT122" s="77"/>
-      <c r="BU122" s="78"/>
+      <c r="BT122" s="76"/>
+      <c r="BU122" s="77"/>
       <c r="CC122" s="22"/>
       <c r="CD122" s="22"/>
       <c r="CF122" s="22"/>
@@ -58900,17 +58850,17 @@
         <v>409</v>
       </c>
       <c r="BI124" s="41"/>
-      <c r="BQ124" s="77" t="s">
+      <c r="BQ124" s="76" t="s">
         <v>255</v>
       </c>
-      <c r="BR124" s="77" t="s">
+      <c r="BR124" s="76" t="s">
         <v>410</v>
       </c>
-      <c r="BS124" s="78"/>
-      <c r="BT124" s="77" t="s">
+      <c r="BS124" s="77"/>
+      <c r="BT124" s="76" t="s">
         <v>411</v>
       </c>
-      <c r="BU124" s="78"/>
+      <c r="BU124" s="77"/>
       <c r="CC124" s="22"/>
       <c r="CD124" s="22"/>
       <c r="CF124" s="22"/>
@@ -59064,19 +59014,19 @@
       <c r="BI125" s="56" t="s">
         <v>424</v>
       </c>
-      <c r="BQ125" s="77" t="s">
+      <c r="BQ125" s="76" t="s">
         <v>420</v>
       </c>
-      <c r="BR125" s="77" t="s">
+      <c r="BR125" s="76" t="s">
         <v>1724</v>
       </c>
-      <c r="BS125" s="79" t="s">
+      <c r="BS125" s="78" t="s">
         <v>426</v>
       </c>
-      <c r="BT125" s="77" t="s">
+      <c r="BT125" s="76" t="s">
         <v>1725</v>
       </c>
-      <c r="BU125" s="79" t="s">
+      <c r="BU125" s="78" t="s">
         <v>428</v>
       </c>
       <c r="CC125" s="22"/>
@@ -59244,19 +59194,19 @@
       <c r="BI126" s="56" t="s">
         <v>461</v>
       </c>
-      <c r="BQ126" s="77" t="s">
+      <c r="BQ126" s="76" t="s">
         <v>458</v>
       </c>
-      <c r="BR126" s="77" t="s">
+      <c r="BR126" s="76" t="s">
         <v>1740</v>
       </c>
-      <c r="BS126" s="79" t="s">
+      <c r="BS126" s="78" t="s">
         <v>462</v>
       </c>
-      <c r="BT126" s="77" t="s">
+      <c r="BT126" s="76" t="s">
         <v>1725</v>
       </c>
-      <c r="BU126" s="79" t="s">
+      <c r="BU126" s="78" t="s">
         <v>463</v>
       </c>
       <c r="CC126" s="22"/>
@@ -59424,19 +59374,19 @@
       <c r="BI127" s="56" t="s">
         <v>489</v>
       </c>
-      <c r="BQ127" s="77" t="s">
+      <c r="BQ127" s="76" t="s">
         <v>485</v>
       </c>
-      <c r="BR127" s="77" t="s">
+      <c r="BR127" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="BS127" s="79" t="s">
+      <c r="BS127" s="78" t="s">
         <v>491</v>
       </c>
-      <c r="BT127" s="77" t="s">
+      <c r="BT127" s="76" t="s">
         <v>1756</v>
       </c>
-      <c r="BU127" s="79" t="s">
+      <c r="BU127" s="78" t="s">
         <v>493</v>
       </c>
       <c r="CC127" s="22"/>
@@ -59584,19 +59534,19 @@
       <c r="BI128" s="56" t="s">
         <v>526</v>
       </c>
-      <c r="BQ128" s="77" t="s">
+      <c r="BQ128" s="76" t="s">
         <v>522</v>
       </c>
-      <c r="BR128" s="77" t="s">
+      <c r="BR128" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="BS128" s="79" t="s">
+      <c r="BS128" s="78" t="s">
         <v>527</v>
       </c>
-      <c r="BT128" s="77" t="s">
+      <c r="BT128" s="76" t="s">
         <v>1767</v>
       </c>
-      <c r="BU128" s="79" t="s">
+      <c r="BU128" s="78" t="s">
         <v>529</v>
       </c>
       <c r="CC128" s="22"/>
@@ -59733,19 +59683,19 @@
       <c r="BI129" s="56" t="s">
         <v>555</v>
       </c>
-      <c r="BQ129" s="77" t="s">
+      <c r="BQ129" s="76" t="s">
         <v>552</v>
       </c>
-      <c r="BR129" s="77" t="s">
+      <c r="BR129" s="76" t="s">
         <v>1776</v>
       </c>
-      <c r="BS129" s="79" t="s">
+      <c r="BS129" s="78" t="s">
         <v>556</v>
       </c>
-      <c r="BT129" s="77" t="s">
+      <c r="BT129" s="76" t="s">
         <v>1756</v>
       </c>
-      <c r="BU129" s="79" t="s">
+      <c r="BU129" s="78" t="s">
         <v>557</v>
       </c>
       <c r="CC129" s="22"/>
@@ -59905,19 +59855,19 @@
       <c r="BI130" s="56" t="s">
         <v>582</v>
       </c>
-      <c r="BQ130" s="77" t="s">
+      <c r="BQ130" s="76" t="s">
         <v>579</v>
       </c>
-      <c r="BR130" s="77" t="s">
+      <c r="BR130" s="76" t="s">
         <v>1755</v>
       </c>
-      <c r="BS130" s="79" t="s">
+      <c r="BS130" s="78" t="s">
         <v>583</v>
       </c>
-      <c r="BT130" s="77" t="s">
+      <c r="BT130" s="76" t="s">
         <v>1767</v>
       </c>
-      <c r="BU130" s="79" t="s">
+      <c r="BU130" s="78" t="s">
         <v>584</v>
       </c>
       <c r="CC130" s="22"/>
@@ -60065,19 +60015,19 @@
       <c r="BI131" s="56" t="s">
         <v>603</v>
       </c>
-      <c r="BQ131" s="77" t="s">
+      <c r="BQ131" s="76" t="s">
         <v>599</v>
       </c>
-      <c r="BR131" s="77" t="s">
+      <c r="BR131" s="76" t="s">
         <v>1793</v>
       </c>
-      <c r="BS131" s="79" t="s">
+      <c r="BS131" s="78" t="s">
         <v>605</v>
       </c>
-      <c r="BT131" s="77" t="s">
+      <c r="BT131" s="76" t="s">
         <v>1794</v>
       </c>
-      <c r="BU131" s="79" t="s">
+      <c r="BU131" s="78" t="s">
         <v>607</v>
       </c>
       <c r="CC131" s="22"/>
@@ -60213,19 +60163,19 @@
       <c r="BI132" s="56" t="s">
         <v>633</v>
       </c>
-      <c r="BQ132" s="77" t="s">
+      <c r="BQ132" s="76" t="s">
         <v>630</v>
       </c>
-      <c r="BR132" s="77" t="s">
+      <c r="BR132" s="76" t="s">
         <v>1803</v>
       </c>
-      <c r="BS132" s="79" t="s">
+      <c r="BS132" s="78" t="s">
         <v>634</v>
       </c>
-      <c r="BT132" s="77" t="s">
+      <c r="BT132" s="76" t="s">
         <v>1725</v>
       </c>
-      <c r="BU132" s="79" t="s">
+      <c r="BU132" s="78" t="s">
         <v>635</v>
       </c>
       <c r="CC132" s="22"/>
@@ -60357,17 +60307,17 @@
       </c>
       <c r="BH133" s="41"/>
       <c r="BI133" s="56"/>
-      <c r="BQ133" s="77" t="s">
+      <c r="BQ133" s="76" t="s">
         <v>639</v>
       </c>
-      <c r="BR133" s="77" t="s">
+      <c r="BR133" s="76" t="s">
         <v>1813</v>
       </c>
       <c r="BS133" s="57" t="s">
         <v>639</v>
       </c>
-      <c r="BT133" s="77"/>
-      <c r="BU133" s="78"/>
+      <c r="BT133" s="76"/>
+      <c r="BU133" s="77"/>
       <c r="CC133" s="22"/>
       <c r="CD133" s="22"/>
       <c r="CF133" s="22"/>
@@ -61328,7 +61278,7 @@
       <c r="BI142" s="56" t="s">
         <v>603</v>
       </c>
-      <c r="BQ142" s="82" t="s">
+      <c r="BQ142" s="81" t="s">
         <v>599</v>
       </c>
       <c r="BR142" s="27" t="s">
@@ -61634,7 +61584,7 @@
       <c r="CC144" s="22"/>
       <c r="CD144" s="22"/>
       <c r="CF144" s="22"/>
-      <c r="CI144" s="80" t="s">
+      <c r="CI144" s="79" t="s">
         <v>736</v>
       </c>
       <c r="CJ144" s="59" t="s">
@@ -61827,7 +61777,7 @@
       <c r="CC146" s="22"/>
       <c r="CD146" s="22"/>
       <c r="CF146" s="22"/>
-      <c r="CI146" s="81" t="s">
+      <c r="CI146" s="80" t="s">
         <v>336</v>
       </c>
       <c r="CJ146" s="29" t="s">
@@ -61955,7 +61905,7 @@
       <c r="CC147" s="22"/>
       <c r="CD147" s="22"/>
       <c r="CF147" s="22"/>
-      <c r="CI147" s="80" t="s">
+      <c r="CI147" s="79" t="s">
         <v>1661</v>
       </c>
       <c r="CJ147" s="59" t="s">
@@ -62103,7 +62053,7 @@
       <c r="CC148" s="22"/>
       <c r="CD148" s="22"/>
       <c r="CF148" s="22"/>
-      <c r="CI148" s="80" t="s">
+      <c r="CI148" s="79" t="s">
         <v>1669</v>
       </c>
       <c r="CJ148" s="59" t="s">
@@ -71733,10 +71683,10 @@
       <c r="B1" s="22" t="s">
         <v>2106</v>
       </c>
-      <c r="C1" s="83" t="s">
+      <c r="C1" s="82" t="s">
         <v>2107</v>
       </c>
-      <c r="D1" s="83" t="s">
+      <c r="D1" s="82" t="s">
         <v>2108</v>
       </c>
       <c r="E1" s="22" t="s">
@@ -71748,2288 +71698,2288 @@
       <c r="G1" s="22" t="s">
         <v>2111</v>
       </c>
-      <c r="H1" s="83" t="s">
+      <c r="H1" s="82" t="s">
         <v>2112</v>
       </c>
       <c r="I1" s="22" t="s">
         <v>2113</v>
       </c>
-      <c r="J1" s="83" t="s">
+      <c r="J1" s="82" t="s">
         <v>2114</v>
       </c>
-      <c r="K1" s="83" t="s">
+      <c r="K1" s="82" t="s">
         <v>2115</v>
       </c>
-      <c r="L1" s="83" t="s">
+      <c r="L1" s="82" t="s">
         <v>2116</v>
       </c>
-      <c r="M1" s="83" t="s">
+      <c r="M1" s="82" t="s">
         <v>2117</v>
       </c>
-      <c r="N1" s="83" t="s">
+      <c r="N1" s="82" t="s">
         <v>2118</v>
       </c>
       <c r="AMI1" s="20"/>
       <c r="AMJ1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="84" t="s">
+      <c r="A2" s="83" t="s">
         <v>420</v>
       </c>
-      <c r="B2" s="84" t="s">
+      <c r="B2" s="83" t="s">
         <v>2119</v>
       </c>
-      <c r="C2" s="84" t="s">
+      <c r="C2" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E2" s="85" t="s">
+      <c r="E2" s="84" t="s">
         <v>2120</v>
       </c>
-      <c r="F2" s="85" t="s">
+      <c r="F2" s="84" t="s">
         <v>2121</v>
       </c>
-      <c r="G2" s="85" t="s">
+      <c r="G2" s="84" t="s">
         <v>2122</v>
       </c>
-      <c r="H2" s="85" t="s">
+      <c r="H2" s="84" t="s">
         <v>2123</v>
       </c>
-      <c r="I2" s="84" t="s">
+      <c r="I2" s="83" t="s">
         <v>2124</v>
       </c>
-      <c r="J2" s="84" t="s">
+      <c r="J2" s="83" t="s">
         <v>2125</v>
       </c>
-      <c r="K2" s="85" t="s">
+      <c r="K2" s="84" t="s">
         <v>2126</v>
       </c>
-      <c r="L2" s="85" t="s">
+      <c r="L2" s="84" t="s">
         <v>2127</v>
       </c>
-      <c r="M2" s="85" t="s">
+      <c r="M2" s="84" t="s">
         <v>2128</v>
       </c>
-      <c r="N2" s="85" t="s">
+      <c r="N2" s="84" t="s">
         <v>2129</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="83" t="s">
         <v>458</v>
       </c>
-      <c r="B3" s="84" t="s">
+      <c r="B3" s="83" t="s">
         <v>2130</v>
       </c>
-      <c r="C3" s="84" t="s">
+      <c r="C3" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E3" s="85" t="s">
+      <c r="E3" s="84" t="s">
         <v>2131</v>
       </c>
-      <c r="F3" s="85" t="s">
+      <c r="F3" s="84" t="s">
         <v>2132</v>
       </c>
-      <c r="G3" s="85" t="s">
+      <c r="G3" s="84" t="s">
         <v>2133</v>
       </c>
-      <c r="H3" s="85" t="s">
+      <c r="H3" s="84" t="s">
         <v>2134</v>
       </c>
-      <c r="I3" s="84" t="s">
+      <c r="I3" s="83" t="s">
         <v>2135</v>
       </c>
-      <c r="J3" s="84" t="s">
+      <c r="J3" s="83" t="s">
         <v>2136</v>
       </c>
-      <c r="K3" s="85" t="s">
+      <c r="K3" s="84" t="s">
         <v>2137</v>
       </c>
-      <c r="L3" s="85" t="s">
+      <c r="L3" s="84" t="s">
         <v>2138</v>
       </c>
-      <c r="M3" s="85" t="s">
+      <c r="M3" s="84" t="s">
         <v>2139</v>
       </c>
-      <c r="N3" s="85" t="s">
+      <c r="N3" s="84" t="s">
         <v>2140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="84" t="s">
+      <c r="A4" s="83" t="s">
         <v>485</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="83" t="s">
         <v>2141</v>
       </c>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E4" s="85" t="s">
+      <c r="E4" s="84" t="s">
         <v>2142</v>
       </c>
-      <c r="F4" s="85" t="s">
+      <c r="F4" s="84" t="s">
         <v>2143</v>
       </c>
-      <c r="G4" s="85" t="s">
+      <c r="G4" s="84" t="s">
         <v>2144</v>
       </c>
-      <c r="H4" s="85" t="s">
+      <c r="H4" s="84" t="s">
         <v>2145</v>
       </c>
-      <c r="I4" s="84" t="s">
+      <c r="I4" s="83" t="s">
         <v>2146</v>
       </c>
-      <c r="J4" s="84" t="s">
+      <c r="J4" s="83" t="s">
         <v>2147</v>
       </c>
-      <c r="K4" s="85" t="s">
+      <c r="K4" s="84" t="s">
         <v>2148</v>
       </c>
-      <c r="L4" s="85" t="s">
+      <c r="L4" s="84" t="s">
         <v>2149</v>
       </c>
-      <c r="M4" s="85" t="s">
+      <c r="M4" s="84" t="s">
         <v>2150</v>
       </c>
-      <c r="N4" s="85" t="s">
+      <c r="N4" s="84" t="s">
         <v>2151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="83" t="s">
         <v>522</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="83" t="s">
         <v>2152</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="C5" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E5" s="85" t="s">
+      <c r="E5" s="84" t="s">
         <v>2153</v>
       </c>
-      <c r="F5" s="85" t="s">
+      <c r="F5" s="84" t="s">
         <v>2154</v>
       </c>
-      <c r="G5" s="85" t="s">
+      <c r="G5" s="84" t="s">
         <v>2155</v>
       </c>
-      <c r="H5" s="85" t="s">
+      <c r="H5" s="84" t="s">
         <v>2156</v>
       </c>
-      <c r="I5" s="84" t="s">
+      <c r="I5" s="83" t="s">
         <v>2157</v>
       </c>
-      <c r="J5" s="84" t="s">
+      <c r="J5" s="83" t="s">
         <v>2158</v>
       </c>
-      <c r="K5" s="85" t="s">
+      <c r="K5" s="84" t="s">
         <v>2159</v>
       </c>
-      <c r="L5" s="85" t="s">
+      <c r="L5" s="84" t="s">
         <v>2160</v>
       </c>
-      <c r="M5" s="85" t="s">
+      <c r="M5" s="84" t="s">
         <v>2161</v>
       </c>
-      <c r="N5" s="85" t="s">
+      <c r="N5" s="84" t="s">
         <v>2162</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="84" t="s">
+      <c r="A6" s="83" t="s">
         <v>552</v>
       </c>
-      <c r="B6" s="84" t="s">
+      <c r="B6" s="83" t="s">
         <v>2163</v>
       </c>
-      <c r="C6" s="84" t="s">
+      <c r="C6" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E6" s="85" t="s">
+      <c r="E6" s="84" t="s">
         <v>2164</v>
       </c>
-      <c r="F6" s="85" t="s">
+      <c r="F6" s="84" t="s">
         <v>2165</v>
       </c>
-      <c r="G6" s="85" t="s">
+      <c r="G6" s="84" t="s">
         <v>2166</v>
       </c>
-      <c r="H6" s="85" t="s">
+      <c r="H6" s="84" t="s">
         <v>2167</v>
       </c>
-      <c r="I6" s="84" t="s">
+      <c r="I6" s="83" t="s">
         <v>2168</v>
       </c>
-      <c r="J6" s="84" t="s">
+      <c r="J6" s="83" t="s">
         <v>2169</v>
       </c>
-      <c r="K6" s="85" t="s">
+      <c r="K6" s="84" t="s">
         <v>2170</v>
       </c>
-      <c r="L6" s="85" t="s">
+      <c r="L6" s="84" t="s">
         <v>2171</v>
       </c>
-      <c r="M6" s="85" t="s">
+      <c r="M6" s="84" t="s">
         <v>2172</v>
       </c>
-      <c r="N6" s="85" t="s">
+      <c r="N6" s="84" t="s">
         <v>2173</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="84" t="s">
+      <c r="A7" s="83" t="s">
         <v>579</v>
       </c>
-      <c r="B7" s="84" t="s">
+      <c r="B7" s="83" t="s">
         <v>2174</v>
       </c>
-      <c r="C7" s="84" t="s">
+      <c r="C7" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E7" s="85" t="s">
+      <c r="E7" s="84" t="s">
         <v>2175</v>
       </c>
-      <c r="F7" s="85" t="s">
+      <c r="F7" s="84" t="s">
         <v>2176</v>
       </c>
-      <c r="G7" s="85" t="s">
+      <c r="G7" s="84" t="s">
         <v>2177</v>
       </c>
-      <c r="H7" s="85" t="s">
+      <c r="H7" s="84" t="s">
         <v>2178</v>
       </c>
-      <c r="I7" s="84" t="s">
+      <c r="I7" s="83" t="s">
         <v>2179</v>
       </c>
-      <c r="J7" s="84" t="s">
+      <c r="J7" s="83" t="s">
         <v>2180</v>
       </c>
-      <c r="K7" s="85" t="s">
+      <c r="K7" s="84" t="s">
         <v>2181</v>
       </c>
-      <c r="L7" s="85" t="s">
+      <c r="L7" s="84" t="s">
         <v>2182</v>
       </c>
-      <c r="M7" s="85" t="s">
+      <c r="M7" s="84" t="s">
         <v>2183</v>
       </c>
-      <c r="N7" s="85" t="s">
+      <c r="N7" s="84" t="s">
         <v>2184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="84" t="s">
+      <c r="A8" s="83" t="s">
         <v>599</v>
       </c>
-      <c r="B8" s="84" t="s">
+      <c r="B8" s="83" t="s">
         <v>2185</v>
       </c>
-      <c r="C8" s="84" t="s">
+      <c r="C8" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E8" s="85" t="s">
+      <c r="E8" s="84" t="s">
         <v>2186</v>
       </c>
-      <c r="F8" s="85" t="s">
+      <c r="F8" s="84" t="s">
         <v>2187</v>
       </c>
-      <c r="G8" s="85" t="s">
+      <c r="G8" s="84" t="s">
         <v>2188</v>
       </c>
-      <c r="H8" s="85" t="s">
+      <c r="H8" s="84" t="s">
         <v>2189</v>
       </c>
-      <c r="I8" s="84" t="s">
+      <c r="I8" s="83" t="s">
         <v>2190</v>
       </c>
-      <c r="J8" s="84" t="s">
+      <c r="J8" s="83" t="s">
         <v>2191</v>
       </c>
-      <c r="K8" s="85" t="s">
+      <c r="K8" s="84" t="s">
         <v>2192</v>
       </c>
-      <c r="L8" s="85" t="s">
+      <c r="L8" s="84" t="s">
         <v>2193</v>
       </c>
-      <c r="M8" s="85" t="s">
+      <c r="M8" s="84" t="s">
         <v>2194</v>
       </c>
-      <c r="N8" s="85" t="s">
+      <c r="N8" s="84" t="s">
         <v>2195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="84" t="s">
+      <c r="A9" s="83" t="s">
         <v>630</v>
       </c>
-      <c r="B9" s="84" t="s">
+      <c r="B9" s="83" t="s">
         <v>2196</v>
       </c>
-      <c r="C9" s="84" t="s">
+      <c r="C9" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E9" s="85" t="s">
+      <c r="E9" s="84" t="s">
         <v>2197</v>
       </c>
-      <c r="F9" s="85" t="s">
+      <c r="F9" s="84" t="s">
         <v>2198</v>
       </c>
-      <c r="G9" s="85" t="s">
+      <c r="G9" s="84" t="s">
         <v>2199</v>
       </c>
-      <c r="H9" s="85" t="s">
+      <c r="H9" s="84" t="s">
         <v>2200</v>
       </c>
-      <c r="I9" s="84" t="s">
+      <c r="I9" s="83" t="s">
         <v>2201</v>
       </c>
-      <c r="J9" s="84" t="s">
+      <c r="J9" s="83" t="s">
         <v>2202</v>
       </c>
-      <c r="K9" s="85" t="s">
+      <c r="K9" s="84" t="s">
         <v>2203</v>
       </c>
-      <c r="L9" s="85" t="s">
+      <c r="L9" s="84" t="s">
         <v>2204</v>
       </c>
-      <c r="M9" s="85" t="s">
+      <c r="M9" s="84" t="s">
         <v>2205</v>
       </c>
-      <c r="N9" s="85" t="s">
+      <c r="N9" s="84" t="s">
         <v>2206</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="84" t="s">
+      <c r="A10" s="83" t="s">
         <v>639</v>
       </c>
-      <c r="B10" s="84" t="s">
+      <c r="B10" s="83" t="s">
         <v>2207</v>
       </c>
-      <c r="E10" s="85" t="s">
+      <c r="E10" s="84" t="s">
         <v>2208</v>
       </c>
-      <c r="F10" s="85" t="s">
+      <c r="F10" s="84" t="s">
         <v>2208</v>
       </c>
-      <c r="G10" s="85" t="s">
+      <c r="G10" s="84" t="s">
         <v>2209</v>
       </c>
-      <c r="H10" s="85" t="s">
+      <c r="H10" s="84" t="s">
         <v>2210</v>
       </c>
-      <c r="I10" s="84" t="s">
+      <c r="I10" s="83" t="s">
         <v>2211</v>
       </c>
-      <c r="J10" s="84" t="s">
+      <c r="J10" s="83" t="s">
         <v>2212</v>
       </c>
-      <c r="K10" s="85" t="s">
+      <c r="K10" s="84" t="s">
         <v>2213</v>
       </c>
-      <c r="L10" s="85" t="s">
+      <c r="L10" s="84" t="s">
         <v>2213</v>
       </c>
-      <c r="M10" s="85" t="s">
+      <c r="M10" s="84" t="s">
         <v>2214</v>
       </c>
-      <c r="N10" s="85" t="s">
+      <c r="N10" s="84" t="s">
         <v>2215</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="84" t="s">
+      <c r="A12" s="83" t="s">
         <v>2216</v>
       </c>
-      <c r="B12" s="84" t="s">
+      <c r="B12" s="83" t="s">
         <v>2217</v>
       </c>
-      <c r="C12" s="84" t="s">
+      <c r="C12" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E12" s="85" t="s">
+      <c r="E12" s="84" t="s">
         <v>2218</v>
       </c>
-      <c r="F12" s="85" t="s">
+      <c r="F12" s="84" t="s">
         <v>2219</v>
       </c>
-      <c r="G12" s="85" t="s">
+      <c r="G12" s="84" t="s">
         <v>2220</v>
       </c>
-      <c r="H12" s="85" t="s">
+      <c r="H12" s="84" t="s">
         <v>2221</v>
       </c>
-      <c r="I12" s="84" t="s">
+      <c r="I12" s="83" t="s">
         <v>2222</v>
       </c>
-      <c r="J12" s="84" t="s">
+      <c r="J12" s="83" t="s">
         <v>2223</v>
       </c>
-      <c r="K12" s="85" t="s">
+      <c r="K12" s="84" t="s">
         <v>2224</v>
       </c>
-      <c r="L12" s="85" t="s">
+      <c r="L12" s="84" t="s">
         <v>2225</v>
       </c>
-      <c r="M12" s="85" t="s">
+      <c r="M12" s="84" t="s">
         <v>2226</v>
       </c>
-      <c r="N12" s="85" t="s">
+      <c r="N12" s="84" t="s">
         <v>2227</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="84" t="s">
+      <c r="A13" s="83" t="s">
         <v>2228</v>
       </c>
-      <c r="B13" s="84" t="s">
+      <c r="B13" s="83" t="s">
         <v>2229</v>
       </c>
-      <c r="C13" s="84" t="s">
+      <c r="C13" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E13" s="85" t="s">
+      <c r="E13" s="84" t="s">
         <v>2230</v>
       </c>
-      <c r="F13" s="85" t="s">
+      <c r="F13" s="84" t="s">
         <v>2231</v>
       </c>
-      <c r="G13" s="85" t="s">
+      <c r="G13" s="84" t="s">
         <v>2232</v>
       </c>
-      <c r="H13" s="85" t="s">
+      <c r="H13" s="84" t="s">
         <v>2233</v>
       </c>
-      <c r="I13" s="84" t="s">
+      <c r="I13" s="83" t="s">
         <v>2234</v>
       </c>
-      <c r="J13" s="84" t="s">
+      <c r="J13" s="83" t="s">
         <v>2235</v>
       </c>
-      <c r="K13" s="85" t="s">
+      <c r="K13" s="84" t="s">
         <v>2236</v>
       </c>
-      <c r="L13" s="85" t="s">
+      <c r="L13" s="84" t="s">
         <v>2237</v>
       </c>
-      <c r="M13" s="85" t="s">
+      <c r="M13" s="84" t="s">
         <v>2238</v>
       </c>
-      <c r="N13" s="85" t="s">
+      <c r="N13" s="84" t="s">
         <v>2239</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="84" t="s">
+      <c r="A14" s="83" t="s">
         <v>2240</v>
       </c>
-      <c r="B14" s="84" t="s">
+      <c r="B14" s="83" t="s">
         <v>2241</v>
       </c>
-      <c r="C14" s="84" t="s">
+      <c r="C14" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E14" s="85" t="s">
+      <c r="E14" s="84" t="s">
         <v>2242</v>
       </c>
-      <c r="F14" s="85" t="s">
+      <c r="F14" s="84" t="s">
         <v>2243</v>
       </c>
-      <c r="G14" s="85" t="s">
+      <c r="G14" s="84" t="s">
         <v>2244</v>
       </c>
-      <c r="H14" s="85" t="s">
+      <c r="H14" s="84" t="s">
         <v>2245</v>
       </c>
-      <c r="I14" s="84" t="s">
+      <c r="I14" s="83" t="s">
         <v>2246</v>
       </c>
-      <c r="J14" s="84" t="s">
+      <c r="J14" s="83" t="s">
         <v>2247</v>
       </c>
-      <c r="K14" s="85" t="s">
+      <c r="K14" s="84" t="s">
         <v>2248</v>
       </c>
-      <c r="L14" s="85" t="s">
+      <c r="L14" s="84" t="s">
         <v>2249</v>
       </c>
-      <c r="M14" s="85" t="s">
+      <c r="M14" s="84" t="s">
         <v>2250</v>
       </c>
-      <c r="N14" s="85" t="s">
+      <c r="N14" s="84" t="s">
         <v>2251</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="84" t="s">
+      <c r="A15" s="83" t="s">
         <v>2252</v>
       </c>
-      <c r="B15" s="84" t="s">
+      <c r="B15" s="83" t="s">
         <v>2253</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E15" s="85" t="s">
+      <c r="E15" s="84" t="s">
         <v>2254</v>
       </c>
-      <c r="F15" s="85" t="s">
+      <c r="F15" s="84" t="s">
         <v>2254</v>
       </c>
-      <c r="G15" s="85" t="s">
+      <c r="G15" s="84" t="s">
         <v>2255</v>
       </c>
-      <c r="H15" s="85" t="s">
+      <c r="H15" s="84" t="s">
         <v>2256</v>
       </c>
-      <c r="I15" s="84" t="s">
+      <c r="I15" s="83" t="s">
         <v>2257</v>
       </c>
-      <c r="J15" s="84" t="s">
+      <c r="J15" s="83" t="s">
         <v>2258</v>
       </c>
-      <c r="K15" s="85" t="s">
+      <c r="K15" s="84" t="s">
         <v>2259</v>
       </c>
-      <c r="L15" s="85" t="s">
+      <c r="L15" s="84" t="s">
         <v>2259</v>
       </c>
-      <c r="M15" s="85" t="s">
+      <c r="M15" s="84" t="s">
         <v>2260</v>
       </c>
-      <c r="N15" s="85" t="s">
+      <c r="N15" s="84" t="s">
         <v>2261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="84" t="s">
+      <c r="A17" s="83" t="s">
         <v>416</v>
       </c>
-      <c r="B17" s="84" t="s">
+      <c r="B17" s="83" t="s">
         <v>2262</v>
       </c>
-      <c r="C17" s="84" t="s">
+      <c r="C17" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E17" s="85" t="s">
+      <c r="E17" s="84" t="s">
         <v>2263</v>
       </c>
-      <c r="F17" s="85" t="s">
+      <c r="F17" s="84" t="s">
         <v>2264</v>
       </c>
-      <c r="G17" s="85" t="s">
+      <c r="G17" s="84" t="s">
         <v>2265</v>
       </c>
-      <c r="H17" s="85" t="s">
+      <c r="H17" s="84" t="s">
         <v>2266</v>
       </c>
-      <c r="I17" s="84" t="s">
+      <c r="I17" s="83" t="s">
         <v>2267</v>
       </c>
-      <c r="J17" s="84" t="s">
+      <c r="J17" s="83" t="s">
         <v>2268</v>
       </c>
-      <c r="K17" s="85" t="s">
+      <c r="K17" s="84" t="s">
         <v>2269</v>
       </c>
-      <c r="L17" s="85" t="s">
+      <c r="L17" s="84" t="s">
         <v>2270</v>
       </c>
-      <c r="M17" s="85" t="s">
+      <c r="M17" s="84" t="s">
         <v>2271</v>
       </c>
-      <c r="N17" s="85" t="s">
+      <c r="N17" s="84" t="s">
         <v>2272</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="84" t="s">
+      <c r="A18" s="83" t="s">
         <v>417</v>
       </c>
-      <c r="B18" s="84" t="s">
+      <c r="B18" s="83" t="s">
         <v>2273</v>
       </c>
-      <c r="C18" s="84" t="s">
+      <c r="C18" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E18" s="85" t="s">
+      <c r="E18" s="84" t="s">
         <v>2274</v>
       </c>
-      <c r="F18" s="85" t="s">
+      <c r="F18" s="84" t="s">
         <v>2275</v>
       </c>
-      <c r="G18" s="85" t="s">
+      <c r="G18" s="84" t="s">
         <v>2276</v>
       </c>
-      <c r="H18" s="85" t="s">
+      <c r="H18" s="84" t="s">
         <v>2277</v>
       </c>
-      <c r="I18" s="84" t="s">
+      <c r="I18" s="83" t="s">
         <v>2278</v>
       </c>
-      <c r="J18" s="84" t="s">
+      <c r="J18" s="83" t="s">
         <v>2279</v>
       </c>
-      <c r="K18" s="85" t="s">
+      <c r="K18" s="84" t="s">
         <v>2280</v>
       </c>
-      <c r="L18" s="85" t="s">
+      <c r="L18" s="84" t="s">
         <v>2281</v>
       </c>
-      <c r="M18" s="85" t="s">
+      <c r="M18" s="84" t="s">
         <v>2282</v>
       </c>
-      <c r="N18" s="85" t="s">
+      <c r="N18" s="84" t="s">
         <v>2283</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="84" t="s">
+      <c r="A19" s="83" t="s">
         <v>1305</v>
       </c>
-      <c r="B19" s="84" t="s">
+      <c r="B19" s="83" t="s">
         <v>1305</v>
       </c>
-      <c r="C19" s="84" t="s">
+      <c r="C19" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E19" s="85" t="s">
+      <c r="E19" s="84" t="s">
         <v>2284</v>
       </c>
-      <c r="F19" s="85" t="s">
+      <c r="F19" s="84" t="s">
         <v>2285</v>
       </c>
-      <c r="G19" s="85" t="s">
+      <c r="G19" s="84" t="s">
         <v>2286</v>
       </c>
-      <c r="H19" s="85" t="s">
+      <c r="H19" s="84" t="s">
         <v>2287</v>
       </c>
-      <c r="I19" s="84" t="s">
+      <c r="I19" s="83" t="s">
         <v>2288</v>
       </c>
-      <c r="J19" s="84" t="s">
+      <c r="J19" s="83" t="s">
         <v>2289</v>
       </c>
-      <c r="K19" s="85" t="s">
+      <c r="K19" s="84" t="s">
         <v>2290</v>
       </c>
-      <c r="L19" s="85" t="s">
+      <c r="L19" s="84" t="s">
         <v>2291</v>
       </c>
-      <c r="M19" s="85" t="s">
+      <c r="M19" s="84" t="s">
         <v>2292</v>
       </c>
-      <c r="N19" s="85" t="s">
+      <c r="N19" s="84" t="s">
         <v>2293</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="84" t="s">
+      <c r="A21" s="83" t="s">
         <v>2294</v>
       </c>
-      <c r="B21" s="84" t="s">
+      <c r="B21" s="83" t="s">
         <v>2295</v>
       </c>
-      <c r="C21" s="84" t="s">
+      <c r="C21" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E21" s="85" t="s">
+      <c r="E21" s="84" t="s">
         <v>2296</v>
       </c>
-      <c r="F21" s="85" t="s">
+      <c r="F21" s="84" t="s">
         <v>2297</v>
       </c>
-      <c r="G21" s="85" t="s">
+      <c r="G21" s="84" t="s">
         <v>2298</v>
       </c>
-      <c r="H21" s="85" t="s">
+      <c r="H21" s="84" t="s">
         <v>2299</v>
       </c>
-      <c r="I21" s="84" t="s">
+      <c r="I21" s="83" t="s">
         <v>2300</v>
       </c>
-      <c r="J21" s="84" t="s">
+      <c r="J21" s="83" t="s">
         <v>2301</v>
       </c>
-      <c r="K21" s="85" t="s">
+      <c r="K21" s="84" t="s">
         <v>2302</v>
       </c>
-      <c r="L21" s="85" t="s">
+      <c r="L21" s="84" t="s">
         <v>2303</v>
       </c>
-      <c r="M21" s="85" t="s">
+      <c r="M21" s="84" t="s">
         <v>2304</v>
       </c>
-      <c r="N21" s="85" t="s">
+      <c r="N21" s="84" t="s">
         <v>2305</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="84" t="s">
+      <c r="A22" s="83" t="s">
         <v>2306</v>
       </c>
-      <c r="B22" s="84" t="s">
+      <c r="B22" s="83" t="s">
         <v>2307</v>
       </c>
-      <c r="C22" s="84" t="s">
+      <c r="C22" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E22" s="85" t="s">
+      <c r="E22" s="84" t="s">
         <v>2308</v>
       </c>
-      <c r="F22" s="85" t="s">
+      <c r="F22" s="84" t="s">
         <v>2309</v>
       </c>
-      <c r="G22" s="85" t="s">
+      <c r="G22" s="84" t="s">
         <v>2310</v>
       </c>
-      <c r="H22" s="85" t="s">
+      <c r="H22" s="84" t="s">
         <v>2311</v>
       </c>
-      <c r="I22" s="84" t="s">
+      <c r="I22" s="83" t="s">
         <v>2312</v>
       </c>
-      <c r="J22" s="84" t="s">
+      <c r="J22" s="83" t="s">
         <v>2313</v>
       </c>
-      <c r="K22" s="85" t="s">
+      <c r="K22" s="84" t="s">
         <v>2314</v>
       </c>
-      <c r="L22" s="85" t="s">
+      <c r="L22" s="84" t="s">
         <v>2315</v>
       </c>
-      <c r="M22" s="85" t="s">
+      <c r="M22" s="84" t="s">
         <v>2316</v>
       </c>
-      <c r="N22" s="85" t="s">
+      <c r="N22" s="84" t="s">
         <v>2317</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="84" t="s">
+      <c r="A24" s="83" t="s">
         <v>2318</v>
       </c>
-      <c r="B24" s="84" t="s">
+      <c r="B24" s="83" t="s">
         <v>2319</v>
       </c>
-      <c r="C24" s="84" t="s">
+      <c r="C24" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D24" s="84" t="s">
+      <c r="D24" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E24" s="85" t="s">
+      <c r="E24" s="84" t="s">
         <v>2320</v>
       </c>
-      <c r="F24" s="85" t="s">
+      <c r="F24" s="84" t="s">
         <v>2321</v>
       </c>
-      <c r="G24" s="85" t="s">
+      <c r="G24" s="84" t="s">
         <v>2322</v>
       </c>
-      <c r="H24" s="85" t="s">
+      <c r="H24" s="84" t="s">
         <v>2323</v>
       </c>
-      <c r="I24" s="84" t="s">
+      <c r="I24" s="83" t="s">
         <v>2324</v>
       </c>
-      <c r="J24" s="84" t="s">
+      <c r="J24" s="83" t="s">
         <v>2325</v>
       </c>
-      <c r="K24" s="85" t="s">
+      <c r="K24" s="84" t="s">
         <v>2326</v>
       </c>
-      <c r="L24" s="85" t="s">
+      <c r="L24" s="84" t="s">
         <v>2327</v>
       </c>
-      <c r="M24" s="85" t="s">
+      <c r="M24" s="84" t="s">
         <v>2328</v>
       </c>
-      <c r="N24" s="85" t="s">
+      <c r="N24" s="84" t="s">
         <v>2329</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="84" t="s">
+      <c r="A25" s="83" t="s">
         <v>2330</v>
       </c>
-      <c r="B25" s="84" t="s">
+      <c r="B25" s="83" t="s">
         <v>2331</v>
       </c>
-      <c r="C25" s="84" t="s">
+      <c r="C25" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D25" s="84" t="s">
+      <c r="D25" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E25" s="85" t="s">
+      <c r="E25" s="84" t="s">
         <v>2332</v>
       </c>
-      <c r="F25" s="85" t="s">
+      <c r="F25" s="84" t="s">
         <v>2333</v>
       </c>
-      <c r="G25" s="85" t="s">
+      <c r="G25" s="84" t="s">
         <v>2334</v>
       </c>
-      <c r="H25" s="85" t="s">
+      <c r="H25" s="84" t="s">
         <v>2335</v>
       </c>
-      <c r="I25" s="84" t="s">
+      <c r="I25" s="83" t="s">
         <v>2336</v>
       </c>
-      <c r="J25" s="84" t="s">
+      <c r="J25" s="83" t="s">
         <v>2337</v>
       </c>
-      <c r="K25" s="85" t="s">
+      <c r="K25" s="84" t="s">
         <v>2338</v>
       </c>
-      <c r="L25" s="85" t="s">
+      <c r="L25" s="84" t="s">
         <v>2339</v>
       </c>
-      <c r="M25" s="85" t="s">
+      <c r="M25" s="84" t="s">
         <v>2340</v>
       </c>
-      <c r="N25" s="85" t="s">
+      <c r="N25" s="84" t="s">
         <v>2341</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="84" t="s">
+      <c r="A26" s="83" t="s">
         <v>2342</v>
       </c>
-      <c r="B26" s="84" t="s">
+      <c r="B26" s="83" t="s">
         <v>2343</v>
       </c>
-      <c r="C26" s="84" t="s">
+      <c r="C26" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D26" s="84" t="s">
+      <c r="D26" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E26" s="85" t="s">
+      <c r="E26" s="84" t="s">
         <v>2344</v>
       </c>
-      <c r="F26" s="85" t="s">
+      <c r="F26" s="84" t="s">
         <v>2345</v>
       </c>
-      <c r="G26" s="85" t="s">
+      <c r="G26" s="84" t="s">
         <v>2346</v>
       </c>
-      <c r="H26" s="85" t="s">
+      <c r="H26" s="84" t="s">
         <v>2347</v>
       </c>
-      <c r="I26" s="84" t="s">
+      <c r="I26" s="83" t="s">
         <v>2348</v>
       </c>
-      <c r="J26" s="84" t="s">
+      <c r="J26" s="83" t="s">
         <v>2349</v>
       </c>
-      <c r="K26" s="85" t="s">
+      <c r="K26" s="84" t="s">
         <v>2350</v>
       </c>
-      <c r="L26" s="85" t="s">
+      <c r="L26" s="84" t="s">
         <v>2351</v>
       </c>
-      <c r="M26" s="85" t="s">
+      <c r="M26" s="84" t="s">
         <v>2352</v>
       </c>
-      <c r="N26" s="85" t="s">
+      <c r="N26" s="84" t="s">
         <v>2353</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="84" t="s">
+      <c r="A27" s="83" t="s">
         <v>2354</v>
       </c>
-      <c r="B27" s="84" t="s">
+      <c r="B27" s="83" t="s">
         <v>2355</v>
       </c>
-      <c r="C27" s="84" t="s">
+      <c r="C27" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D27" s="84" t="s">
+      <c r="D27" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E27" s="85" t="s">
+      <c r="E27" s="84" t="s">
         <v>2356</v>
       </c>
-      <c r="F27" s="85" t="s">
+      <c r="F27" s="84" t="s">
         <v>2357</v>
       </c>
-      <c r="G27" s="85" t="s">
+      <c r="G27" s="84" t="s">
         <v>2358</v>
       </c>
-      <c r="H27" s="85" t="s">
+      <c r="H27" s="84" t="s">
         <v>2359</v>
       </c>
-      <c r="I27" s="84" t="s">
+      <c r="I27" s="83" t="s">
         <v>2360</v>
       </c>
-      <c r="J27" s="84" t="s">
+      <c r="J27" s="83" t="s">
         <v>2361</v>
       </c>
-      <c r="K27" s="85" t="s">
+      <c r="K27" s="84" t="s">
         <v>2362</v>
       </c>
-      <c r="L27" s="85" t="s">
+      <c r="L27" s="84" t="s">
         <v>2193</v>
       </c>
-      <c r="M27" s="85" t="s">
+      <c r="M27" s="84" t="s">
         <v>2363</v>
       </c>
-      <c r="N27" s="85" t="s">
+      <c r="N27" s="84" t="s">
         <v>2364</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="84" t="s">
+      <c r="A28" s="83" t="s">
         <v>2365</v>
       </c>
-      <c r="B28" s="84" t="s">
+      <c r="B28" s="83" t="s">
         <v>2366</v>
       </c>
-      <c r="C28" s="84" t="s">
+      <c r="C28" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D28" s="84" t="s">
+      <c r="D28" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E28" s="85" t="s">
+      <c r="E28" s="84" t="s">
         <v>2367</v>
       </c>
-      <c r="F28" s="85" t="s">
+      <c r="F28" s="84" t="s">
         <v>2368</v>
       </c>
-      <c r="G28" s="85" t="s">
+      <c r="G28" s="84" t="s">
         <v>2369</v>
       </c>
-      <c r="H28" s="85" t="s">
+      <c r="H28" s="84" t="s">
         <v>2370</v>
       </c>
-      <c r="I28" s="84" t="s">
+      <c r="I28" s="83" t="s">
         <v>2371</v>
       </c>
-      <c r="J28" s="84" t="s">
+      <c r="J28" s="83" t="s">
         <v>2372</v>
       </c>
-      <c r="K28" s="85" t="s">
+      <c r="K28" s="84" t="s">
         <v>2373</v>
       </c>
-      <c r="L28" s="85" t="s">
+      <c r="L28" s="84" t="s">
         <v>2171</v>
       </c>
-      <c r="M28" s="85" t="s">
+      <c r="M28" s="84" t="s">
         <v>2374</v>
       </c>
-      <c r="N28" s="85" t="s">
+      <c r="N28" s="84" t="s">
         <v>2375</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="84" t="s">
+      <c r="A29" s="83" t="s">
         <v>2376</v>
       </c>
-      <c r="B29" s="84" t="s">
+      <c r="B29" s="83" t="s">
         <v>2377</v>
       </c>
-      <c r="C29" s="84" t="s">
+      <c r="C29" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D29" s="84" t="s">
+      <c r="D29" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E29" s="85" t="s">
+      <c r="E29" s="84" t="s">
         <v>2378</v>
       </c>
-      <c r="F29" s="85" t="s">
+      <c r="F29" s="84" t="s">
         <v>2379</v>
       </c>
-      <c r="G29" s="85" t="s">
+      <c r="G29" s="84" t="s">
         <v>2380</v>
       </c>
-      <c r="H29" s="85" t="s">
+      <c r="H29" s="84" t="s">
         <v>2381</v>
       </c>
-      <c r="I29" s="84" t="s">
+      <c r="I29" s="83" t="s">
         <v>2382</v>
       </c>
-      <c r="J29" s="84" t="s">
+      <c r="J29" s="83" t="s">
         <v>2383</v>
       </c>
-      <c r="K29" s="85" t="s">
+      <c r="K29" s="84" t="s">
         <v>2384</v>
       </c>
-      <c r="L29" s="85" t="s">
+      <c r="L29" s="84" t="s">
         <v>2385</v>
       </c>
-      <c r="M29" s="85" t="s">
+      <c r="M29" s="84" t="s">
         <v>2386</v>
       </c>
-      <c r="N29" s="85" t="s">
+      <c r="N29" s="84" t="s">
         <v>2387</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="84" t="s">
+      <c r="A30" s="83" t="s">
         <v>2388</v>
       </c>
-      <c r="B30" s="84" t="s">
+      <c r="B30" s="83" t="s">
         <v>2389</v>
       </c>
-      <c r="C30" s="84" t="s">
+      <c r="C30" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D30" s="84" t="s">
+      <c r="D30" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E30" s="85" t="s">
+      <c r="E30" s="84" t="s">
         <v>2390</v>
       </c>
-      <c r="F30" s="85" t="s">
+      <c r="F30" s="84" t="s">
         <v>2391</v>
       </c>
-      <c r="G30" s="85" t="s">
+      <c r="G30" s="84" t="s">
         <v>2392</v>
       </c>
-      <c r="H30" s="85" t="s">
+      <c r="H30" s="84" t="s">
         <v>2393</v>
       </c>
-      <c r="I30" s="84" t="s">
+      <c r="I30" s="83" t="s">
         <v>2394</v>
       </c>
-      <c r="J30" s="84" t="s">
+      <c r="J30" s="83" t="s">
         <v>2395</v>
       </c>
-      <c r="K30" s="85" t="s">
+      <c r="K30" s="84" t="s">
         <v>2396</v>
       </c>
-      <c r="L30" s="85" t="s">
+      <c r="L30" s="84" t="s">
         <v>2397</v>
       </c>
-      <c r="M30" s="85" t="s">
+      <c r="M30" s="84" t="s">
         <v>2398</v>
       </c>
-      <c r="N30" s="85" t="s">
+      <c r="N30" s="84" t="s">
         <v>2399</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="84" t="s">
+      <c r="A31" s="83" t="s">
         <v>2400</v>
       </c>
-      <c r="B31" s="84" t="s">
+      <c r="B31" s="83" t="s">
         <v>2401</v>
       </c>
-      <c r="C31" s="84" t="s">
+      <c r="C31" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="D31" s="84" t="s">
+      <c r="D31" s="83" t="s">
         <v>2108</v>
       </c>
-      <c r="E31" s="85" t="s">
+      <c r="E31" s="84" t="s">
         <v>2402</v>
       </c>
-      <c r="F31" s="85" t="s">
+      <c r="F31" s="84" t="s">
         <v>2403</v>
       </c>
-      <c r="G31" s="85" t="s">
+      <c r="G31" s="84" t="s">
         <v>2404</v>
       </c>
-      <c r="H31" s="85" t="s">
+      <c r="H31" s="84" t="s">
         <v>2405</v>
       </c>
-      <c r="I31" s="84" t="s">
+      <c r="I31" s="83" t="s">
         <v>2406</v>
       </c>
-      <c r="J31" s="84" t="s">
+      <c r="J31" s="83" t="s">
         <v>2407</v>
       </c>
-      <c r="K31" s="85" t="s">
+      <c r="K31" s="84" t="s">
         <v>2408</v>
       </c>
-      <c r="L31" s="85" t="s">
+      <c r="L31" s="84" t="s">
         <v>2409</v>
       </c>
-      <c r="M31" s="85" t="s">
+      <c r="M31" s="84" t="s">
         <v>2410</v>
       </c>
-      <c r="N31" s="85" t="s">
+      <c r="N31" s="84" t="s">
         <v>2411</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="84" t="s">
+      <c r="A33" s="83" t="s">
         <v>2412</v>
       </c>
-      <c r="B33" s="84" t="s">
+      <c r="B33" s="83" t="s">
         <v>2413</v>
       </c>
-      <c r="C33" s="84" t="s">
+      <c r="C33" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E33" s="85" t="s">
+      <c r="E33" s="84" t="s">
         <v>2414</v>
       </c>
-      <c r="F33" s="85" t="s">
+      <c r="F33" s="84" t="s">
         <v>2415</v>
       </c>
-      <c r="G33" s="85" t="s">
+      <c r="G33" s="84" t="s">
         <v>2416</v>
       </c>
-      <c r="H33" s="85" t="s">
+      <c r="H33" s="84" t="s">
         <v>2417</v>
       </c>
       <c r="I33" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="84" t="s">
+      <c r="J33" s="83" t="s">
         <v>2418</v>
       </c>
-      <c r="K33" s="85" t="s">
+      <c r="K33" s="84" t="s">
         <v>2419</v>
       </c>
-      <c r="L33" s="85" t="s">
+      <c r="L33" s="84" t="s">
         <v>2420</v>
       </c>
-      <c r="M33" s="85" t="s">
+      <c r="M33" s="84" t="s">
         <v>2421</v>
       </c>
-      <c r="N33" s="85" t="s">
+      <c r="N33" s="84" t="s">
         <v>2422</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="84" t="s">
+      <c r="A34" s="83" t="s">
         <v>2423</v>
       </c>
-      <c r="B34" s="84" t="s">
+      <c r="B34" s="83" t="s">
         <v>2424</v>
       </c>
-      <c r="C34" s="84" t="s">
+      <c r="C34" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E34" s="85" t="s">
+      <c r="E34" s="84" t="s">
         <v>2425</v>
       </c>
-      <c r="F34" s="85" t="s">
+      <c r="F34" s="84" t="s">
         <v>2426</v>
       </c>
-      <c r="G34" s="85" t="s">
+      <c r="G34" s="84" t="s">
         <v>2427</v>
       </c>
-      <c r="H34" s="85" t="s">
+      <c r="H34" s="84" t="s">
         <v>2428</v>
       </c>
       <c r="I34" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="J34" s="84" t="s">
+      <c r="J34" s="83" t="s">
         <v>2429</v>
       </c>
-      <c r="K34" s="85" t="s">
+      <c r="K34" s="84" t="s">
         <v>2430</v>
       </c>
-      <c r="L34" s="85" t="s">
+      <c r="L34" s="84" t="s">
         <v>2431</v>
       </c>
-      <c r="M34" s="85" t="s">
+      <c r="M34" s="84" t="s">
         <v>2432</v>
       </c>
-      <c r="N34" s="85" t="s">
+      <c r="N34" s="84" t="s">
         <v>2433</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="84" t="s">
+      <c r="A35" s="83" t="s">
         <v>2434</v>
       </c>
-      <c r="B35" s="84" t="s">
+      <c r="B35" s="83" t="s">
         <v>2435</v>
       </c>
-      <c r="C35" s="84" t="s">
+      <c r="C35" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E35" s="85" t="s">
+      <c r="E35" s="84" t="s">
         <v>2436</v>
       </c>
-      <c r="F35" s="85" t="s">
+      <c r="F35" s="84" t="s">
         <v>2437</v>
       </c>
-      <c r="G35" s="85" t="s">
+      <c r="G35" s="84" t="s">
         <v>2438</v>
       </c>
-      <c r="H35" s="85" t="s">
+      <c r="H35" s="84" t="s">
         <v>2439</v>
       </c>
       <c r="I35" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="J35" s="84" t="s">
+      <c r="J35" s="83" t="s">
         <v>2440</v>
       </c>
-      <c r="K35" s="85" t="s">
+      <c r="K35" s="84" t="s">
         <v>2441</v>
       </c>
-      <c r="L35" s="85" t="s">
+      <c r="L35" s="84" t="s">
         <v>2442</v>
       </c>
-      <c r="M35" s="85" t="s">
+      <c r="M35" s="84" t="s">
         <v>2443</v>
       </c>
-      <c r="N35" s="85" t="s">
+      <c r="N35" s="84" t="s">
         <v>2444</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="84" t="s">
+      <c r="A37" s="83" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="84" t="s">
+      <c r="B37" s="83" t="s">
         <v>2445</v>
       </c>
-      <c r="C37" s="84" t="s">
+      <c r="C37" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="G37" s="85" t="s">
+      <c r="G37" s="84" t="s">
         <v>2446</v>
       </c>
-      <c r="H37" s="85" t="s">
+      <c r="H37" s="84" t="s">
         <v>2446</v>
       </c>
-      <c r="I37" s="84" t="s">
+      <c r="I37" s="83" t="s">
         <v>2447</v>
       </c>
-      <c r="J37" s="84" t="s">
+      <c r="J37" s="83" t="s">
         <v>2448</v>
       </c>
-      <c r="M37" s="85" t="s">
+      <c r="M37" s="84" t="s">
         <v>2449</v>
       </c>
-      <c r="N37" s="85" t="s">
+      <c r="N37" s="84" t="s">
         <v>2450</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="84" t="s">
+      <c r="A38" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="B38" s="84" t="s">
+      <c r="B38" s="83" t="s">
         <v>2451</v>
       </c>
-      <c r="C38" s="84" t="s">
+      <c r="C38" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E38" s="85" t="s">
+      <c r="E38" s="84" t="s">
         <v>2452</v>
       </c>
-      <c r="F38" s="85" t="s">
+      <c r="F38" s="84" t="s">
         <v>2452</v>
       </c>
-      <c r="G38" s="85" t="s">
+      <c r="G38" s="84" t="s">
         <v>2453</v>
       </c>
-      <c r="H38" s="85" t="s">
+      <c r="H38" s="84" t="s">
         <v>2454</v>
       </c>
-      <c r="I38" s="84" t="s">
+      <c r="I38" s="83" t="s">
         <v>2455</v>
       </c>
-      <c r="J38" s="84" t="s">
+      <c r="J38" s="83" t="s">
         <v>2456</v>
       </c>
-      <c r="K38" s="85" t="s">
+      <c r="K38" s="84" t="s">
         <v>2457</v>
       </c>
-      <c r="L38" s="85" t="s">
+      <c r="L38" s="84" t="s">
         <v>2457</v>
       </c>
-      <c r="M38" s="85" t="s">
+      <c r="M38" s="84" t="s">
         <v>2458</v>
       </c>
-      <c r="N38" s="85" t="s">
+      <c r="N38" s="84" t="s">
         <v>2459</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="84" t="s">
+      <c r="A39" s="83" t="s">
         <v>2460</v>
       </c>
-      <c r="B39" s="84" t="s">
+      <c r="B39" s="83" t="s">
         <v>2461</v>
       </c>
-      <c r="C39" s="84" t="s">
+      <c r="C39" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E39" s="85" t="s">
+      <c r="E39" s="84" t="s">
         <v>2462</v>
       </c>
-      <c r="F39" s="85" t="s">
+      <c r="F39" s="84" t="s">
         <v>2462</v>
       </c>
-      <c r="G39" s="85" t="s">
+      <c r="G39" s="84" t="s">
         <v>2463</v>
       </c>
-      <c r="H39" s="85" t="s">
+      <c r="H39" s="84" t="s">
         <v>2464</v>
       </c>
-      <c r="I39" s="84" t="s">
+      <c r="I39" s="83" t="s">
         <v>2465</v>
       </c>
-      <c r="J39" s="84" t="s">
+      <c r="J39" s="83" t="s">
         <v>2466</v>
       </c>
-      <c r="K39" s="85" t="s">
+      <c r="K39" s="84" t="s">
         <v>2467</v>
       </c>
-      <c r="L39" s="85" t="s">
+      <c r="L39" s="84" t="s">
         <v>2467</v>
       </c>
-      <c r="M39" s="85" t="s">
+      <c r="M39" s="84" t="s">
         <v>2468</v>
       </c>
-      <c r="N39" s="85" t="s">
+      <c r="N39" s="84" t="s">
         <v>2469</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="84" t="s">
+      <c r="C40" s="83" t="s">
         <v>2107</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="84" t="s">
+      <c r="A41" s="83" t="s">
         <v>2470</v>
       </c>
-      <c r="B41" s="84" t="s">
+      <c r="B41" s="83" t="s">
         <v>2471</v>
       </c>
-      <c r="C41" s="84" t="s">
+      <c r="C41" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E41" s="85" t="s">
+      <c r="E41" s="84" t="s">
         <v>2472</v>
       </c>
-      <c r="F41" s="85" t="s">
+      <c r="F41" s="84" t="s">
         <v>2472</v>
       </c>
-      <c r="G41" s="85" t="s">
+      <c r="G41" s="84" t="s">
         <v>2473</v>
       </c>
-      <c r="H41" s="85" t="s">
+      <c r="H41" s="84" t="s">
         <v>2474</v>
       </c>
-      <c r="I41" s="84" t="s">
+      <c r="I41" s="83" t="s">
         <v>2475</v>
       </c>
-      <c r="J41" s="84" t="s">
+      <c r="J41" s="83" t="s">
         <v>2476</v>
       </c>
-      <c r="K41" s="85" t="s">
+      <c r="K41" s="84" t="s">
         <v>2477</v>
       </c>
-      <c r="M41" s="85" t="s">
+      <c r="M41" s="84" t="s">
         <v>2478</v>
       </c>
-      <c r="N41" s="85" t="s">
+      <c r="N41" s="84" t="s">
         <v>2479</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="84" t="s">
+      <c r="A42" s="83" t="s">
         <v>2480</v>
       </c>
-      <c r="B42" s="84" t="s">
+      <c r="B42" s="83" t="s">
         <v>2481</v>
       </c>
-      <c r="C42" s="84" t="s">
+      <c r="C42" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E42" s="85" t="s">
+      <c r="E42" s="84" t="s">
         <v>2482</v>
       </c>
-      <c r="F42" s="85" t="s">
+      <c r="F42" s="84" t="s">
         <v>2482</v>
       </c>
-      <c r="G42" s="85" t="s">
+      <c r="G42" s="84" t="s">
         <v>2483</v>
       </c>
-      <c r="H42" s="85" t="s">
+      <c r="H42" s="84" t="s">
         <v>2484</v>
       </c>
-      <c r="I42" s="84" t="s">
+      <c r="I42" s="83" t="s">
         <v>2485</v>
       </c>
-      <c r="J42" s="84" t="s">
+      <c r="J42" s="83" t="s">
         <v>2486</v>
       </c>
-      <c r="K42" s="85" t="s">
+      <c r="K42" s="84" t="s">
         <v>2487</v>
       </c>
-      <c r="L42" s="85" t="s">
+      <c r="L42" s="84" t="s">
         <v>2488</v>
       </c>
-      <c r="M42" s="85" t="s">
+      <c r="M42" s="84" t="s">
         <v>2489</v>
       </c>
-      <c r="N42" s="85" t="s">
+      <c r="N42" s="84" t="s">
         <v>2490</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="84" t="s">
+      <c r="A43" s="83" t="s">
         <v>2491</v>
       </c>
-      <c r="B43" s="84" t="s">
+      <c r="B43" s="83" t="s">
         <v>2492</v>
       </c>
-      <c r="C43" s="84" t="s">
+      <c r="C43" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E43" s="85" t="s">
+      <c r="E43" s="84" t="s">
         <v>2493</v>
       </c>
-      <c r="F43" s="85" t="s">
+      <c r="F43" s="84" t="s">
         <v>2494</v>
       </c>
-      <c r="G43" s="85" t="s">
+      <c r="G43" s="84" t="s">
         <v>2495</v>
       </c>
-      <c r="H43" s="85" t="s">
+      <c r="H43" s="84" t="s">
         <v>2496</v>
       </c>
-      <c r="I43" s="84" t="s">
+      <c r="I43" s="83" t="s">
         <v>2497</v>
       </c>
-      <c r="J43" s="84" t="s">
+      <c r="J43" s="83" t="s">
         <v>2498</v>
       </c>
-      <c r="M43" s="85" t="s">
+      <c r="M43" s="84" t="s">
         <v>2499</v>
       </c>
-      <c r="N43" s="85" t="s">
+      <c r="N43" s="84" t="s">
         <v>2500</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="84" t="s">
+      <c r="A44" s="83" t="s">
         <v>2501</v>
       </c>
-      <c r="B44" s="84" t="s">
+      <c r="B44" s="83" t="s">
         <v>2501</v>
       </c>
-      <c r="C44" s="84" t="s">
+      <c r="C44" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E44" s="85" t="s">
+      <c r="E44" s="84" t="s">
         <v>2502</v>
       </c>
-      <c r="G44" s="85" t="s">
+      <c r="G44" s="84" t="s">
         <v>2503</v>
       </c>
-      <c r="H44" s="85" t="s">
+      <c r="H44" s="84" t="s">
         <v>2503</v>
       </c>
-      <c r="I44" s="84" t="s">
+      <c r="I44" s="83" t="s">
         <v>2504</v>
       </c>
-      <c r="J44" s="84" t="s">
+      <c r="J44" s="83" t="s">
         <v>2505</v>
       </c>
-      <c r="K44" s="85" t="s">
+      <c r="K44" s="84" t="s">
         <v>2506</v>
       </c>
-      <c r="L44" s="85" t="s">
+      <c r="L44" s="84" t="s">
         <v>2506</v>
       </c>
-      <c r="M44" s="85" t="s">
+      <c r="M44" s="84" t="s">
         <v>2507</v>
       </c>
-      <c r="N44" s="85" t="s">
+      <c r="N44" s="84" t="s">
         <v>2508</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="84" t="s">
+      <c r="A45" s="83" t="s">
         <v>2509</v>
       </c>
-      <c r="B45" s="84" t="s">
+      <c r="B45" s="83" t="s">
         <v>2510</v>
       </c>
-      <c r="C45" s="84" t="s">
+      <c r="C45" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E45" s="85" t="s">
+      <c r="E45" s="84" t="s">
         <v>2511</v>
       </c>
-      <c r="F45" s="85" t="s">
+      <c r="F45" s="84" t="s">
         <v>2512</v>
       </c>
-      <c r="G45" s="85" t="s">
+      <c r="G45" s="84" t="s">
         <v>2513</v>
       </c>
-      <c r="H45" s="85" t="s">
+      <c r="H45" s="84" t="s">
         <v>2514</v>
       </c>
-      <c r="I45" s="84" t="s">
+      <c r="I45" s="83" t="s">
         <v>2515</v>
       </c>
-      <c r="J45" s="84" t="s">
+      <c r="J45" s="83" t="s">
         <v>2516</v>
       </c>
-      <c r="K45" s="85" t="s">
+      <c r="K45" s="84" t="s">
         <v>2517</v>
       </c>
-      <c r="L45" s="85" t="s">
+      <c r="L45" s="84" t="s">
         <v>2517</v>
       </c>
-      <c r="M45" s="85" t="s">
+      <c r="M45" s="84" t="s">
         <v>2518</v>
       </c>
-      <c r="N45" s="85" t="s">
+      <c r="N45" s="84" t="s">
         <v>2519</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="84" t="s">
+      <c r="A46" s="83" t="s">
         <v>2520</v>
       </c>
-      <c r="B46" s="84" t="s">
+      <c r="B46" s="83" t="s">
         <v>2520</v>
       </c>
-      <c r="C46" s="84" t="s">
+      <c r="C46" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E46" s="85" t="s">
+      <c r="E46" s="84" t="s">
         <v>2521</v>
       </c>
-      <c r="F46" s="85" t="s">
+      <c r="F46" s="84" t="s">
         <v>2521</v>
       </c>
-      <c r="G46" s="85" t="s">
+      <c r="G46" s="84" t="s">
         <v>2522</v>
       </c>
-      <c r="H46" s="85" t="s">
+      <c r="H46" s="84" t="s">
         <v>2523</v>
       </c>
-      <c r="I46" s="84" t="s">
+      <c r="I46" s="83" t="s">
         <v>2524</v>
       </c>
-      <c r="J46" s="84" t="s">
+      <c r="J46" s="83" t="s">
         <v>2525</v>
       </c>
-      <c r="K46" s="85" t="s">
+      <c r="K46" s="84" t="s">
         <v>2526</v>
       </c>
-      <c r="L46" s="85" t="s">
+      <c r="L46" s="84" t="s">
         <v>2526</v>
       </c>
-      <c r="M46" s="85" t="s">
+      <c r="M46" s="84" t="s">
         <v>2527</v>
       </c>
-      <c r="N46" s="85" t="s">
+      <c r="N46" s="84" t="s">
         <v>2528</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="84" t="s">
+      <c r="A47" s="83" t="s">
         <v>2529</v>
       </c>
-      <c r="B47" s="84" t="s">
+      <c r="B47" s="83" t="s">
         <v>2529</v>
       </c>
-      <c r="C47" s="84" t="s">
+      <c r="C47" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E47" s="85" t="s">
+      <c r="E47" s="84" t="s">
         <v>2530</v>
       </c>
-      <c r="F47" s="85" t="s">
+      <c r="F47" s="84" t="s">
         <v>2531</v>
       </c>
-      <c r="G47" s="85" t="s">
+      <c r="G47" s="84" t="s">
         <v>2209</v>
       </c>
-      <c r="H47" s="85" t="s">
+      <c r="H47" s="84" t="s">
         <v>2532</v>
       </c>
-      <c r="I47" s="84" t="s">
+      <c r="I47" s="83" t="s">
         <v>2533</v>
       </c>
-      <c r="J47" s="84" t="s">
+      <c r="J47" s="83" t="s">
         <v>2534</v>
       </c>
-      <c r="K47" s="85" t="s">
+      <c r="K47" s="84" t="s">
         <v>2535</v>
       </c>
-      <c r="L47" s="85" t="s">
+      <c r="L47" s="84" t="s">
         <v>2535</v>
       </c>
-      <c r="M47" s="85" t="s">
+      <c r="M47" s="84" t="s">
         <v>2214</v>
       </c>
-      <c r="N47" s="85" t="s">
+      <c r="N47" s="84" t="s">
         <v>2536</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="84" t="s">
+      <c r="A48" s="83" t="s">
         <v>2537</v>
       </c>
-      <c r="B48" s="84" t="s">
+      <c r="B48" s="83" t="s">
         <v>2538</v>
       </c>
-      <c r="C48" s="84" t="s">
+      <c r="C48" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E48" s="85" t="s">
+      <c r="E48" s="84" t="s">
         <v>2539</v>
       </c>
-      <c r="F48" s="85" t="s">
+      <c r="F48" s="84" t="s">
         <v>2539</v>
       </c>
-      <c r="G48" s="85" t="s">
+      <c r="G48" s="84" t="s">
         <v>2540</v>
       </c>
-      <c r="H48" s="85" t="s">
+      <c r="H48" s="84" t="s">
         <v>2540</v>
       </c>
-      <c r="I48" s="84" t="s">
+      <c r="I48" s="83" t="s">
         <v>2541</v>
       </c>
-      <c r="J48" s="84" t="s">
+      <c r="J48" s="83" t="s">
         <v>2542</v>
       </c>
-      <c r="K48" s="85" t="s">
+      <c r="K48" s="84" t="s">
         <v>2543</v>
       </c>
-      <c r="L48" s="85" t="s">
+      <c r="L48" s="84" t="s">
         <v>2543</v>
       </c>
-      <c r="M48" s="85" t="s">
+      <c r="M48" s="84" t="s">
         <v>2544</v>
       </c>
-      <c r="N48" s="85" t="s">
+      <c r="N48" s="84" t="s">
         <v>2544</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="84" t="s">
+      <c r="A49" s="83" t="s">
         <v>2545</v>
       </c>
-      <c r="B49" s="84" t="s">
+      <c r="B49" s="83" t="s">
         <v>2546</v>
       </c>
-      <c r="C49" s="84" t="s">
+      <c r="C49" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E49" s="85" t="s">
+      <c r="E49" s="84" t="s">
         <v>2547</v>
       </c>
-      <c r="F49" s="85" t="s">
+      <c r="F49" s="84" t="s">
         <v>2547</v>
       </c>
-      <c r="G49" s="85" t="s">
+      <c r="G49" s="84" t="s">
         <v>2473</v>
       </c>
-      <c r="H49" s="85" t="s">
+      <c r="H49" s="84" t="s">
         <v>2474</v>
       </c>
-      <c r="I49" s="84" t="s">
+      <c r="I49" s="83" t="s">
         <v>2548</v>
       </c>
-      <c r="J49" s="84" t="s">
+      <c r="J49" s="83" t="s">
         <v>2549</v>
       </c>
-      <c r="K49" s="85" t="s">
+      <c r="K49" s="84" t="s">
         <v>2550</v>
       </c>
-      <c r="L49" s="85" t="s">
+      <c r="L49" s="84" t="s">
         <v>2550</v>
       </c>
-      <c r="M49" s="85" t="s">
+      <c r="M49" s="84" t="s">
         <v>2551</v>
       </c>
-      <c r="N49" s="85" t="s">
+      <c r="N49" s="84" t="s">
         <v>2552</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="84" t="s">
+      <c r="A50" s="83" t="s">
         <v>2553</v>
       </c>
-      <c r="B50" s="84" t="s">
+      <c r="B50" s="83" t="s">
         <v>2553</v>
       </c>
-      <c r="C50" s="84" t="s">
+      <c r="C50" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="G50" s="85" t="s">
+      <c r="G50" s="84" t="s">
         <v>2554</v>
       </c>
-      <c r="H50" s="85" t="s">
+      <c r="H50" s="84" t="s">
         <v>2554</v>
       </c>
-      <c r="I50" s="84" t="s">
+      <c r="I50" s="83" t="s">
         <v>2555</v>
       </c>
-      <c r="J50" s="84" t="s">
+      <c r="J50" s="83" t="s">
         <v>2555</v>
       </c>
-      <c r="M50" s="85" t="s">
+      <c r="M50" s="84" t="s">
         <v>2556</v>
       </c>
-      <c r="N50" s="85" t="s">
+      <c r="N50" s="84" t="s">
         <v>2557</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="84" t="s">
+      <c r="A51" s="83" t="s">
         <v>2558</v>
       </c>
-      <c r="B51" s="84" t="s">
+      <c r="B51" s="83" t="s">
         <v>2559</v>
       </c>
-      <c r="C51" s="84" t="s">
+      <c r="C51" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E51" s="85" t="s">
+      <c r="E51" s="84" t="s">
         <v>2560</v>
       </c>
-      <c r="F51" s="85" t="s">
+      <c r="F51" s="84" t="s">
         <v>2560</v>
       </c>
-      <c r="G51" s="85" t="s">
+      <c r="G51" s="84" t="s">
         <v>2561</v>
       </c>
-      <c r="H51" s="85" t="s">
+      <c r="H51" s="84" t="s">
         <v>2561</v>
       </c>
-      <c r="I51" s="84" t="s">
+      <c r="I51" s="83" t="s">
         <v>2562</v>
       </c>
-      <c r="J51" s="84" t="s">
+      <c r="J51" s="83" t="s">
         <v>2563</v>
       </c>
-      <c r="K51" s="85" t="s">
+      <c r="K51" s="84" t="s">
         <v>2564</v>
       </c>
-      <c r="L51" s="85" t="s">
+      <c r="L51" s="84" t="s">
         <v>2565</v>
       </c>
-      <c r="M51" s="85" t="s">
+      <c r="M51" s="84" t="s">
         <v>2566</v>
       </c>
-      <c r="N51" s="85" t="s">
+      <c r="N51" s="84" t="s">
         <v>2567</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="84" t="s">
+      <c r="A52" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="B52" s="84" t="s">
+      <c r="B52" s="83" t="s">
         <v>2</v>
       </c>
-      <c r="C52" s="84" t="s">
+      <c r="C52" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E52" s="85" t="s">
+      <c r="E52" s="84" t="s">
         <v>2568</v>
       </c>
-      <c r="F52" s="85" t="s">
+      <c r="F52" s="84" t="s">
         <v>2569</v>
       </c>
-      <c r="G52" s="85" t="s">
+      <c r="G52" s="84" t="s">
         <v>2570</v>
       </c>
-      <c r="H52" s="85" t="s">
+      <c r="H52" s="84" t="s">
         <v>2570</v>
       </c>
-      <c r="I52" s="84" t="s">
+      <c r="I52" s="83" t="s">
         <v>2571</v>
       </c>
-      <c r="J52" s="84" t="s">
+      <c r="J52" s="83" t="s">
         <v>2571</v>
       </c>
-      <c r="K52" s="85" t="s">
+      <c r="K52" s="84" t="s">
         <v>2572</v>
       </c>
-      <c r="L52" s="85" t="s">
+      <c r="L52" s="84" t="s">
         <v>2572</v>
       </c>
-      <c r="M52" s="85" t="s">
+      <c r="M52" s="84" t="s">
         <v>2573</v>
       </c>
-      <c r="N52" s="85" t="s">
+      <c r="N52" s="84" t="s">
         <v>2574</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="84" t="s">
+      <c r="A53" s="83" t="s">
         <v>2575</v>
       </c>
-      <c r="B53" s="84" t="s">
+      <c r="B53" s="83" t="s">
         <v>2576</v>
       </c>
-      <c r="C53" s="84" t="s">
+      <c r="C53" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="G53" s="85" t="s">
+      <c r="G53" s="84" t="s">
         <v>2577</v>
       </c>
-      <c r="H53" s="85" t="s">
+      <c r="H53" s="84" t="s">
         <v>2578</v>
       </c>
-      <c r="I53" s="84" t="s">
+      <c r="I53" s="83" t="s">
         <v>2579</v>
       </c>
-      <c r="J53" s="84" t="s">
+      <c r="J53" s="83" t="s">
         <v>2580</v>
       </c>
-      <c r="K53" s="85" t="s">
+      <c r="K53" s="84" t="s">
         <v>2581</v>
       </c>
-      <c r="L53" s="85" t="s">
+      <c r="L53" s="84" t="s">
         <v>2581</v>
       </c>
-      <c r="M53" s="85" t="s">
+      <c r="M53" s="84" t="s">
         <v>2582</v>
       </c>
-      <c r="N53" s="85" t="s">
+      <c r="N53" s="84" t="s">
         <v>2583</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="84" t="s">
+      <c r="A54" s="83" t="s">
         <v>2584</v>
       </c>
-      <c r="B54" s="84" t="s">
+      <c r="B54" s="83" t="s">
         <v>2584</v>
       </c>
-      <c r="C54" s="84" t="s">
+      <c r="C54" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E54" s="85" t="s">
+      <c r="E54" s="84" t="s">
         <v>2218</v>
       </c>
-      <c r="F54" s="85" t="s">
+      <c r="F54" s="84" t="s">
         <v>2218</v>
       </c>
-      <c r="G54" s="85" t="s">
+      <c r="G54" s="84" t="s">
         <v>2585</v>
       </c>
-      <c r="H54" s="85" t="s">
+      <c r="H54" s="84" t="s">
         <v>2585</v>
       </c>
-      <c r="I54" s="84" t="s">
+      <c r="I54" s="83" t="s">
         <v>2586</v>
       </c>
-      <c r="J54" s="84" t="s">
+      <c r="J54" s="83" t="s">
         <v>2586</v>
       </c>
-      <c r="K54" s="85" t="s">
+      <c r="K54" s="84" t="s">
         <v>2587</v>
       </c>
-      <c r="L54" s="85" t="s">
+      <c r="L54" s="84" t="s">
         <v>2587</v>
       </c>
-      <c r="M54" s="85" t="s">
+      <c r="M54" s="84" t="s">
         <v>2588</v>
       </c>
-      <c r="N54" s="85" t="s">
+      <c r="N54" s="84" t="s">
         <v>2589</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="84" t="s">
+      <c r="A55" s="83" t="s">
         <v>2590</v>
       </c>
-      <c r="B55" s="84" t="s">
+      <c r="B55" s="83" t="s">
         <v>2591</v>
       </c>
-      <c r="C55" s="84" t="s">
+      <c r="C55" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E55" s="85" t="s">
+      <c r="E55" s="84" t="s">
         <v>2592</v>
       </c>
-      <c r="F55" s="85" t="s">
+      <c r="F55" s="84" t="s">
         <v>2592</v>
       </c>
-      <c r="G55" s="85" t="s">
+      <c r="G55" s="84" t="s">
         <v>2593</v>
       </c>
-      <c r="H55" s="85" t="s">
+      <c r="H55" s="84" t="s">
         <v>2594</v>
       </c>
-      <c r="I55" s="84" t="s">
+      <c r="I55" s="83" t="s">
         <v>2595</v>
       </c>
-      <c r="J55" s="84" t="s">
+      <c r="J55" s="83" t="s">
         <v>2596</v>
       </c>
-      <c r="K55" s="85" t="s">
+      <c r="K55" s="84" t="s">
         <v>2597</v>
       </c>
-      <c r="L55" s="85" t="s">
+      <c r="L55" s="84" t="s">
         <v>2597</v>
       </c>
-      <c r="M55" s="85" t="s">
+      <c r="M55" s="84" t="s">
         <v>2598</v>
       </c>
-      <c r="N55" s="85" t="s">
+      <c r="N55" s="84" t="s">
         <v>2598</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="84" t="s">
+      <c r="A56" s="83" t="s">
         <v>2599</v>
       </c>
-      <c r="B56" s="84" t="s">
+      <c r="B56" s="83" t="s">
         <v>2599</v>
       </c>
-      <c r="C56" s="84" t="s">
+      <c r="C56" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E56" s="85" t="s">
+      <c r="E56" s="84" t="s">
         <v>2600</v>
       </c>
-      <c r="F56" s="85" t="s">
+      <c r="F56" s="84" t="s">
         <v>2600</v>
       </c>
-      <c r="G56" s="85" t="s">
+      <c r="G56" s="84" t="s">
         <v>2601</v>
       </c>
-      <c r="H56" s="85" t="s">
+      <c r="H56" s="84" t="s">
         <v>2602</v>
       </c>
-      <c r="I56" s="84" t="s">
+      <c r="I56" s="83" t="s">
         <v>2603</v>
       </c>
-      <c r="J56" s="84" t="s">
+      <c r="J56" s="83" t="s">
         <v>2604</v>
       </c>
-      <c r="K56" s="85" t="s">
+      <c r="K56" s="84" t="s">
         <v>2605</v>
       </c>
-      <c r="L56" s="85" t="s">
+      <c r="L56" s="84" t="s">
         <v>2605</v>
       </c>
-      <c r="M56" s="85" t="s">
+      <c r="M56" s="84" t="s">
         <v>2606</v>
       </c>
-      <c r="N56" s="85" t="s">
+      <c r="N56" s="84" t="s">
         <v>2607</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="84" t="s">
+      <c r="A57" s="83" t="s">
         <v>2608</v>
       </c>
-      <c r="B57" s="84" t="s">
+      <c r="B57" s="83" t="s">
         <v>2609</v>
       </c>
-      <c r="C57" s="84" t="s">
+      <c r="C57" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E57" s="85" t="s">
+      <c r="E57" s="84" t="s">
         <v>2610</v>
       </c>
-      <c r="F57" s="85" t="s">
+      <c r="F57" s="84" t="s">
         <v>2610</v>
       </c>
-      <c r="G57" s="85" t="s">
+      <c r="G57" s="84" t="s">
         <v>2611</v>
       </c>
-      <c r="H57" s="85" t="s">
+      <c r="H57" s="84" t="s">
         <v>2612</v>
       </c>
-      <c r="I57" s="84" t="s">
+      <c r="I57" s="83" t="s">
         <v>2613</v>
       </c>
-      <c r="J57" s="84" t="s">
+      <c r="J57" s="83" t="s">
         <v>2614</v>
       </c>
-      <c r="K57" s="85" t="s">
+      <c r="K57" s="84" t="s">
         <v>2615</v>
       </c>
-      <c r="L57" s="85" t="s">
+      <c r="L57" s="84" t="s">
         <v>2615</v>
       </c>
-      <c r="M57" s="85" t="s">
+      <c r="M57" s="84" t="s">
         <v>2616</v>
       </c>
-      <c r="N57" s="85" t="s">
+      <c r="N57" s="84" t="s">
         <v>2617</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="84" t="s">
+      <c r="A58" s="83" t="s">
         <v>2618</v>
       </c>
-      <c r="B58" s="84" t="s">
+      <c r="B58" s="83" t="s">
         <v>2619</v>
       </c>
-      <c r="C58" s="84" t="s">
+      <c r="C58" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E58" s="85" t="s">
+      <c r="E58" s="84" t="s">
         <v>2620</v>
       </c>
-      <c r="F58" s="85" t="s">
+      <c r="F58" s="84" t="s">
         <v>2621</v>
       </c>
-      <c r="G58" s="85" t="s">
+      <c r="G58" s="84" t="s">
         <v>2622</v>
       </c>
-      <c r="H58" s="85" t="s">
+      <c r="H58" s="84" t="s">
         <v>2623</v>
       </c>
-      <c r="I58" s="84" t="s">
+      <c r="I58" s="83" t="s">
         <v>2624</v>
       </c>
-      <c r="J58" s="84" t="s">
+      <c r="J58" s="83" t="s">
         <v>2625</v>
       </c>
-      <c r="K58" s="85" t="s">
+      <c r="K58" s="84" t="s">
         <v>2626</v>
       </c>
-      <c r="L58" s="85" t="s">
+      <c r="L58" s="84" t="s">
         <v>2626</v>
       </c>
-      <c r="M58" s="85" t="s">
+      <c r="M58" s="84" t="s">
         <v>2627</v>
       </c>
-      <c r="N58" s="85" t="s">
+      <c r="N58" s="84" t="s">
         <v>2627</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="84" t="s">
+      <c r="A59" s="83" t="s">
         <v>2628</v>
       </c>
-      <c r="B59" s="84" t="s">
+      <c r="B59" s="83" t="s">
         <v>2629</v>
       </c>
-      <c r="C59" s="84" t="s">
+      <c r="C59" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="G59" s="85" t="s">
+      <c r="G59" s="84" t="s">
         <v>2630</v>
       </c>
-      <c r="H59" s="85" t="s">
+      <c r="H59" s="84" t="s">
         <v>2631</v>
       </c>
-      <c r="I59" s="84" t="s">
+      <c r="I59" s="83" t="s">
         <v>2632</v>
       </c>
-      <c r="J59" s="84" t="s">
+      <c r="J59" s="83" t="s">
         <v>2633</v>
       </c>
-      <c r="K59" s="85" t="s">
+      <c r="K59" s="84" t="s">
         <v>2634</v>
       </c>
-      <c r="L59" s="85" t="s">
+      <c r="L59" s="84" t="s">
         <v>2634</v>
       </c>
-      <c r="M59" s="85" t="s">
+      <c r="M59" s="84" t="s">
         <v>2635</v>
       </c>
-      <c r="N59" s="85" t="s">
+      <c r="N59" s="84" t="s">
         <v>2635</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="84" t="s">
+      <c r="A60" s="83" t="s">
         <v>2636</v>
       </c>
-      <c r="B60" s="84" t="s">
+      <c r="B60" s="83" t="s">
         <v>2636</v>
       </c>
-      <c r="C60" s="84" t="s">
+      <c r="C60" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E60" s="85" t="s">
+      <c r="E60" s="84" t="s">
         <v>2637</v>
       </c>
-      <c r="F60" s="85" t="s">
+      <c r="F60" s="84" t="s">
         <v>2637</v>
       </c>
-      <c r="G60" s="85" t="s">
+      <c r="G60" s="84" t="s">
         <v>2638</v>
       </c>
-      <c r="H60" s="85" t="s">
+      <c r="H60" s="84" t="s">
         <v>2639</v>
       </c>
-      <c r="I60" s="84" t="s">
+      <c r="I60" s="83" t="s">
         <v>2640</v>
       </c>
-      <c r="J60" s="84" t="s">
+      <c r="J60" s="83" t="s">
         <v>2640</v>
       </c>
-      <c r="K60" s="85" t="s">
+      <c r="K60" s="84" t="s">
         <v>2641</v>
       </c>
-      <c r="L60" s="85" t="s">
+      <c r="L60" s="84" t="s">
         <v>2641</v>
       </c>
-      <c r="M60" s="85" t="s">
+      <c r="M60" s="84" t="s">
         <v>2642</v>
       </c>
-      <c r="N60" s="85" t="s">
+      <c r="N60" s="84" t="s">
         <v>2643</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="84" t="s">
+      <c r="A61" s="83" t="s">
         <v>2644</v>
       </c>
-      <c r="B61" s="84" t="s">
+      <c r="B61" s="83" t="s">
         <v>2644</v>
       </c>
-      <c r="C61" s="84" t="s">
+      <c r="C61" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E61" s="85" t="s">
+      <c r="E61" s="84" t="s">
         <v>2645</v>
       </c>
-      <c r="F61" s="85" t="s">
+      <c r="F61" s="84" t="s">
         <v>2645</v>
       </c>
-      <c r="G61" s="85" t="s">
+      <c r="G61" s="84" t="s">
         <v>2646</v>
       </c>
-      <c r="H61" s="85" t="s">
+      <c r="H61" s="84" t="s">
         <v>2646</v>
       </c>
-      <c r="I61" s="84" t="s">
+      <c r="I61" s="83" t="s">
         <v>2647</v>
       </c>
-      <c r="J61" s="84" t="s">
+      <c r="J61" s="83" t="s">
         <v>2647</v>
       </c>
-      <c r="K61" s="85" t="s">
+      <c r="K61" s="84" t="s">
         <v>2648</v>
       </c>
-      <c r="L61" s="85" t="s">
+      <c r="L61" s="84" t="s">
         <v>2648</v>
       </c>
-      <c r="M61" s="85" t="s">
+      <c r="M61" s="84" t="s">
         <v>2649</v>
       </c>
-      <c r="N61" s="85" t="s">
+      <c r="N61" s="84" t="s">
         <v>2649</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="84" t="s">
+      <c r="A62" s="83" t="s">
         <v>2650</v>
       </c>
-      <c r="B62" s="84" t="s">
+      <c r="B62" s="83" t="s">
         <v>2650</v>
       </c>
-      <c r="C62" s="84" t="s">
+      <c r="C62" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E62" s="85" t="s">
+      <c r="E62" s="84" t="s">
         <v>2651</v>
       </c>
-      <c r="F62" s="85" t="s">
+      <c r="F62" s="84" t="s">
         <v>2651</v>
       </c>
-      <c r="G62" s="85" t="s">
+      <c r="G62" s="84" t="s">
         <v>2652</v>
       </c>
-      <c r="H62" s="85" t="s">
+      <c r="H62" s="84" t="s">
         <v>2652</v>
       </c>
-      <c r="I62" s="84" t="s">
+      <c r="I62" s="83" t="s">
         <v>2653</v>
       </c>
-      <c r="J62" s="84" t="s">
+      <c r="J62" s="83" t="s">
         <v>2654</v>
       </c>
-      <c r="K62" s="85" t="s">
+      <c r="K62" s="84" t="s">
         <v>2655</v>
       </c>
-      <c r="L62" s="85" t="s">
+      <c r="L62" s="84" t="s">
         <v>2655</v>
       </c>
-      <c r="M62" s="85" t="s">
+      <c r="M62" s="84" t="s">
         <v>2656</v>
       </c>
-      <c r="N62" s="85" t="s">
+      <c r="N62" s="84" t="s">
         <v>2657</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="84" t="s">
+      <c r="A63" s="83" t="s">
         <v>2658</v>
       </c>
-      <c r="B63" s="84" t="s">
+      <c r="B63" s="83" t="s">
         <v>2659</v>
       </c>
-      <c r="C63" s="84" t="s">
+      <c r="C63" s="83" t="s">
         <v>2107</v>
       </c>
-      <c r="E63" s="85" t="s">
+      <c r="E63" s="84" t="s">
         <v>2521</v>
       </c>
-      <c r="F63" s="85" t="s">
+      <c r="F63" s="84" t="s">
         <v>2521</v>
       </c>
-      <c r="G63" s="85" t="s">
+      <c r="G63" s="84" t="s">
         <v>2522</v>
       </c>
-      <c r="H63" s="85" t="s">
+      <c r="H63" s="84" t="s">
         <v>2523</v>
       </c>
-      <c r="I63" s="84" t="s">
+      <c r="I63" s="83" t="s">
         <v>2660</v>
       </c>
-      <c r="J63" s="84" t="s">
+      <c r="J63" s="83" t="s">
         <v>2661</v>
       </c>
-      <c r="K63" s="85" t="s">
+      <c r="K63" s="84" t="s">
         <v>2526</v>
       </c>
-      <c r="L63" s="85" t="s">
+      <c r="L63" s="84" t="s">
         <v>2526</v>
       </c>
-      <c r="M63" s="85" t="s">
+      <c r="M63" s="84" t="s">
         <v>2527</v>
       </c>
-      <c r="N63" s="85" t="s">
+      <c r="N63" s="84" t="s">
         <v>2528</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="84" t="s">
+      <c r="A64" s="83" t="s">
         <v>2662</v>
       </c>
-      <c r="B64" s="84" t="s">
+      <c r="B64" s="83" t="s">
         <v>2662</v>
       </c>
-      <c r="C64" s="84" t="s">
+      <c r="C64" s="83" t="s">
         <v>2107</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="84" t="s">
+      <c r="A66" s="83" t="s">
         <v>2663</v>
       </c>
-      <c r="B66" s="84" t="s">
+      <c r="B66" s="83" t="s">
         <v>2664</v>
       </c>
-      <c r="C66" s="84" t="s">
+      <c r="C66" s="83" t="s">
         <v>2107</v>
       </c>
     </row>
@@ -74057,154 +74007,154 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2"/>
-      <c r="B1" s="86" t="s">
+      <c r="B1" s="85" t="s">
         <v>2665</v>
       </c>
-      <c r="C1" s="86" t="s">
+      <c r="C1" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="85" t="s">
         <v>2115</v>
       </c>
-      <c r="B2" s="86" t="s">
+      <c r="B2" s="85" t="s">
         <v>2667</v>
       </c>
-      <c r="C2" s="86" t="s">
+      <c r="C2" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="86" t="s">
+      <c r="A3" s="85" t="s">
         <v>2668</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="85" t="s">
         <v>2669</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="86" t="s">
+      <c r="A4" s="85" t="s">
         <v>2113</v>
       </c>
-      <c r="B4" s="86" t="s">
+      <c r="B4" s="85" t="s">
         <v>2670</v>
       </c>
-      <c r="C4" s="86" t="s">
+      <c r="C4" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="86" t="s">
+      <c r="A5" s="85" t="s">
         <v>2111</v>
       </c>
-      <c r="B5" s="86" t="s">
+      <c r="B5" s="85" t="s">
         <v>2671</v>
       </c>
-      <c r="C5" s="86" t="s">
+      <c r="C5" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="86" t="s">
+      <c r="A6" s="85" t="s">
         <v>2672</v>
       </c>
-      <c r="B6" s="86" t="s">
+      <c r="B6" s="85" t="s">
         <v>2673</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="86" t="s">
+      <c r="A7" s="85" t="s">
         <v>2674</v>
       </c>
-      <c r="B7" s="86" t="s">
+      <c r="B7" s="85" t="s">
         <v>2675</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="86" t="s">
+      <c r="A8" s="85" t="s">
         <v>2676</v>
       </c>
-      <c r="B8" s="86" t="s">
+      <c r="B8" s="85" t="s">
         <v>2677</v>
       </c>
       <c r="C8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="86" t="s">
+      <c r="A9" s="85" t="s">
         <v>2678</v>
       </c>
-      <c r="B9" s="86" t="s">
+      <c r="B9" s="85" t="s">
         <v>2679</v>
       </c>
       <c r="C9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="86" t="s">
+      <c r="A10" s="85" t="s">
         <v>2680</v>
       </c>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="85" t="s">
         <v>2681</v>
       </c>
       <c r="C10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="86" t="s">
+      <c r="A11" s="85" t="s">
         <v>2682</v>
       </c>
-      <c r="B11" s="86" t="s">
+      <c r="B11" s="85" t="s">
         <v>2683</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="86" t="s">
+      <c r="A12" s="85" t="s">
         <v>2684</v>
       </c>
-      <c r="B12" s="86" t="s">
+      <c r="B12" s="85" t="s">
         <v>2665</v>
       </c>
-      <c r="C12" s="86" t="s">
+      <c r="C12" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="86" t="s">
+      <c r="A13" s="85" t="s">
         <v>2685</v>
       </c>
-      <c r="B13" s="86" t="s">
+      <c r="B13" s="85" t="s">
         <v>2686</v>
       </c>
       <c r="C13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="86" t="s">
+      <c r="A14" s="85" t="s">
         <v>2687</v>
       </c>
-      <c r="B14" s="86" t="s">
+      <c r="B14" s="85" t="s">
         <v>2688</v>
       </c>
       <c r="C14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="86" t="s">
+      <c r="A15" s="85" t="s">
         <v>2109</v>
       </c>
-      <c r="B15" s="86" t="s">
+      <c r="B15" s="85" t="s">
         <v>2689</v>
       </c>
-      <c r="C15" s="86" t="s">
+      <c r="C15" s="85" t="s">
         <v>2666</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="86" t="s">
+      <c r="A16" s="85" t="s">
         <v>2117</v>
       </c>
-      <c r="B16" s="86" t="s">
+      <c r="B16" s="85" t="s">
         <v>2690</v>
       </c>
       <c r="C16" s="2" t="s">
@@ -74212,19 +74162,19 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="86" t="s">
+      <c r="A17" s="85" t="s">
         <v>2691</v>
       </c>
-      <c r="B17" s="86" t="s">
+      <c r="B17" s="85" t="s">
         <v>2692</v>
       </c>
       <c r="C17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="86" t="s">
+      <c r="A18" s="85" t="s">
         <v>2693</v>
       </c>
-      <c r="B18" s="86" t="s">
+      <c r="B18" s="85" t="s">
         <v>2694</v>
       </c>
       <c r="C18" s="2"/>

</xml_diff>